<commit_message>
CHORE: ML-FEATURE-MISMATCH closed (predict pctrank fix + refresh)
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-06-09.xlsx
+++ b/cache/open_items_2026-06-09.xlsx
@@ -706,13 +706,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="105" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>ML-FEATURE-MISMATCH</t>
+          <t>STRUCT-TARGETS-M25-CUTOVER</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -722,22 +722,22 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>ML · Inference</t>
+          <t>Strategy / Targets</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Live predict_one degenerate — 29-feat model vs 17-feat extractor</t>
+          <t>Structural targets · M2.5 — cutover gate (flip use_structural_targets=true)</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Models retrained 2026-06-09 on 29 features but ml.feature_extractor.FEATURE_COLS still emits 17, so live predict_one feeds a mismatched vector and returns ~0 p_up for EVERY ticker (AI Edge 0% bug, all names). Batch ml-predict path extracts 29 correctly. /api/ml now prefers the batch cache + rejects degenerate live; ROOT FIX still needed: align FEATURE_COLS to 29 (or guard retrain to the live feature set). Also cache 4d stale.</t>
+          <t>Pending. After M2.1-2.4 settle in production (one week of nightly precompute + dashboard observation with flag=false), flip use_structural_targets=true in config/config.json so build_data.py overlays structural fields into data.json. Frontend consumers (Plan tab, candidate ladder, target behavior) start picking up t1_structural/t2_structural in parallel with legacy t1/t2.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>server /api/ml cache-first + degenerate guard (done); align ml/feature_extractor.FEATURE_COLS to model n_features_in_ (pending)</t>
+          <t>Cutover requires: (1) one week of clean nightly precompute (no &gt;10 percent failure rate per scripts/precompute_targets.py exit code), (2) one clean te_regression run with errors &lt;= 1, (3) v2 dashboard frontend updated to read t1_structural fields when present (still falls back to t1 legacy when not). Until all three pass, leave flag=false.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -752,38 +752,38 @@
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="8" t="inlineStr"/>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>STRUCT-TARGETS-M25-CUTOVER</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>SCALE-2</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Targets</t>
+          <t>Auth · 500-user</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Structural targets · M2.5 — cutover gate (flip use_structural_targets=true)</t>
+          <t>Enforce per-user Supabase login (not shared basic-auth)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Pending. After M2.1-2.4 settle in production (one week of nightly precompute + dashboard observation with flag=false), flip use_structural_targets=true in config/config.json so build_data.py overlays structural fields into data.json. Frontend consumers (Plan tab, candidate ladder, target behavior) start picking up t1_structural/t2_structural in parallel with legacy t1/t2.</t>
+          <t>Per-user UserPrefs isolation (NAV/plans/watchlist) only holds when users authenticate via Supabase; if they share the single basic-auth (gari/Swing2026), UserPrefs falls back to per-browser localStorage = no true per-user separation</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Cutover requires: (1) one week of clean nightly precompute (no &gt;10 percent failure rate per scripts/precompute_targets.py exit code), (2) one clean te_regression run with errors &lt;= 1, (3) v2 dashboard frontend updated to read t1_structural fields when present (still falls back to t1 legacy when not). Until all three pass, leave flag=false.</t>
+          <t>Require Supabase login for multi-user; verify UserPrefs keys per auth id end-to-end (user-prefs.jsx setUser binds sb.auth.getUser)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -798,13 +798,13 @@
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="8" t="inlineStr"/>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="75" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SCALE-2</t>
+          <t>BUG-WEEKEND-PHANTOM-PICKS</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -814,22 +814,22 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Auth · 500-user</t>
+          <t>Bugs / Audit Ledger</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Enforce per-user Supabase login (not shared basic-auth)</t>
+          <t>Weekend phantom picks in audit ledger</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Per-user UserPrefs isolation (NAV/plans/watchlist) only holds when users authenticate via Supabase; if they share the single basic-auth (gari/Swing2026), UserPrefs falls back to per-browser localStorage = no true per-user separation</t>
+          <t>Audit ledger shows phantom picks on May 10 (Sun), May 16 (Sat), May 17 (Sun) — markets closed. Likely a scan-date assignment bug (writing today's date to a Friday pick that re-scans on Sat/Sun, or weekend cron runs that should skip).</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Require Supabase login for multi-user; verify UserPrefs keys per auth id end-to-end (user-prefs.jsx setUser binds sb.auth.getUser)</t>
+          <t>Trace which writer emits these entries: check run_daily_scan.sh weekday gate, swing_trade.py scan-date logic, and infra/prototype/build_audit_ledger.py date assignment. Weekend launchd should be gated; if it runs intentionally for paper-resolve, mark those rows as REPLAY not PICK.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -844,13 +844,13 @@
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="8" t="inlineStr"/>
     </row>
-    <row r="5" ht="75" customHeight="1">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>BUG-WEEKEND-PHANTOM-PICKS</t>
+          <t>DATA-BROKEN-IPO-CALENDAR</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -860,22 +860,22 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Bugs / Audit Ledger</t>
+          <t>Data / Calendars (broken)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Weekend phantom picks in audit ledger</t>
+          <t>ipo_calendar — NASDAQ API times out</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Audit ledger shows phantom picks on May 10 (Sun), May 16 (Sat), May 17 (Sun) — markets closed. Likely a scan-date assignment bug (writing today's date to a Friday pick that re-scans on Sat/Sun, or weekend cron runs that should skip).</t>
+          <t>NASDAQ public IPO API times out from this host (~30s no response). Calendar slot is wired but produces 0 rows.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Trace which writer emits these entries: check run_daily_scan.sh weekday gate, swing_trade.py scan-date logic, and infra/prototype/build_audit_ledger.py date assignment. Weekend launchd should be gated; if it runs intentionally for paper-resolve, mark those rows as REPLAY not PICK.</t>
+          <t>Investigate timeout first (UA headers / proxy / rate-limited IP) before alt-source. Candidate alternates: SEC S-1 filings via EDGAR full-text-search, IPO Monitor RSS, Yahoo Finance IPO page.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>DATA-BROKEN-IPO-CALENDAR</t>
+          <t>DATA-BROKEN-CONGRESSIONAL-TRADES</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -906,22 +906,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Data / Calendars (broken)</t>
+          <t>Data / Catalysts (broken)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>ipo_calendar — NASDAQ API times out</t>
+          <t>congressional_trades — sources dead</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>NASDAQ public IPO API times out from this host (~30s no response). Calendar slot is wired but produces 0 rows.</t>
+          <t>Senate Stock Watcher GitHub + S3 mirror both return dead/empty responses. The catalysts slot is wired but the scraper produces 0 rows.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Investigate timeout first (UA headers / proxy / rate-limited IP) before alt-source. Candidate alternates: SEC S-1 filings via EDGAR full-text-search, IPO Monitor RSS, Yahoo Finance IPO page.</t>
+          <t>Replace dead source with direct efts.sec.gov integration (Form 4 XBRL parsing); add House Clerk site fallback for House STOCK Act filings. Scope: 1-2d dev + XBRL schema work. Free-data only per CLAUDE.md.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>DATA-BROKEN-CONGRESSIONAL-TRADES</t>
+          <t>PARITY-REALTIME-DATA</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -952,22 +952,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Data / Catalysts (broken)</t>
+          <t>Data / Infrastructure / Platform Parity</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>congressional_trades — sources dead</t>
+          <t>Real-Time Data (streaming quotes)</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Senate Stock Watcher GitHub + S3 mirror both return dead/empty responses. The catalysts slot is wired but the scraper produces 0 rows.</t>
+          <t>Replace the 5-minute batch refresh with sub-second streaming quotes during market hours so charts + price ladder + Trade Plan PnL update in real time.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Replace dead source with direct efts.sec.gov integration (Form 4 XBRL parsing); add House Clerk site fallback for House STOCK Act filings. Scope: 1-2d dev + XBRL schema work. Free-data only per CLAUDE.md.</t>
+          <t>Use the Schwab websocket feed (already in the paid stack — no new license per CLAUDE.md) into a local pub/sub buffer; kairos sub-tabs subscribe via SSE/WebSocket from server.py; cache TTL pinned at 1s during RTH.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -988,7 +988,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>PARITY-REALTIME-DATA</t>
+          <t>BARSTORE-1</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -998,22 +998,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Data / Infrastructure / Platform Parity</t>
+          <t>Data Infra / Bar-Store</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Real-Time Data (streaming quotes)</t>
+          <t>SQLite daily_bars schema + read/write</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Replace the 5-minute batch refresh with sub-second streaming quotes during market hours so charts + price ladder + Trade Plan PnL update in real time.</t>
+          <t>No local OHLCV history store exists; scans re-fetch per-ticker daily bars from EODHD (~10K calls/day, ~68% of 2026-06-08 usage; tripped 95K quota guard). See docs/scope_bar_store.md.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Use the Schwab websocket feed (already in the paid stack — no new license per CLAUDE.md) into a local pub/sub buffer; kairos sub-tabs subscribe via SSE/WebSocket from server.py; cache TTL pinned at 1s during RTH.</t>
+          <t>Add daily_bars(ticker,date,o,h,l,c,v,adjusted_close,source,ingested_at) to data/swingtrade.db (PK ticker+date, idx). Idempotent upsert writer + DB reader + tests. SQLite stays primary; no new deps.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-1</t>
+          <t>BARSTORE-2</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1049,17 +1049,17 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>SQLite daily_bars schema + read/write</t>
+          <t>One-time 20yr backfill</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>No local OHLCV history store exists; scans re-fetch per-ticker daily bars from EODHD (~10K calls/day, ~68% of 2026-06-08 usage; tripped 95K quota guard). See docs/scope_bar_store.md.</t>
+          <t>One eod(ticker,from_date=2005) returns full history = 1 call/ticker; backfilling the universe is ~6-8K calls ONCE vs ~10K/day recurring.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Add daily_bars(ticker,date,o,h,l,c,v,adjusted_close,source,ingested_at) to data/swingtrade.db (PK ticker+date, idx). Idempotent upsert writer + DB reader + tests. SQLite stays primary; no new deps.</t>
+          <t>eodhd_client.backfill_history() pages the universe 1-call/ticker, paced under EODHD_SHARED_LIMITER (950/min), overnight launchd only, resumable. NO new license (uses existing EODHD).</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-2</t>
+          <t>BARSTORE-3</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1095,17 +1095,17 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>One-time 20yr backfill</t>
+          <t>DB-first failover in fetch_ohlcv_with_failover</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>One eod(ticker,from_date=2005) returns full history = 1 call/ticker; backfilling the universe is ~6-8K calls ONCE vs ~10K/day recurring.</t>
+          <t>Once history is local, scans/backtests must read DB-first and hit EODHD only for the current incomplete day + gaps.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>eodhd_client.backfill_history() pages the universe 1-call/ticker, paced under EODHD_SHARED_LIMITER (950/min), overnight launchd only, resumable. NO new license (uses existing EODHD).</t>
+          <t>Repoint data_fetcher.fetch_ohlcv_with_failover to read daily_bars first; EODHD fallback for today/gaps. Parity-check 100 tickers vs current cache/eodhd within float tol.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1120,13 +1120,13 @@
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="8" t="inlineStr"/>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="75" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-3</t>
+          <t>MODE-4</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1136,22 +1136,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Data Infra / Bar-Store</t>
+          <t>Decision Engine</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>DB-first failover in fetch_ohlcv_with_failover</t>
+          <t>Walk-forward validation of Phase-3 per-mode pillar weights</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Once history is local, scans/backtests must read DB-first and hit EODHD only for the current incomplete day + gaps.</t>
+          <t>MODE-3 shipped intuition-based pillar weights without backtest evidence (principle 7 override). Need walk-forward validation that the per-mode weights don't degrade vs the single-set baseline.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Repoint data_fetcher.fetch_ohlcv_with_failover to read daily_bars first; EODHD fallback for today/gaps. Parity-check 100 tickers vs current cache/eodhd within float tol.</t>
+          <t>scripts/validate_per_mode_weights.py: runs baseline backtest + 3 mode-weighted backtests (252d, min_score=50), compares WR/PF/maxDD/Sharpe per mode. Revert criterion: any mode ≤1.0× PF or ≤-5pp WR vs baseline → flip per_mode_pillar_reweight._enabled to false. See docs/per_mode_decisions_roadmap.md Phase 3.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1166,13 +1166,13 @@
       <c r="M11" s="3" t="inlineStr"/>
       <c r="N11" s="8" t="inlineStr"/>
     </row>
-    <row r="12" ht="75" customHeight="1">
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>MODE-4</t>
+          <t>SCALE-1</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1182,22 +1182,22 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine</t>
+          <t>Deployment · 500-user</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Walk-forward validation of Phase-3 per-mode pillar weights</t>
+          <t>Multi-worker server + concurrency load test</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>MODE-3 shipped intuition-based pillar weights without backtest evidence (principle 7 override). Need walk-forward validation that the per-mode weights don't degrade vs the single-set baseline.</t>
+          <t>Single uvicorn worker (uvicorn.run, no workers=); CPU-bound paths (65MB ML-file parse, scoring) block the event loop; untested at 500 concurrent on one Cloudflare tunnel</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>scripts/validate_per_mode_weights.py: runs baseline backtest + 3 mode-weighted backtests (252d, min_score=50), compares WR/PF/maxDD/Sharpe per mode. Revert criterion: any mode ≤1.0× PF or ≤-5pp WR vs baseline → flip per_mode_pillar_reweight._enabled to false. See docs/per_mode_decisions_roadmap.md Phase 3.</t>
+          <t>gunicorn/uvicorn --workers N (or app server), profile + offload blocking calls, run a 500-concurrent load test before certifying</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1212,13 +1212,13 @@
       <c r="M12" s="3" t="inlineStr"/>
       <c r="N12" s="8" t="inlineStr"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="75" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>SCALE-1</t>
+          <t>PARITY-PAPER-TRADING-RT</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1228,22 +1228,22 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Deployment · 500-user</t>
+          <t>Execution / Paper / Platform Parity</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Multi-worker server + concurrency load test</t>
+          <t>Real-Time Paper Trading</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Single uvicorn worker (uvicorn.run, no workers=); CPU-bound paths (65MB ML-file parse, scoring) block the event loop; untested at 500 concurrent on one Cloudflare tunnel</t>
+          <t>Execute simulated trades against live market prices via the Alpaca paper account; track fills, slippage and PnL in real time so paper validation mirrors what live trading would look like.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>gunicorn/uvicorn --workers N (or app server), profile + offload blocking calls, run a 500-concurrent load test before certifying</t>
+          <t>Extend executor.py to route signals through the Alpaca paper REST + websocket API; webhook fills back into cache/portfolio.json; expose a 'Paper Trade' toggle on the Trade Plan card. Partially built (executor.py --submit), needs always-on wrapper.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -1258,13 +1258,13 @@
       <c r="M13" s="3" t="inlineStr"/>
       <c r="N13" s="8" t="inlineStr"/>
     </row>
-    <row r="14" ht="75" customHeight="1">
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>PARITY-PAPER-TRADING-RT</t>
+          <t>REGIME-CONDITIONAL-MODELS</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -1274,22 +1274,22 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Execution / Paper / Platform Parity</t>
+          <t>ML / Accuracy</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Real-Time Paper Trading</t>
+          <t>Regime-conditional ML models (principle 5)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Execute simulated trades against live market prices via the Alpaca paper account; track fills, slippage and PnL in real time so paper validation mirrors what live trading would look like.</t>
+          <t>train separate direction models per regime instead of one spanning all; #1 accuracy lever</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Extend executor.py to route signals through the Alpaca paper REST + websocket API; webhook fills back into cache/portfolio.json; expose a 'Paper Trade' toggle on the Trade Plan card. Partially built (executor.py --submit), needs always-on wrapper.</t>
+          <t>ml/train.py regime split</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>REGIME-CONDITIONAL-MODELS</t>
+          <t>OPS-1</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1320,27 +1320,39 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>ML / Accuracy</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional ML models (principle 5)</t>
+          <t>Snapshot cleanup (scripts/cleanup_after_2026_05_16.sh)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>train separate direction models per regime instead of one spanning all; #1 accuracy lever</t>
+          <t>Pre-Saturday session migration created intermediate snapshot files safe to remove after a week.</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>ml/train.py regime split</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
+          <t>Run scripts/cleanup_after_2026_05_16.sh after 2026-05-16 cutoff.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>2 min</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Win: cleaner repo.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Calendar reminder for 2026-05-16.</t>
+        </is>
+      </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1348,15 +1360,19 @@
       </c>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16" ht="45" customHeight="1">
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>OPS-1</t>
+          <t>SCHWAB-REAUTH-PENDING</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1366,39 +1382,27 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Ops / Schwab (operational)</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Snapshot cleanup (scripts/cleanup_after_2026_05_16.sh)</t>
+          <t>Schwab re-auth to unlock option Greeks</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Pre-Saturday session migration created intermediate snapshot files safe to remove after a week.</t>
+          <t>refresh token expired (invalid_grant, 7-day). Run python3 schwab_auth.py oauth -&gt; real option premiums/Greeks flow into the Options calc (currently honest BS-model fallback).</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Run scripts/cleanup_after_2026_05_16.sh after 2026-05-16 cutoff.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>2 min</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>Win: cleaner repo.</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>Calendar reminder for 2026-05-16.</t>
-        </is>
-      </c>
+          <t>user action: schwab_auth.py oauth</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1406,11 +1410,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="3" t="inlineStr"/>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
+      <c r="N16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>SCHWAB-REAUTH-PENDING</t>
+          <t>QUANT-5</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1428,27 +1428,39 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Ops / Schwab (operational)</t>
+          <t>Quant</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Schwab re-auth to unlock option Greeks</t>
+          <t>Mover predictor v3 — NLP earnings tone + options flow features</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>refresh token expired (invalid_grant, 7-day). Run python3 schwab_auth.py oauth -&gt; real option premiums/Greeks flow into the Options calc (currently honest BS-model fallback).</t>
+          <t>v1 had leakage. v2 fixed leakage but AUC stuck at 0.546 — pure technical features at entry don't predict mover success.</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>user action: schwab_auth.py oauth</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr"/>
+          <t>Build v3 with NEW feature classes (don't retrain): NLP earnings-call tone embeddings, options-flow IV skew + UOA put/call delta, catalyst-conditional models (subset by tag). A6 logger captures most inputs going forward.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Caveat: exploratory research, not config-tuning.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Don't retrain v1/v2 — both definitive AUC 0.546 negative.</t>
+        </is>
+      </c>
       <c r="K17" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1456,15 +1468,19 @@
       </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="8" t="inlineStr"/>
-    </row>
-    <row r="18" ht="60" customHeight="1">
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="165" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>QUANT-5</t>
+          <t>TV-RATING-CROSS-CHECK</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -1474,37 +1490,37 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Quant</t>
+          <t>Signals / Cross-Check</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Mover predictor v3 — NLP earnings tone + options flow features</t>
+          <t>Validate (or zero out) the ±3 TV-rating tech-score bonus</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>v1 had leakage. v2 fixed leakage but AUC stuck at 0.546 — pure technical features at entry don't predict mover success.</t>
+          <t>DISCOVERY 2026-05-11: TV-rating ±3 score bonus has been live in analysis.py:8627 for some time, modifying every BUY signal's technical pillar score. NO _validations entry, NO Wilson-CI, NO walk-forward justification for the ±3 magnitude. Worse: tv_rating was never captured on the 689 closed trades in picks_history or 1,301 signal_log entries — retroactive validation is impossible. Violates Principle 1 (n&lt;30 refusal) + Principle 7 (no knob-tweaking without evidence).</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Build v3 with NEW feature classes (don't retrain): NLP earnings-call tone embeddings, options-flow IV skew + UOA put/call delta, catalyst-conditional models (subset by tag). A6 logger captures most inputs going forward.</t>
+          <t>Phase 1 (SHIPPED 2026-05-11): (a) tv_bonus zeroed in analysis.py:8627 — score no longer mutated; (b) tv_recommendation + tv_rec_value + buy/sell/neutral counts now logged per signal in signal_tracker.log_signals() so prospective evidence accumulates; (c) tv_rating still surfaced in tech['details'] as INFORMATIONAL only — no score impact. Phase 2 (PENDING n&gt;=30, est. 6-12 weeks): run Wilson-LB(BUY|TV STRONG_BUY) vs Wilson-LB(BUY) over the prospectively-logged signals. If the agreement-conditional Wilson-LB beats unconditional by a meaningful margin (&gt;=3pp), re-enable with a magnitude justified by the regression. If not, kill the cross-check permanently (Principle 4 falsification — do not retune, do not lower the threshold).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>Phase 1: hours (done). Phase 2: hours of analysis + calendar wait for n&gt;=30.</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Caveat: exploratory research, not config-tuning.</t>
+          <t>Mechanism (Principle 2): TV rating is an independent server-side aggregation of ~26 indicators. Two independent technical aggregations may improve precision over our 5-pillar score alone. Falsification (Principle 4): if agreement-conditional Wilson-LB &lt;= unconditional after n&gt;=30, the cross-check has no edge — kill, don't retune. Risk of CURRENT state (Phase 1): we have been over-weighting TV-STRONG_BUY signals by +3 tech-pts with zero evidence; this could have systematically biased BUY selection. Capping at 0 removes that bias going forward but does not undo past trade selection bias.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Don't retrain v1/v2 — both definitive AUC 0.546 negative.</t>
+          <t>Default apply_to_score=false locked. Validation requires logged tv_rating on &gt;=30 CLOSED BUY trades (currently 0). Earliest Phase-2 validation window: ~6-12 weeks of scans from 2026-05-11. Pairs with the v2 dashboard TV sub-tab (infra/prototype/subtabs/tv/) which is iframe-only today. Do NOT add per-mode / per-regime elaboration until Phase 2 evidence justifies even the basic bonus.</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
@@ -1516,17 +1532,17 @@
       <c r="M18" s="3" t="inlineStr"/>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="165" customHeight="1">
+          <t>Phase 1 smoke: run python3 swing_trade.py and confirm (1) tech['details']['tv_rating'] still appears in deep-dive output labeled 'informational — bonus disabled pending validation'; (2) signal_log.json entries for new scans contain tv_recommendation + tv_rec_value + buy/sell/neutral_count populated. Phase 2 trigger: when `python3 -c 'import json; print(sum(1 for r in json.load(open("data/signal_log.json")) if r.get("tv_recommendation") and r.get("result")))'` &gt;= 30, run the agreement-conditional Wilson-LB analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>TV-RATING-CROSS-CHECK</t>
+          <t>TEST-MAE-MFE</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1536,39 +1552,27 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Signals / Cross-Check</t>
+          <t>Testing / Validation (Tier 1)</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Validate (or zero out) the ±3 TV-rating tech-score bonus</t>
+          <t>MAE / MFE Analyzer — tune stops + targets from data</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>DISCOVERY 2026-05-11: TV-rating ±3 score bonus has been live in analysis.py:8627 for some time, modifying every BUY signal's technical pillar score. NO _validations entry, NO Wilson-CI, NO walk-forward justification for the ±3 magnitude. Worse: tv_rating was never captured on the 689 closed trades in picks_history or 1,301 signal_log entries — retroactive validation is impossible. Violates Principle 1 (n&lt;30 refusal) + Principle 7 (no knob-tweaking without evidence).</t>
+          <t>Maximum Adverse Excursion vs Maximum Favorable Excursion analyzer. signal_log.json already tracks mae_pct + mfe_pct for closed trades. Output: 'Stops triggered at -5% on winners that later hit +20% → stops too tight' or 'Trades exited at +6% target left avg +12% on table → targets too conservative'. Directly improves trade-plan math.</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (SHIPPED 2026-05-11): (a) tv_bonus zeroed in analysis.py:8627 — score no longer mutated; (b) tv_recommendation + tv_rec_value + buy/sell/neutral counts now logged per signal in signal_tracker.log_signals() so prospective evidence accumulates; (c) tv_rating still surfaced in tech['details'] as INFORMATIONAL only — no score impact. Phase 2 (PENDING n&gt;=30, est. 6-12 weeks): run Wilson-LB(BUY|TV STRONG_BUY) vs Wilson-LB(BUY) over the prospectively-logged signals. If the agreement-conditional Wilson-LB beats unconditional by a meaningful margin (&gt;=3pp), re-enable with a magnitude justified by the regression. If not, kill the cross-check permanently (Principle 4 falsification — do not retune, do not lower the threshold).</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Phase 1: hours (done). Phase 2: hours of analysis + calendar wait for n&gt;=30.</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Mechanism (Principle 2): TV rating is an independent server-side aggregation of ~26 indicators. Two independent technical aggregations may improve precision over our 5-pillar score alone. Falsification (Principle 4): if agreement-conditional Wilson-LB &lt;= unconditional after n&gt;=30, the cross-check has no edge — kill, don't retune. Risk of CURRENT state (Phase 1): we have been over-weighting TV-STRONG_BUY signals by +3 tech-pts with zero evidence; this could have systematically biased BUY selection. Capping at 0 removes that bias going forward but does not undo past trade selection bias.</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>Default apply_to_score=false locked. Validation requires logged tv_rating on &gt;=30 CLOSED BUY trades (currently 0). Earliest Phase-2 validation window: ~6-12 weeks of scans from 2026-05-11. Pairs with the v2 dashboard TV sub-tab (infra/prototype/subtabs/tv/) which is iframe-only today. Do NOT add per-mode / per-regime elaboration until Phase 2 evidence justifies even the basic bonus.</t>
-        </is>
-      </c>
+          <t>Read signal_log.json closed entries; scatter-plot mae vs realized PnL + mfe vs realized PnL; quantile bins (10/25/50/75/90); render as a new Testing tab card. Effort ~30min — data already there.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr"/>
       <c r="K19" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1576,11 +1580,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="8" t="inlineStr">
-        <is>
-          <t>Phase 1 smoke: run python3 swing_trade.py and confirm (1) tech['details']['tv_rating'] still appears in deep-dive output labeled 'informational — bonus disabled pending validation'; (2) signal_log.json entries for new scans contain tv_recommendation + tv_rec_value + buy/sell/neutral_count populated. Phase 2 trigger: when `python3 -c 'import json; print(sum(1 for r in json.load(open("data/signal_log.json")) if r.get("tv_recommendation") and r.get("result")))'` &gt;= 30, run the agreement-conditional Wilson-LB analysis.</t>
-        </is>
-      </c>
+      <c r="N19" s="8" t="inlineStr"/>
     </row>
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>TEST-MAE-MFE</t>
+          <t>TEST-MC-BOOTSTRAP</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -1603,17 +1603,17 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>MAE / MFE Analyzer — tune stops + targets from data</t>
+          <t>Monte Carlo Bootstrap — confidence intervals on Sharpe/PF/WR</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Maximum Adverse Excursion vs Maximum Favorable Excursion analyzer. signal_log.json already tracks mae_pct + mfe_pct for closed trades. Output: 'Stops triggered at -5% on winners that later hit +20% → stops too tight' or 'Trades exited at +6% target left avg +12% on table → targets too conservative'. Directly improves trade-plan math.</t>
+          <t>Randomly resample closed trades 10,000x to build distributions over each metric. Wilson LB only covers WR; this covers Sharpe, Sortino, PF, max-DD, hit-rate, payoff ratio. Output: 'Sharpe 1.42, 95% CI [0.88, 1.94]' — you would know whether 1.42 is robust or noise. Standard hedge-fund metric, supports principle #1 (statistical rigor).</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Read signal_log.json closed entries; scatter-plot mae vs realized PnL + mfe vs realized PnL; quantile bins (10/25/50/75/90); render as a new Testing tab card. Effort ~30min — data already there.</t>
+          <t>Numpy bootstrap on signal_log trade PnL array, k=10000 resamples; compute distributions over each metric; render percentile bands. Effort 1-2hr.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>TEST-MC-BOOTSTRAP</t>
+          <t>TEST-PERMUTATION</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Monte Carlo Bootstrap — confidence intervals on Sharpe/PF/WR</t>
+          <t>Permutation Test — is the edge REAL or coin flip?</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Randomly resample closed trades 10,000x to build distributions over each metric. Wilson LB only covers WR; this covers Sharpe, Sortino, PF, max-DD, hit-rate, payoff ratio. Output: 'Sharpe 1.42, 95% CI [0.88, 1.94]' — you would know whether 1.42 is robust or noise. Standard hedge-fund metric, supports principle #1 (statistical rigor).</t>
+          <t>Randomly shuffle BUY/SELL/AVOID labels on historical signals 1000x, recompute strategy returns. If real returns are not significantly better than scrambled returns, there is no edge. Direct test of principle #4 (adversarial mindset / falsification). Output: 'Real strategy: +18.7%. Random labels (1000 sims): +0.2% +/- 4.1%. p-value: 0.0001'.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Numpy bootstrap on signal_log trade PnL array, k=10000 resamples; compute distributions over each metric; render percentile bands. Effort 1-2hr.</t>
+          <t>Shuffle decision-column of signal_log 1000x; recompute portfolio return per shuffle; rank real return vs null distribution; report p-value. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>TEST-PERMUTATION</t>
+          <t>TEST-REGIME-COND</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -1695,17 +1695,17 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Permutation Test — is the edge REAL or coin flip?</t>
+          <t>Regime-Conditional Performance — where does it work?</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Randomly shuffle BUY/SELL/AVOID labels on historical signals 1000x, recompute strategy returns. If real returns are not significantly better than scrambled returns, there is no edge. Direct test of principle #4 (adversarial mindset / falsification). Output: 'Real strategy: +18.7%. Random labels (1000 sims): +0.2% +/- 4.1%. p-value: 0.0001'.</t>
+          <t>Partition closed trades by regime (risk_on_trending / choppy / risk_off / panic) and compute WR / PF / Sharpe per regime. Per principle #5 (regime conditioning over averages). Example output: 'Trend Continuation WR: 41% overall · 62% in risk_on_trending · 18% in choppy'. Tells you which sleeves to size up/down per regime.</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Shuffle decision-column of signal_log 1000x; recompute portfolio return per shuffle; rank real return vs null distribution; report p-value. Effort ~1hr.</t>
+          <t>Group signal_log entries by regime_at_signal (already logged); compute Wilson LB on WR + bootstrapped PF/Sharpe per regime; output a (setup x regime) heatmap. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1720,38 +1720,38 @@
       <c r="M22" s="3" t="inlineStr"/>
       <c r="N22" s="8" t="inlineStr"/>
     </row>
-    <row r="23" ht="90" customHeight="1">
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>TEST-REGIME-COND</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>PARITY-BACKTEST-UI</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Testing / Validation (Tier 1)</t>
+          <t>Backtesting / Platform Parity</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Regime-Conditional Performance — where does it work?</t>
+          <t>In-app Backtesting UI</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Partition closed trades by regime (risk_on_trending / choppy / risk_off / panic) and compute WR / PF / Sharpe per regime. Per principle #5 (regime conditioning over averages). Example output: 'Trend Continuation WR: 41% overall · 62% in risk_on_trending · 18% in choppy'. Tells you which sleeves to size up/down per regime.</t>
+          <t>Expose backtest.py + walk_forward_v2.py inside the kairos UI — a user picks a strategy/date range/universe and runs it without dropping to the terminal.</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Group signal_log entries by regime_at_signal (already logged); compute Wilson LB on WR + bootstrapped PF/Sharpe per regime; output a (setup x regime) heatmap. Effort ~1hr.</t>
+          <t>Add a 'Backtest' workspace in the kairos sidebar; wire a form to a /v2/backtest endpoint that shells out to backtest.py and streams stdout via SSE; render Sharpe / PF / Wilson-LB / equity curve when the run completes.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>PARITY-BACKTEST-UI</t>
+          <t>BUG-MISSING-D1S</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1782,22 +1782,22 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Backtesting / Platform Parity</t>
+          <t>Bugs / Audit Ledger</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>In-app Backtesting UI</t>
+          <t>4 missing D1s for May 15 (out of 87)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Expose backtest.py + walk_forward_v2.py inside the kairos UI — a user picks a strategy/date range/universe and runs it without dropping to the terminal.</t>
+          <t>4 of 87 May-15 picks have null D1 (next-day close). Probably thin EODHD coverage on small-caps — acceptable noise band but worth confirming.</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Add a 'Backtest' workspace in the kairos sidebar; wire a form to a /v2/backtest endpoint that shells out to backtest.py and streams stdout via SSE; render Sharpe / PF / Wilson-LB / equity curve when the run completes.</t>
+          <t>Identify the 4 tickers; check EODHD eod() response for each on 2026-05-16; if EODHD returned null, document as known-limitation; if EODHD returned a value, fix the ingest. Effort ~20min.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>BUG-MISSING-D1S</t>
+          <t>PARITY-CHANNEL-BAR</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1828,22 +1828,22 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Bugs / Audit Ledger</t>
+          <t>Chart Indicators / Platform Parity</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>4 missing D1s for May 15 (out of 87)</t>
+          <t>Channel Bar overlay</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>4 of 87 May-15 picks have null D1 (next-day close). Probably thin EODHD coverage on small-caps — acceptable noise band but worth confirming.</t>
+          <t>Donchian / Keltner / Bollinger envelope overlay on the chart — top + bottom band with mid-line.</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Identify the 4 tickers; check EODHD eod() response for each on 2026-05-16; if EODHD returned null, document as known-limitation; if EODHD returned a value, fix the ingest. Effort ~20min.</t>
+          <t>Compute channels via pandas-ta in feature_extractor.py (or live in chart.js using bar data); render as semi-transparent band; toggle in the Chart sub-tab control bar.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>PARITY-CHANNEL-BAR</t>
+          <t>PARITY-RBI-GBI-WINDOW</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -1879,17 +1879,17 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Channel Bar overlay</t>
+          <t>RBI/GBI Window (regime bias bands)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Donchian / Keltner / Bollinger envelope overlay on the chart — top + bottom band with mid-line.</t>
+          <t>Color-coded vertical bands on the chart timeline showing risk-on (green/GBI) vs risk-off (red/RBI) regime windows so the user can see at-a-glance whether prior price action happened in a hostile or friendly regime.</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Compute channels via pandas-ta in feature_extractor.py (or live in chart.js using bar data); render as semi-transparent band; toggle in the Chart sub-tab control bar.</t>
+          <t>Read cache/regime_history.json and draw vertical color bands at each regime transition on the chart canvas; tooltip explains the regime classification (4-regime model: risk_on_trending / risk_on_choppy / risk_off_trending / panic).</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1904,13 +1904,13 @@
       <c r="M26" s="3" t="inlineStr"/>
       <c r="N26" s="8" t="inlineStr"/>
     </row>
-    <row r="27" ht="60" customHeight="1">
+    <row r="27" ht="45" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>PARITY-RBI-GBI-WINDOW</t>
+          <t>CLEAN-HOT-SECTORS-DEAD</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -1920,22 +1920,22 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Chart Indicators / Platform Parity</t>
+          <t>Code Cleanup</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>RBI/GBI Window (regime bias bands)</t>
+          <t>panelHotSectors() dead-code in kairos.html</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Color-coded vertical bands on the chart timeline showing risk-on (green/GBI) vs risk-off (red/RBI) regime windows so the user can see at-a-glance whether prior price action happened in a hostile or friendly regime.</t>
+          <t>Hot Sectors panel was removed from the Signal Scanner grid but the panelHotSectors() function is still defined in kairos.html — dead code.</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Read cache/regime_history.json and draw vertical color bands at each regime transition on the chart canvas; tooltip explains the regime classification (4-regime model: risk_on_trending / risk_on_choppy / risk_off_trending / panic).</t>
+          <t>grep for panelHotSectors callers; delete function + any unused helpers; verify no console errors. Effort ~2min.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-HOT-SECTORS-DEAD</t>
+          <t>CLEAN-4</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1966,27 +1966,39 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>panelHotSectors() dead-code in kairos.html</t>
+          <t>scripts/migrate_role_capabilities.py — cleanup after 2026-05-16</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Hot Sectors panel was removed from the Signal Scanner grid but the panelHotSectors() function is still defined in kairos.html — dead code.</t>
+          <t>One-shot CapStudio backfill. Already run. Tied to OPS-1 cleanup window.</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>grep for panelHotSectors callers; delete function + any unused helpers; verify no console errors. Effort ~2min.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr"/>
+          <t>Delete during OPS-1 cleanup pass after 2026-05-16.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>1 min</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Win: -X lines.</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Couples with OPS-1.</t>
+        </is>
+      </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1994,15 +2006,19 @@
       </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr"/>
-      <c r="N28" s="8" t="inlineStr"/>
-    </row>
-    <row r="29" ht="45" customHeight="1">
+      <c r="N28" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="60" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-4</t>
+          <t>DATA-FUTURE-EARNINGS-CAL-PIT</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -2012,39 +2028,27 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Data / Calendars (future)</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>scripts/migrate_role_capabilities.py — cleanup after 2026-05-16</t>
+          <t>earnings_calendar_pit — point-in-time integrity</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>One-shot CapStudio backfill. Already run. Tied to OPS-1 cleanup window.</t>
+          <t>Earnings calendar with point-in-time integrity (what was expected when). Needed for clean PEAD backtest replay; today's calendar uses the most-recent snapshot only, which leaks future revisions into prior dates.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Delete during OPS-1 cleanup pass after 2026-05-16.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>1 min</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>Win: -X lines.</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>Couples with OPS-1.</t>
-        </is>
-      </c>
+          <t>Snapshot the EODHD earnings calendar daily into a versioned earnings_calendar_history table; join on (ticker, report_date, snapshot_date) for PIT correctness in PEAD backtests.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="5" t="inlineStr"/>
+      <c r="J29" s="5" t="inlineStr"/>
       <c r="K29" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -2052,19 +2056,15 @@
       </c>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr"/>
-      <c r="N29" s="8" t="inlineStr">
-        <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="60" customHeight="1">
+      <c r="N29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30" ht="45" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-EARNINGS-CAL-PIT</t>
+          <t>DATA-FUTURE-ECONOMIC-CAL</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -2079,17 +2079,17 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>earnings_calendar_pit — point-in-time integrity</t>
+          <t>economic_calendar — CPI/PCE/NFP/FOMC dates</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Earnings calendar with point-in-time integrity (what was expected when). Needed for clean PEAD backtest replay; today's calendar uses the most-recent snapshot only, which leaks future revisions into prior dates.</t>
+          <t>Macro event calendar with consensus expectations. No source wired today; the pre-FOMC sleeve uses hard-coded FOMC dates and there is no CPI/PCE/NFP awareness.</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Snapshot the EODHD earnings calendar daily into a versioned earnings_calendar_history table; join on (ticker, report_date, snapshot_date) for PIT correctness in PEAD backtests.</t>
+          <t>Investing.com calendar scrape OR Trading Economics free tier; daily refresh; write to economic_calendar; feed pre-FOMC sleeve + risk_off blackout windows.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-ECONOMIC-CAL</t>
+          <t>DATA-FUTURE-FDA-CAL</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -2125,17 +2125,17 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>economic_calendar — CPI/PCE/NFP/FOMC dates</t>
+          <t>fda_calendar — PDUFA / AdCom dates</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Macro event calendar with consensus expectations. No source wired today; the pre-FOMC sleeve uses hard-coded FOMC dates and there is no CPI/PCE/NFP awareness.</t>
+          <t>FDA decision calendar (PDUFA dates, Advisory Committee meetings) for biotech catalyst tracking.</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Investing.com calendar scrape OR Trading Economics free tier; daily refresh; write to economic_calendar; feed pre-FOMC sleeve + risk_off blackout windows.</t>
+          <t>FDA public calendar scrape + BiopharmCatalyst free RSS; write to fda_calendar; surface as catalyst tier in any biotech sleeve.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-FDA-CAL</t>
+          <t>DATA-EMPTY-SPLITS-CALENDAR</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -2166,22 +2166,22 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Data / Calendars (future)</t>
+          <t>Data / Corporate Actions (empty by sample)</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>fda_calendar — PDUFA / AdCom dates</t>
+          <t>splits_calendar — 0 splits in current universe sample</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>FDA decision calendar (PDUFA dates, Advisory Committee meetings) for biotech catalyst tracking.</t>
+          <t>corporate_actions table populates from EODHD but the current universe sample (449 tickers) had 0 splits in the recent window. Calendar reads empty.</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>FDA public calendar scrape + BiopharmCatalyst free RSS; write to fda_calendar; surface as catalyst tier in any biotech sleeve.</t>
+          <t>Expand corporate-actions polling universe to S&amp;P 500 + Russell 1000 (universe list already available); 1-line change in the populator script.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-SPLITS-CALENDAR</t>
+          <t>DATA-EMPTY-MODEL-CALIBRATION</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -2212,22 +2212,22 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Data / Corporate Actions (empty by sample)</t>
+          <t>Data / ML (empty by design)</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>splits_calendar — 0 splits in current universe sample</t>
+          <t>model_calibration — waiting on realization</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>corporate_actions table populates from EODHD but the current universe sample (449 tickers) had 0 splits in the recent window. Calendar reads empty.</t>
+          <t>Calibration metrics table has no rows because the 5-20 day prediction horizons have not elapsed yet (today's predictions realize over 1-4 weeks).</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Expand corporate-actions polling universe to S&amp;P 500 + Russell 1000 (universe list already available); 1-line change in the populator script.</t>
+          <t>No code action; populates passively as time passes. Re-check after 2026-06-15 (30d post-shipping).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-MODEL-CALIBRATION</t>
+          <t>DATA-EMPTY-VAR-BREACHES</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2258,22 +2258,22 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Data / ML (empty by design)</t>
+          <t>Data / Risk (empty by design)</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>model_calibration — waiting on realization</t>
+          <t>var_breaches — waiting on snapshots + drawdown</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Calibration metrics table has no rows because the 5-20 day prediction horizons have not elapsed yet (today's predictions realize over 1-4 weeks).</t>
+          <t>VaR breach log empty because (1) daily portfolio_risk snapshots are still ramping up and (2) no real drawdown day has happened to trigger a breach.</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>No code action; populates passively as time passes. Re-check after 2026-06-15 (30d post-shipping).</t>
+          <t>No code action; populates passively. Re-check after first portfolio drawdown &gt;2% or after 60 daily snapshots.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -2288,13 +2288,13 @@
       <c r="M34" s="3" t="inlineStr"/>
       <c r="N34" s="8" t="inlineStr"/>
     </row>
-    <row r="35" ht="45" customHeight="1">
+    <row r="35" ht="60" customHeight="1">
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-VAR-BREACHES</t>
+          <t>DATA-FUTURE-INSIDER-EDGAR</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -2304,22 +2304,22 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Data / Risk (empty by design)</t>
+          <t>Data / SEC EDGAR (future)</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>var_breaches — waiting on snapshots + drawdown</t>
+          <t>insider_transactions via Form 4 XBRL</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>VaR breach log empty because (1) daily portfolio_risk snapshots are still ramping up and (2) no real drawdown day has happened to trigger a breach.</t>
+          <t>Per-ticker insider buy/sell stream sourced direct from SEC Form 4 filings. Today sourced indirectly via Finviz Elite bulk; direct EDGAR is point-in-time accurate and free.</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>No code action; populates passively. Re-check after first portfolio drawdown &gt;2% or after 60 daily snapshots.</t>
+          <t>Build Form 4 XBRL parser; daily ingest from efts.sec.gov; write to insider_transactions table; reconcile against Finviz bulk for cross-check.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -2334,13 +2334,13 @@
       <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="8" t="inlineStr"/>
     </row>
-    <row r="36" ht="60" customHeight="1">
+    <row r="36" ht="45" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-INSIDER-EDGAR</t>
+          <t>DATA-FUTURE-INSTITUTIONAL-EDGAR</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>insider_transactions via Form 4 XBRL</t>
+          <t>institutional_holdings via 13F XBRL</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker insider buy/sell stream sourced direct from SEC Form 4 filings. Today sourced indirectly via Finviz Elite bulk; direct EDGAR is point-in-time accurate and free.</t>
+          <t>Per-ticker institutional ownership tracking (Form 13F, quarterly). Useful for the Smart Money pillar; today only Finviz inst_own_pct snapshot.</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Build Form 4 XBRL parser; daily ingest from efts.sec.gov; write to insider_transactions table; reconcile against Finviz bulk for cross-check.</t>
+          <t>13F XBRL parser; quarterly ingest from EDGAR; write to institutional_holdings table with the 45-day reporting lag accounted for in any backtest joins.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-INSTITUTIONAL-EDGAR</t>
+          <t>DATA-FUTURE-CONGRESSIONAL-EDGAR</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -2396,22 +2396,22 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Data / SEC EDGAR (future)</t>
+          <t>Data / SEC EDGAR (future, alt for broken)</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>institutional_holdings via 13F XBRL</t>
+          <t>congressional_trades via EDGAR / House Clerk (alt source)</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker institutional ownership tracking (Form 13F, quarterly). Useful for the Smart Money pillar; today only Finviz inst_own_pct snapshot.</t>
+          <t>Alternate sourcing for congressional trades after Senate Stock Watcher death (see DATA-BROKEN-CONGRESSIONAL-TRADES). Direct from House Clerk + Senate eFD.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>13F XBRL parser; quarterly ingest from EDGAR; write to institutional_holdings table with the 45-day reporting lag accounted for in any backtest joins.</t>
+          <t>Scrape House STOCK Act PTR PDFs (House Clerk site); Senate eFD JSON; merge into normalized congressional_trades table.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-CONGRESSIONAL-EDGAR</t>
+          <t>SUPABASE-SYNC-VERIFY</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -2442,22 +2442,22 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Data / SEC EDGAR (future, alt for broken)</t>
+          <t>Data / Supabase</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>congressional_trades via EDGAR / House Clerk (alt source)</t>
+          <t>Verify supabase_analysis_sync actually writes</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Alternate sourcing for congressional trades after Senate Stock Watcher death (see DATA-BROKEN-CONGRESSIONAL-TRADES). Direct from House Clerk + Senate eFD.</t>
+          <t>confirm sync_scan writes (psycopg2 raw SQL not .table API); not silent no-op</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Scrape House STOCK Act PTR PDFs (House Clerk site); Senate eFD JSON; merge into normalized congressional_trades table.</t>
+          <t>supabase_analysis_sync.py</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -2472,13 +2472,13 @@
       <c r="M38" s="3" t="inlineStr"/>
       <c r="N38" s="8" t="inlineStr"/>
     </row>
-    <row r="39" ht="45" customHeight="1">
+    <row r="39" ht="60" customHeight="1">
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>SUPABASE-SYNC-VERIFY</t>
+          <t>DATA-EMPTY-PROD-ENGINE-DEFERRED</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -2488,22 +2488,22 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Data / Supabase</t>
+          <t>Data / Telemetry (deferred for safety)</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Verify supabase_analysis_sync actually writes</t>
+          <t>8 empty slots — production-engine touches deferred</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>confirm sync_scan writes (psycopg2 raw SQL not .table API); not silent no-op</t>
+          <t>8 telemetry/data slots remain empty because populating them requires editing backtest.py / executor.py / signal_filter.py / analysis.py. Deliberately deferred to avoid risk to the live scan + exec paths.</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>supabase_analysis_sync.py</t>
+          <t>Enumerate the 8 specifically and grade each one for in-place vs side-car instrumentation. Side-car (write to telemetry DB without changing decision flow) is preferred over hot-path edits.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -2518,13 +2518,13 @@
       <c r="M39" s="3" t="inlineStr"/>
       <c r="N39" s="8" t="inlineStr"/>
     </row>
-    <row r="40" ht="60" customHeight="1">
+    <row r="40" ht="45" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-PROD-ENGINE-DEFERRED</t>
+          <t>BARSTORE-4</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -2534,22 +2534,22 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Data / Telemetry (deferred for safety)</t>
+          <t>Data Infra / Bar-Store</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>8 empty slots — production-engine touches deferred</t>
+          <t>Daily incremental via bulk_eod</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>8 telemetry/data slots remain empty because populating them requires editing backtest.py / executor.py / signal_filter.py / analysis.py. Deliberately deferred to avoid risk to the live scan + exec paths.</t>
+          <t>After backfill, only the latest bar is needed daily; bulk_eod returns the whole exchange in 1 call.</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Enumerate the 8 specifically and grade each one for in-place vs side-car instrumentation. Side-car (write to telemetry DB without changing decision flow) is preferred over hot-path edits.</t>
+          <t>Daily launchd job: 1 bulk_eod(exchange) appends last-day bar for all tickers into daily_bars. Target &lt;=2 EODHD calls/day total for OHLCV.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-4</t>
+          <t>BARSTORE-5</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
@@ -2585,17 +2585,17 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Daily incremental via bulk_eod</t>
+          <t>Corporate-action re-adjustment</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>After backfill, only the latest bar is needed daily; bulk_eod returns the whole exchange in 1 call.</t>
+          <t>Stored history must stay split/div-adjusted; a new split re-bases all prior bars. This is where data-integrity bugs hide.</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Daily launchd job: 1 bulk_eod(exchange) appends last-day bar for all tickers into daily_bars. Target &lt;=2 EODHD calls/day total for OHLCV.</t>
+          <t>Store raw + adjusted_close; small daily job re-adjusts history on split/div events (EODHD div/splits endpoints). Validate no adjustment drift.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -2610,13 +2610,13 @@
       <c r="M41" s="3" t="inlineStr"/>
       <c r="N41" s="8" t="inlineStr"/>
     </row>
-    <row r="42" ht="45" customHeight="1">
+    <row r="42" ht="60" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-5</t>
+          <t>BARSTORE-6</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -2631,17 +2631,17 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Corporate-action re-adjustment</t>
+          <t>Delisted backfill -&gt; survivorship fix</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Stored history must stay split/div-adjusted; a new split re-bases all prior bars. This is where data-integrity bugs hide.</t>
+          <t>Honest backtests need delisted tickers' history + point-in-time membership (membership snapshots already DONE via AIPRED-SURVIVORSHIP). Unblocks audit #1.</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Store raw + adjusted_close; small daily job re-adjusts history on split/div events (EODHD div/splits endpoints). Validate no adjustment drift.</t>
+          <t>Backfill delisted-ticker history into daily_bars; point walk_forward_v2 at DB over 20yr. Enables survivorship-bias-free backtests + free validation of staged accuracy tweaks.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-6</t>
+          <t>EODHD-WIRES-VALIDATE</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -2672,22 +2672,22 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Data Infra / Bar-Store</t>
+          <t>Data Wiring (validate)</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Delisted backfill -&gt; survivorship fix</t>
+          <t>Validate EODHD-side wires on quota reset</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Honest backtests need delisted tickers' history + point-in-time membership (membership snapshots already DONE via AIPRED-SURVIVORSHIP). Unblocks audit #1.</t>
+          <t>DCF net-debt/FCF + per-name beta + Book Risk crowding are code-complete + fallback-safe but untested against live EODHD (quota was exhausted). Confirm real values flow after reset.</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Backfill delisted-ticker history into daily_bars; point walk_forward_v2 at DB over 20yr. Enables survivorship-bias-free backtests + free validation of staged accuracy tweaks.</t>
+          <t>Stocksmith.html /api/fundamentals consumers</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2702,13 +2702,13 @@
       <c r="M43" s="3" t="inlineStr"/>
       <c r="N43" s="8" t="inlineStr"/>
     </row>
-    <row r="44" ht="60" customHeight="1">
+    <row r="44" ht="75" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>EODHD-WIRES-VALIDATE</t>
+          <t>OVERVIEW-VERDICT-RECON</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -2718,22 +2718,22 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Data Wiring (validate)</t>
+          <t>Decision Engine</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Validate EODHD-side wires on quota reset</t>
+          <t>Reconcile compute_final_verdict (stage) vs decisions_by_mode</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>DCF net-debt/FCF + per-name beta + Book Risk crowding are code-complete + fallback-safe but untested against live EODHD (quota was exhausted). Confirm real values flow after reset.</t>
+          <t>Two engines emit different swing score+verdict for the same name (FTNT: stage=BUY/67 vs decisions_by_mode.swing=WATCH/57). decisions_by_mode omits the catalyst-sleeve EXTENDED-entry relaxation that compute_final_verdict applies, so they disagree.</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html /api/fundamentals consumers</t>
+          <t>Have decisions_by_mode consume the same relaxation OR emit a diverges-from-composite flag; decide direction after the entry-quality EXTENDED/MISSED A/B validation lands. Display already fixed (overview.js binds stage).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>OVERVIEW-VERDICT-RECON</t>
+          <t>KAIROS-TRAFFIC-LIGHT-INPUTS</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -2764,22 +2764,22 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine</t>
+          <t>Detail Lens / Traffic Lights</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Reconcile compute_final_verdict (stage) vs decisions_by_mode</t>
+          <t>Per-ticker risk/fundamentals inputs for lens dots</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Two engines emit different swing score+verdict for the same name (FTNT: stage=BUY/67 vs decisions_by_mode.swing=WATCH/57). decisions_by_mode omits the catalyst-sleeve EXTENDED-entry relaxation that compute_final_verdict applies, so they disagree.</t>
+          <t>Wire t.f_score · t.altman_z · t.roic · t.wacc · t.sharpe_1y · t.dd_recovery_months · t.peer_rank · t.is_held into build_data.py. _qdComputeLensStatus has cascading fallbacks (PEG → fund_score → F-score; beta → kelly → Sharpe), so dots upgrade automatically as fields land.</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Have decisions_by_mode consume the same relaxation OR emit a diverges-from-composite flag; decide direction after the entry-quality EXTENDED/MISSED A/B validation lands. Display already fixed (overview.js binds stage).</t>
+          <t>Compute in analysis.py / portfolio.py: Piotroski F (existing data), Altman Z (existing data), ROIC vs WACC, 1y Sharpe from price history, peer_rank from cohort, is_held from portfolio_state.json.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -2794,13 +2794,13 @@
       <c r="M45" s="3" t="inlineStr"/>
       <c r="N45" s="8" t="inlineStr"/>
     </row>
-    <row r="46" ht="75" customHeight="1">
+    <row r="46" ht="60" customHeight="1">
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-TRAFFIC-LIGHT-INPUTS</t>
+          <t>KAIROS-COHORT-SYMPATHY</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
@@ -2810,22 +2810,22 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Detail Lens / Traffic Lights</t>
+          <t>Earnings Lens / Cohort</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Per-ticker risk/fundamentals inputs for lens dots</t>
+          <t>Peer cohort sympathy correlations</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Wire t.f_score · t.altman_z · t.roic · t.wacc · t.sharpe_1y · t.dd_recovery_months · t.peer_rank · t.is_held into build_data.py. _qdComputeLensStatus has cascading fallbacks (PEG → fund_score → F-score; beta → kelly → Sharpe), so dots upgrade automatically as fields land.</t>
+          <t>Wire t.cohort_peers[].er_sympathy_corr + er_sympathy_move_1d + t.sympathy_history in build_data.py. Today: renderEarnings_Sympathy shows scaffold rows from t.cohort_peers if populated, else placeholder.</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Compute in analysis.py / portfolio.py: Piotroski F (existing data), Altman Z (existing data), ROIC vs WACC, 1y Sharpe from price history, peer_rank from cohort, is_held from portfolio_state.json.</t>
+          <t>Compute 8-quarter rolling correlation of 1d post-print move between this name and each cohort peer's ER date. Persist to data.json under t.cohort_peers + t.sympathy_history.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -2840,13 +2840,13 @@
       <c r="M46" s="3" t="inlineStr"/>
       <c r="N46" s="8" t="inlineStr"/>
     </row>
-    <row r="47" ht="60" customHeight="1">
+    <row r="47" ht="75" customHeight="1">
       <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-COHORT-SYMPATHY</t>
+          <t>PARITY-IN-APP-TRADING</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -2856,22 +2856,22 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Earnings Lens / Cohort</t>
+          <t>Execution / Live / Platform Parity</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Peer cohort sympathy correlations</t>
+          <t>In-app Trading (broker-integrated live execution)</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Wire t.cohort_peers[].er_sympathy_corr + er_sympathy_move_1d + t.sympathy_history in build_data.py. Today: renderEarnings_Sympathy shows scaffold rows from t.cohort_peers if populated, else placeholder.</t>
+          <t>One-click BUY/SELL from the dashboard to a live Schwab/Alpaca brokerage account.</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Compute 8-quarter rolling correlation of 1d post-print move between this name and each cohort peer's ER date. Persist to data.json under t.cohort_peers + t.sympathy_history.</t>
+          <t>OAuth-link the Schwab API (already paid stack); surface an 'Execute' button on the Trade Plan card; explicit AUTHORIZE LIVE TRADING gate per CLAUDE.md security protocol; route every order through the existing risk checks (max-loss-pct, drawdown haircut, regime gate).</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>PARITY-IN-APP-TRADING</t>
+          <t>KAIROS-LIVE-D1</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -2902,22 +2902,22 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Execution / Live / Platform Parity</t>
+          <t>Kairos / Audit Ledger</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>In-app Trading (broker-integrated live execution)</t>
+          <t>Live D1 estimate from Schwab quote during RTH</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>One-click BUY/SELL from the dashboard to a live Schwab/Alpaca brokerage account.</t>
+          <t>Replace placeholder D1 (yesterday's close-to-close) with a live Schwab-quote-based intraday estimate during market hours so the audit ledger D1 column is non-stale. Discussed and deferred as semantically muddy (D1 = next-day close, intraday quote is a forecast not a fill).</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>OAuth-link the Schwab API (already paid stack); surface an 'Execute' button on the Trade Plan card; explicit AUTHORIZE LIVE TRADING gate per CLAUDE.md security protocol; route every order through the existing risk checks (max-loss-pct, drawdown haircut, regime gate).</t>
+          <t>Add a SCHWAB_LIVE_D1=1 env flag; when ON and during RTH, compute D1_est = (live_quote - signal_entry) / signal_entry and annotate the cell with an 'est' chip. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -2932,13 +2932,13 @@
       <c r="M48" s="3" t="inlineStr"/>
       <c r="N48" s="8" t="inlineStr"/>
     </row>
-    <row r="49" ht="75" customHeight="1">
+    <row r="49" ht="45" customHeight="1">
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-LIVE-D1</t>
+          <t>KAIROS-SCANNER-BEARS</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -2948,22 +2948,22 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Kairos / Audit Ledger</t>
+          <t>Kairos / Signal Scanner</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Live D1 estimate from Schwab quote during RTH</t>
+          <t>Top 5 Bears panel</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Replace placeholder D1 (yesterday's close-to-close) with a live Schwab-quote-based intraday estimate during market hours so the audit ledger D1 column is non-stale. Discussed and deferred as semantically muddy (D1 = next-day close, intraday quote is a forecast not a fill).</t>
+          <t>Add a 'Top 5 Bears' panel to the Signal Scanner alongside Fresh / Momentum / Earnings / Volume — was proposed but not selected in the initial build.</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Add a SCHWAB_LIVE_D1=1 env flag; when ON and during RTH, compute D1_est = (live_quote - signal_entry) / signal_entry and annotate the cell with an 'est' chip. Effort ~1hr.</t>
+          <t>Mirror existing 4 panels' structure; sort universe by composite bear-score desc; cap at 5; render in the Scanner grid. Effort ~10min.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2978,13 +2978,13 @@
       <c r="M49" s="3" t="inlineStr"/>
       <c r="N49" s="8" t="inlineStr"/>
     </row>
-    <row r="50" ht="45" customHeight="1">
+    <row r="50" ht="60" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-SCANNER-BEARS</t>
+          <t>KAIROS-SCANNER-FLIPS</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -2999,17 +2999,17 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Top 5 Bears panel</t>
+          <t>Today's Flips panel</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Add a 'Top 5 Bears' panel to the Signal Scanner alongside Fresh / Momentum / Earnings / Volume — was proposed but not selected in the initial build.</t>
+          <t>Add a 'Today's Flips' panel to the Signal Scanner — tickers whose verdict flipped vs yesterday (e.g., BUY -&gt; WATCH, WATCH -&gt; BUY, AVOID -&gt; WATCH). Proposed in the 'what else' menu, not selected.</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Mirror existing 4 panels' structure; sort universe by composite bear-score desc; cap at 5; render in the Scanner grid. Effort ~10min.</t>
+          <t>Diff today's bundle.verdict against yesterday.verdict per ticker; surface the 5-10 most material flips. Effort ~30min.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-SCANNER-FLIPS</t>
+          <t>ML-RETRAIN-FINBERT-FEATURE</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -3040,22 +3040,22 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Kairos / Signal Scanner</t>
+          <t>ML / Features (future)</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Today's Flips panel</t>
+          <t>Add FinBERT as a GBM training feature (leak-free)</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Add a 'Today's Flips' panel to the Signal Scanner — tickers whose verdict flipped vs yesterday (e.g., BUY -&gt; WATCH, WATCH -&gt; BUY, AVOID -&gt; WATCH). Proposed in the 'what else' menu, not selected.</t>
+          <t>needs historical sentiment series — accumulate forward via cache/ml/sentiment_log.jsonl (asof-stamped); add as feature #18 + retrain once ~3-6mo of leak-free history exists</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Diff today's bundle.verdict against yesterday.verdict per ticker; surface the 5-10 most material flips. Effort ~30min.</t>
+          <t>ml/feature_extractor + historical backfill</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>ML-RETRAIN-FINBERT-FEATURE</t>
+          <t>ML-AUTOREFRESH-VALIDATE</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -3086,22 +3086,22 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>ML / Features (future)</t>
+          <t>ML / Pipeline (validate)</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Add FinBERT as a GBM training feature (leak-free)</t>
+          <t>Validate ML auto-refresh post-scan + cached-bar reuse</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>needs historical sentiment series — accumulate forward via cache/ml/sentiment_log.jsonl (asof-stamped); add as feature #18 + retrain once ~3-6mo of leak-free history exists</t>
+          <t>ml_edge.run_after_scan=true runs ml.run_ml_edge over the fresh bundle; feature_extractor prefers data_archive (no re-fetch). Confirm end-to-end on next clean scan.</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>ml/feature_extractor + historical backfill</t>
+          <t>swing_trade ML hook + ml/feature_extractor</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>ML-AUTOREFRESH-VALIDATE</t>
+          <t>KAIROS-MACRO-EVENTS</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>ML / Pipeline (validate)</t>
+          <t>Macro Lens / Calendar</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Validate ML auto-refresh post-scan + cached-bar reuse</t>
+          <t>14-day high-impact event window flag</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>ml_edge.run_after_scan=true runs ml.run_ml_edge over the fresh bundle; feature_extractor prefers data_archive (no re-fetch). Confirm end-to-end on next clean scan.</t>
+          <t>Wire t.next_macro_event_days = days to next FOMC/CPI/NFP/jobs. _qdComputeLensStatus reads this and downgrades macro lens to amber when event &lt;= 14d even in risk_on_trending regime.</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>swing_trade ML hook + ml/feature_extractor</t>
+          <t>Add macro_calendar fetch in data_fetcher.py (FRED/Trading Economics free tier or EODHD calendar). Persist to t.next_macro_event_days.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -3162,13 +3162,13 @@
       <c r="M53" s="3" t="inlineStr"/>
       <c r="N53" s="8" t="inlineStr"/>
     </row>
-    <row r="54" ht="60" customHeight="1">
+    <row r="54" ht="45" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-MACRO-EVENTS</t>
+          <t>CACHE-RECLAIM</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -3178,22 +3178,22 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Macro Lens / Calendar</t>
+          <t>Ops / Hygiene</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>14-day high-impact event window flag</t>
+          <t>Reclaim ~6GB cache (stray bak + edgar TTL)</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Wire t.next_macro_event_days = days to next FOMC/CPI/NFP/jobs. _qdComputeLensStatus reads this and downgrades macro lens to amber when event &lt;= 14d even in risk_on_trending regime.</t>
+          <t>delete 300MB last_bundle.json.bak.precap_promote + add edgar companyfacts prune/TTL (6.1GB)</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Add macro_calendar fetch in data_fetcher.py (FRED/Trading Economics free tier or EODHD calendar). Persist to t.next_macro_event_days.</t>
+          <t>cache cleanup + edgar_client TTL</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>CACHE-RECLAIM</t>
+          <t>JOBS-MOMENTUM-SNAPSHOT</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -3224,22 +3224,22 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Ops / Hygiene</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Reclaim ~6GB cache (stray bak + edgar TTL)</t>
+          <t>Decide momentum-snapshot job: load or disable</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>delete 300MB last_bundle.json.bak.precap_promote + add edgar companyfacts prune/TTL (6.1GB)</t>
+          <t>valid plist in repo but not currently loaded; decide launchctl bootstrap vs move to disabled/.</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>cache cleanup + edgar_client TTL</t>
+          <t>infra/launchd/com.swingtrade.momentum-snapshot.plist</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -3254,13 +3254,13 @@
       <c r="M55" s="3" t="inlineStr"/>
       <c r="N55" s="8" t="inlineStr"/>
     </row>
-    <row r="56" ht="45" customHeight="1">
+    <row r="56" ht="60" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>JOBS-MOMENTUM-SNAPSHOT</t>
+          <t>DATA-FUTURE-OPS-TELEMETRY-6</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -3270,22 +3270,22 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Telemetry (future)</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot job: load or disable</t>
+          <t>6 ops telemetry slots — app-side instrumentation</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>valid plist in repo but not currently loaded; decide launchctl bootstrap vs move to disabled/.</t>
+          <t>6 ops telemetry slots remain unbuilt because they require app-side instrumentation: server middleware, git hooks, scan-time emitters, executor probes, sub-tab render timings, fetch-latency probes.</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd/com.swingtrade.momentum-snapshot.plist</t>
+          <t>Build a shared emitter (lib/telemetry.py) writing to a telemetry SQLite; instrument incrementally — server middleware first, then scan emitters; surface in System Status sub-tab.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-OPS-TELEMETRY-6</t>
+          <t>SCALE-4</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -3316,22 +3316,22 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Ops / Telemetry (future)</t>
+          <t>Ops · 500-user</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>6 ops telemetry slots — app-side instrumentation</t>
+          <t>Scan reliability so Home is not sparse</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>6 ops telemetry slots remain unbuilt because they require app-side instrumentation: server middleware, git hooks, scan-time emitters, executor probes, sub-tab render timings, fetch-latency probes.</t>
+          <t>When the daily scan is empty (EODHD quota outage), Home shows honest-empty sections + stale-badged regime; users landing mid-outage see little actionable content</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Build a shared emitter (lib/telemetry.py) writing to a telemetry SQLite; instrument incrementally — server middleware first, then scan emitters; surface in System Status sub-tab.</t>
+          <t>Ensure morning scan runs reliably + quota headroom; keep STALE badge UX; consider serving last-good bundle with clear age</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -3346,13 +3346,13 @@
       <c r="M57" s="3" t="inlineStr"/>
       <c r="N57" s="8" t="inlineStr"/>
     </row>
-    <row r="58" ht="60" customHeight="1">
+    <row r="58" ht="75" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>SCALE-4</t>
+          <t>OV-INVEST-STRUCT</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -3362,22 +3362,22 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Ops · 500-user</t>
+          <t>Overview / Target Engine</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Scan reliability so Home is not sparse</t>
+          <t>Real structural invest targets (kill analyst-PT stub)</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>When the daily scan is empty (EODHD quota outage), Home shows honest-empty sections + stale-badged regime; users landing mid-outage see little actionable content</t>
+          <t>Invest-mode targets fall back to analyst 12mo PT (invest_stub) for low-vol names (e.g. AAPL) when no structural level qualifies in the invest R-band off the wider stop -&gt; near T1, poor R:R. Per-mode stop scaling fix (2026-06-08) made invest coherent for higher-vol names (NVDA stub=False) but low-vol names still stub.</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Ensure morning scan runs reliably + quota headroom; keep STALE badge UX; consider serving last-good bundle with clear age</t>
+          <t>Wire multi-year structural levels (monthly/yearly swing highs, weekly Fib ext) into the invest candidate set so the invest R-band is populated without the analyst-PT fallback; raise invest max_reach_atr to match a 1-5yr horizon.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -3392,13 +3392,13 @@
       <c r="M58" s="3" t="inlineStr"/>
       <c r="N58" s="8" t="inlineStr"/>
     </row>
-    <row r="59" ht="75" customHeight="1">
+    <row r="59" ht="60" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>OV-INVEST-STRUCT</t>
+          <t>SCALE-3</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -3408,22 +3408,22 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Overview / Target Engine</t>
+          <t>Portfolio · 500-user</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Real structural invest targets (kill analyst-PT stub)</t>
+          <t>Per-user portfolio vs shared automated book</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Invest-mode targets fall back to analyst 12mo PT (invest_stub) for low-vol names (e.g. AAPL) when no structural level qualifies in the invest R-band off the wider stop -&gt; near T1, poor R:R. Per-mode stop scaling fix (2026-06-08) made invest coherent for higher-vol names (NVDA stub=False) but low-vol names still stub.</t>
+          <t>Home AUTOMATED BOOK is the single shared Alpaca-paper auto-trade account; every viewer sees identical positions; no per-user book (NAV is per-user, positions are not)</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Wire multi-year structural levels (monthly/yearly swing highs, weekly Fib ext) into the invest candidate set so the invest R-band is populated without the analyst-PT fallback; raise invest max_reach_atr to match a 1-5yr horizon.</t>
+          <t>Decide: keep as shared model/track-record book by design, OR add a per-user position store keyed to UserPrefs auth id</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -3438,13 +3438,13 @@
       <c r="M59" s="3" t="inlineStr"/>
       <c r="N59" s="8" t="inlineStr"/>
     </row>
-    <row r="60" ht="60" customHeight="1">
+    <row r="60" ht="90" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>SCALE-3</t>
+          <t>QUANT-HMM-FF-LGBM-ROADMAP</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -3454,22 +3454,22 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Portfolio · 500-user</t>
+          <t>Quant / Modeling Roadmap</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Per-user portfolio vs shared automated book</t>
+          <t>HMM regime / Fama-French / LightGBM swap (status unclear)</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Home AUTOMATED BOOK is the single shared Alpaca-paper auto-trade account; every viewer sees identical positions; no per-user book (NAV is per-user, positions are not)</t>
+          <t>Roadmap items pasted as a status table — clarification pending whether user wants execution or just context tracking. Three potential upgrades: (a) HMM-based regime classifier replacing the rule-based 4-regime model, (b) Fama-French factor exposure analysis on closed trades, (c) LightGBM swap-in for HistGradientBoosting in ml/train_historical.py. Each 1-3 days.</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>Decide: keep as shared model/track-record book by design, OR add a per-user position store keyed to UserPrefs auth id</t>
+          <t>Confirm intent before executing. If go: HMM first (decouples regime classifier from heuristics, principle #18), then Fama-French attribution (per-strategy factor exposure), then LightGBM swap (likely-marginal accuracy gain vs current HistGB). Each upgrade gated by Wilson-LB validation vs current baseline.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -3484,13 +3484,13 @@
       <c r="M60" s="3" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr"/>
     </row>
-    <row r="61" ht="90" customHeight="1">
+    <row r="61" ht="60" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>QUANT-HMM-FF-LGBM-ROADMAP</t>
+          <t>PARITY-SMART-RISK-LEVELS</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -3500,22 +3500,22 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Quant / Modeling Roadmap</t>
+          <t>Risk / Targets / Platform Parity</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>HMM regime / Fama-French / LightGBM swap (status unclear)</t>
+          <t>Smart Risk Levels (auto stop + T1/T2)</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Roadmap items pasted as a status table — clarification pending whether user wants execution or just context tracking. Three potential upgrades: (a) HMM-based regime classifier replacing the rule-based 4-regime model, (b) Fama-French factor exposure analysis on closed trades, (c) LightGBM swap-in for HistGradientBoosting in ml/train_historical.py. Each 1-3 days.</t>
+          <t>Auto-place stop / T1 / T2 dots on the chart with confluence reasoning (HVN, AVWAP, fractal, ATR, Fib). Already computed by the structural target engine but not surfaced on the new Chart sub-tab.</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Confirm intent before executing. If go: HMM first (decouples regime classifier from heuristics, principle #18), then Fama-French attribution (per-strategy factor exposure), then LightGBM swap (likely-marginal accuracy gain vs current HistGB). Each upgrade gated by Wilson-LB validation vs current baseline.</t>
+          <t>Read cache/target_engine/{TICKER}_{MODE}.json and overlay the levels on the chart canvas with hover tooltips citing the confluence factors; gated by use_structural_targets flag (M2.5 cutover).</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>PARITY-SMART-RISK-LEVELS</t>
+          <t>KAIROS-L2-BOOK</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -3546,22 +3546,22 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Risk / Targets / Platform Parity</t>
+          <t>Risk Lens / Execution</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>Smart Risk Levels (auto stop + T1/T2)</t>
+          <t>L2 bid/ask depth at price levels</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Auto-place stop / T1 / T2 dots on the chart with confluence reasoning (HVN, AVWAP, fractal, ATR, Fib). Already computed by the structural target engine but not surfaced on the new Chart sub-tab.</t>
+          <t>Wire t.l2_book from Schwab streaming API → render in renderRisk_LiquidityLadder. Today: ADV-derived size tiers shown as scaffold. Schwab streaming requires WebSocket session — see schwab_client.py.</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Read cache/target_engine/{TICKER}_{MODE}.json and overlay the levels on the chart canvas with hover tooltips citing the confluence factors; gated by use_structural_targets flag (M2.5 cutover).</t>
+          <t>Subscribe to Schwab Level-II quote stream; persist top-of-book snapshot into t.l2_book = {bid:[{px,size}], ask:[{px,size}]}. Frontend already reads these fields if present.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -3582,7 +3582,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-L2-BOOK</t>
+          <t>PARITY-AI-SIGNALS-V1</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -3592,22 +3592,22 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Risk Lens / Execution</t>
+          <t>Signals / Platform Parity</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>L2 bid/ask depth at price levels</t>
+          <t>1st-Gen AI Signals</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Wire t.l2_book from Schwab streaming API → render in renderRisk_LiquidityLadder. Today: ADV-derived size tiers shown as scaffold. Schwab streaming requires WebSocket session — see schwab_client.py.</t>
+          <t>Surface a baseline AI BUY/SELL signal stream on the chart as quick-glance arrows/dots — the competitor-platform feature (TrendSpider, Trade Ideas) users expect to see at a glance, separate from the full ML Edge sub-tab.</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Subscribe to Schwab Level-II quote stream; persist top-of-book snapshot into t.l2_book = {bid:[{px,size}], ask:[{px,size}]}. Frontend already reads these fields if present.</t>
+          <t>Reuse ML Edge dir-head + cone outputs but render as 1-bar arrows/markers on the new Chart sub-tab; isolate from the 10-section Technicals view; respect cache/ml_edge_predictions.json freshness.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -3622,13 +3622,13 @@
       <c r="M63" s="3" t="inlineStr"/>
       <c r="N63" s="8" t="inlineStr"/>
     </row>
-    <row r="64" ht="60" customHeight="1">
+    <row r="64" ht="45" customHeight="1">
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>PARITY-AI-SIGNALS-V1</t>
+          <t>TEST-AB-PAPER</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -3638,22 +3638,22 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Signals / Platform Parity</t>
+          <t>Testing / Validation (Tier 2)</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>1st-Gen AI Signals</t>
+          <t>A/B Paper Split — live comparison</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Surface a baseline AI BUY/SELL signal stream on the chart as quick-glance arrows/dots — the competitor-platform feature (TrendSpider, Trade Ideas) users expect to see at a glance, separate from the full ML Edge sub-tab.</t>
+          <t>Run config A on half the paper portfolio and config B on the other half; real-time comparison of WR / PF / equity divergence over 30-60d window.</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>Reuse ML Edge dir-head + cone outputs but render as 1-bar arrows/markers on the new Chart sub-tab; isolate from the 10-section Technicals view; respect cache/ml_edge_predictions.json freshness.</t>
+          <t>Extend executor.py to accept --variant flag; persist per-variant portfolio state; cross-section panel in System Status sub-tab. Effort 3-4hr.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -3668,13 +3668,13 @@
       <c r="M64" s="3" t="inlineStr"/>
       <c r="N64" s="8" t="inlineStr"/>
     </row>
-    <row r="65" ht="45" customHeight="1">
+    <row r="65" ht="60" customHeight="1">
       <c r="A65" s="2" t="n">
         <v>64</v>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>TEST-AB-PAPER</t>
+          <t>TEST-BENCHMARK-SPY</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -3689,17 +3689,17 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>A/B Paper Split — live comparison</t>
+          <t>Benchmark vs SPY — alpha / beta / IR</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Run config A on half the paper portfolio and config B on the other half; real-time comparison of WR / PF / equity divergence over 30-60d window.</t>
+          <t>Compute strategy alpha, beta, information ratio vs SPY benchmark. Standard performance attribution; turns 'we made +X%' into 'we made +Y% over SPY at lower drawdown'.</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Extend executor.py to accept --variant flag; persist per-variant portfolio state; cross-section panel in System Status sub-tab. Effort 3-4hr.</t>
+          <t>Daily portfolio_value series joined to SPY adjusted-close; regress daily returns -&gt; SPY returns for beta + alpha; IR = (mean excess return) / (std excess return); render in System Status. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>TEST-BENCHMARK-SPY</t>
+          <t>TEST-DD-DIST</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -3735,17 +3735,17 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Benchmark vs SPY — alpha / beta / IR</t>
+          <t>Drawdown Distribution Simulator</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Compute strategy alpha, beta, information ratio vs SPY benchmark. Standard performance attribution; turns 'we made +X%' into 'we made +Y% over SPY at lower drawdown'.</t>
+          <t>Bootstrap 1000 portfolio paths from closed-trade distribution; measure tail-drawdown probability at p95/p99; supports principle #9 (drawdown asymmetry — losing 50% requires +100% to recover).</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>Daily portfolio_value series joined to SPY adjusted-close; regress daily returns -&gt; SPY returns for beta + alpha; IR = (mean excess return) / (std excess return); render in System Status. Effort ~1hr.</t>
+          <t>Resample trade sequence with replacement; build equity curves; compute max-DD per path; histogram + tail percentiles; feed into position-sizing math. Effort 2-3hr.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>TEST-DD-DIST</t>
+          <t>TEST-SENSITIVITY</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -3781,17 +3781,17 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Drawdown Distribution Simulator</t>
+          <t>Sensitivity / Robustness Test</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Bootstrap 1000 portfolio paths from closed-trade distribution; measure tail-drawdown probability at p95/p99; supports principle #9 (drawdown asymmetry — losing 50% requires +100% to recover).</t>
+          <t>Perturb each config parameter +/-20% (score floors, stop ATR mult, R:R floor, regime thresholds) and check whether the strategy still passes the gate. Finds overfit knobs that only work at one exact value.</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Resample trade sequence with replacement; build equity curves; compute max-DD per path; histogram + tail percentiles; feed into position-sizing math. Effort 2-3hr.</t>
+          <t>Grid-walk key config thresholds; re-run backtest at each point; build sensitivity heatmap (param vs PF); flag any knob whose +/-20% perturbation collapses PF &gt;50%. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>TEST-SENSITIVITY</t>
+          <t>TEST-SLIPPAGE-STRESS</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -3827,17 +3827,17 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Sensitivity / Robustness Test</t>
+          <t>Slippage Stress Test</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Perturb each config parameter +/-20% (score floors, stop ATR mult, R:R floor, regime thresholds) and check whether the strategy still passes the gate. Finds overfit knobs that only work at one exact value.</t>
+          <t>Double the slippage assumption (ATR/ADV-scaled model from audit #5) and recompute backtest stats. Validates fragile execution dependence per principle #19 (slippage realism).</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>Grid-walk key config thresholds; re-run backtest at each point; build sensitivity heatmap (param vs PF); flag any knob whose +/-20% perturbation collapses PF &gt;50%. Effort ~2hr.</t>
+          <t>Re-run backtest with SLIPPAGE_MULT=2.0; compare WR/PF/Sharpe deltas; if a strategy collapses at 2x slippage it is execution-fragile and should be down-sized. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>TEST-SLIPPAGE-STRESS</t>
+          <t>TEST-CORRELATED-FAILURE</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -3868,22 +3868,22 @@
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Testing / Validation (Tier 2)</t>
+          <t>Testing / Validation (Tier 3)</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>Slippage Stress Test</t>
+          <t>Correlated-Failure — what if EODHD goes down 24h?</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Double the slippage assumption (ATR/ADV-scaled model from audit #5) and recompute backtest stats. Validates fragile execution dependence per principle #19 (slippage realism).</t>
+          <t>Simulate the impact of the sole data provider (EODHD) being unavailable for 24-48h during market hours. What happens to (a) the scan, (b) live exec, (c) the dashboard?</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>Re-run backtest with SLIPPAGE_MULT=2.0; compare WR/PF/Sharpe deltas; if a strategy collapses at 2x slippage it is execution-fragile and should be down-sized. Effort ~1hr.</t>
+          <t>Inject EODHD error responses in a paper environment; observe failure modes (fallback to last-known cache vs hard error vs degraded scan); document recovery RTO; tighten any silent-fail paths discovered. Effort 2-3hr.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -3898,13 +3898,13 @@
       <c r="M69" s="3" t="inlineStr"/>
       <c r="N69" s="8" t="inlineStr"/>
     </row>
-    <row r="70" ht="60" customHeight="1">
+    <row r="70" ht="45" customHeight="1">
       <c r="A70" s="2" t="n">
         <v>69</v>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>TEST-CORRELATED-FAILURE</t>
+          <t>TEST-CRASH-REPLAY</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -3919,17 +3919,17 @@
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Correlated-Failure — what if EODHD goes down 24h?</t>
+          <t>Crash Replay — 2008/2020/2022 stress</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Simulate the impact of the sole data provider (EODHD) being unavailable for 24-48h during market hours. What happens to (a) the scan, (b) live exec, (c) the dashboard?</t>
+          <t>Apply current portfolio composition to historical crash days (2008 GFC, 2020 COVID, 2022 rate-shock); measure realized drawdown + recovery time per scenario.</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>Inject EODHD error responses in a paper environment; observe failure modes (fallback to last-known cache vs hard error vs degraded scan); document recovery RTO; tighten any silent-fail paths discovered. Effort 2-3hr.</t>
+          <t>Snapshot today's positions; price-replay against historical daily OHLC from those windows; report per-crisis max-DD and time-to-recovery. Effort 2-3hr.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -3944,13 +3944,13 @@
       <c r="M70" s="3" t="inlineStr"/>
       <c r="N70" s="8" t="inlineStr"/>
     </row>
-    <row r="71" ht="45" customHeight="1">
+    <row r="71" ht="60" customHeight="1">
       <c r="A71" s="2" t="n">
         <v>70</v>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>TEST-CRASH-REPLAY</t>
+          <t>TEST-KELLY-SIM</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -3965,17 +3965,17 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Crash Replay — 2008/2020/2022 stress</t>
+          <t>Half-Kelly vs Full-Kelly sizing simulation</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Apply current portfolio composition to historical crash days (2008 GFC, 2020 COVID, 2022 rate-shock); measure realized drawdown + recovery time per scenario.</t>
+          <t>Visualize portfolio growth under Half-Kelly (current default) vs Full-Kelly vs Quarter-Kelly sizing rules; quantifies the volatility-vs-CAGR tradeoff that principle #9 codifies.</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>Snapshot today's positions; price-replay against historical daily OHLC from those windows; report per-crisis max-DD and time-to-recovery. Effort 2-3hr.</t>
+          <t>Bootstrap N portfolio paths under each Kelly fraction; chart median equity curve + percentile fans; surface terminal-wealth distribution. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>TEST-KELLY-SIM</t>
+          <t>TEST-SLIPPAGE-ATTR</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -4011,17 +4011,17 @@
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Half-Kelly vs Full-Kelly sizing simulation</t>
+          <t>Slippage Attribution — signal PnL vs realized PnL gap</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Visualize portfolio growth under Half-Kelly (current default) vs Full-Kelly vs Quarter-Kelly sizing rules; quantifies the volatility-vs-CAGR tradeoff that principle #9 codifies.</t>
+          <t>For each closed trade, compute the gap between the model's predicted entry/exit and the actual fill price. Aggregate by setup/ticker/regime to find where slippage eats edge.</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>Bootstrap N portfolio paths under each Kelly fraction; chart median equity curve + percentile fans; surface terminal-wealth distribution. Effort ~2hr.</t>
+          <t>Read signal_log entries (which has the signal price) and join to paper_fills.json (which has the realized price); compute slippage_bp per trade; group + percentile. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>TEST-SLIPPAGE-ATTR</t>
+          <t>TEST-TAX-AWARE</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -4057,17 +4057,17 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Slippage Attribution — signal PnL vs realized PnL gap</t>
+          <t>Tax-Aware Backtest — short-term cap-gains haircut</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>For each closed trade, compute the gap between the model's predicted entry/exit and the actual fill price. Aggregate by setup/ticker/regime to find where slippage eats edge.</t>
+          <t>Apply short-term capital-gains tax (35-40% on gains held &lt;1yr) to backtest PnL. Real after-tax return for a US retail account is materially lower than gross.</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>Read signal_log entries (which has the signal price) and join to paper_fills.json (which has the realized price); compute slippage_bp per trade; group + percentile. Effort ~2hr.</t>
+          <t>Add post_tax_pnl column to backtest output; apply 35% haircut to short-term gains (&gt;0 PnL, held &lt;365d) and 15% to long-term; report Sharpe / total-return pre vs post tax. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>TEST-TAX-AWARE</t>
+          <t>WAIT-CALIB-DRIFT-SPARK</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -4098,22 +4098,22 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Testing / Validation (Tier 3)</t>
+          <t>Time-Dependent / Calibration</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Tax-Aware Backtest — short-term cap-gains haircut</t>
+          <t>Calibration drift sparkline populates</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Apply short-term capital-gains tax (35-40% on gains held &lt;1yr) to backtest PnL. Real after-tax return for a US retail account is materially lower than gross.</t>
+          <t>The calibration-drift sparkline in the ML Edge sub-tab needs multiple training cycles to populate (weeks). Each morning scan retrains and appends a calibration row; the sparkline reads from that history table.</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Add post_tax_pnl column to backtest output; apply 35% haircut to short-term gains (&gt;0 PnL, held &lt;365d) and 15% to long-term; report Sharpe / total-return pre vs post tax. Effort ~2hr.</t>
+          <t>Passive wait. Re-check after 4-6 weekly retrain cycles. If still empty, verify ml.train_historical writes to cache/ml/calibration_history.jsonl on each run.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -4128,13 +4128,13 @@
       <c r="M74" s="3" t="inlineStr"/>
       <c r="N74" s="8" t="inlineStr"/>
     </row>
-    <row r="75" ht="60" customHeight="1">
+    <row r="75" ht="45" customHeight="1">
       <c r="A75" s="2" t="n">
         <v>74</v>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>WAIT-CALIB-DRIFT-SPARK</t>
+          <t>WAIT-DRIFT-SNAPSHOTS</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -4144,22 +4144,22 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Calibration</t>
+          <t>Time-Dependent / Drift Tracking</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Calibration drift sparkline populates</t>
+          <t>Diff vs yesterday + 30-day drift populate</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>The calibration-drift sparkline in the ML Edge sub-tab needs multiple training cycles to populate (weeks). Each morning scan retrains and appends a calibration row; the sparkline reads from that history table.</t>
+          <t>The 'diff vs yesterday' + 30-day drift columns need 2+ daily snapshots stored. Starts populating tomorrow's scan.</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>Passive wait. Re-check after 4-6 weekly retrain cycles. If still empty, verify ml.train_historical writes to cache/ml/calibration_history.jsonl on each run.</t>
+          <t>Passive wait; first populated values appear in the next morning's scan output. Verify the snapshot persister wrote a row today.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>WAIT-DRIFT-SNAPSHOTS</t>
+          <t>WAIT-ML-PICKS-RESOLVE</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -4190,22 +4190,22 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Drift Tracking</t>
+          <t>Time-Dependent / Picks History</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Diff vs yesterday + 30-day drift populate</t>
+          <t>Picks-history outcome resolution (resolve_ml_picks.py)</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>The 'diff vs yesterday' + 30-day drift columns need 2+ daily snapshots stored. Starts populating tomorrow's scan.</t>
+          <t>resolve_ml_picks.py needs 5 trading days from each pick to resolve outcomes. First AI Edge batch (picks from ~2026-05-18) resolves around 2026-05-23.</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>Passive wait; first populated values appear in the next morning's scan output. Verify the snapshot persister wrote a row today.</t>
+          <t>Passive wait. Re-check on 2026-05-23; verify resolve_ml_picks.py runs in run_daily_scan.sh and populates picks_history.json outcome columns.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -4220,13 +4220,13 @@
       <c r="M76" s="3" t="inlineStr"/>
       <c r="N76" s="8" t="inlineStr"/>
     </row>
-    <row r="77" ht="45" customHeight="1">
+    <row r="77" ht="60" customHeight="1">
       <c r="A77" s="2" t="n">
         <v>76</v>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>WAIT-ML-PICKS-RESOLVE</t>
+          <t>WAIT-SURVIVORSHIP-DECAY</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -4236,22 +4236,22 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Picks History</t>
+          <t>Time-Dependent / Survivorship Haircut</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Picks-history outcome resolution (resolve_ml_picks.py)</t>
+          <t>Survivorship haircut shrinking 3pp -&gt; 0.5pp</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>resolve_ml_picks.py needs 5 trading days from each pick to resolve outcomes. First AI Edge batch (picks from ~2026-05-18) resolves around 2026-05-23.</t>
+          <t>The -3pp WR survivorship haircut should shrink as monthly S&amp;P 500 / R1000 membership snapshots accumulate (Wikipedia revision history). Once 24+ months of snapshots are stored, the haircut can fade toward 0.5pp.</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>Passive wait. Re-check on 2026-05-23; verify resolve_ml_picks.py runs in run_daily_scan.sh and populates picks_history.json outcome columns.</t>
+          <t>Passive wait — currently only current-membership data. Re-evaluate annually. Until then keep -3pp haircut per CLAUDE.md principle #6.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>WAIT-SURVIVORSHIP-DECAY</t>
+          <t>WAIT-WF-EQUITY-REAL</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -4282,22 +4282,22 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Survivorship Haircut</t>
+          <t>Time-Dependent / Walk-Forward</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Survivorship haircut shrinking 3pp -&gt; 0.5pp</t>
+          <t>Walk-forward equity curve switches to REAL track</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>The -3pp WR survivorship haircut should shrink as monthly S&amp;P 500 / R1000 membership snapshots accumulate (Wikipedia revision history). Once 24+ months of snapshots are stored, the haircut can fade toward 0.5pp.</t>
+          <t>Currently the equity curve renders backtest-derived returns. Switches to REAL track once 5+ resolved AI Edge picks are available — first batch resolves ~2026-05-23, so REAL curve activates ~2026-05-24.</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>Passive wait — currently only current-membership data. Re-evaluate annually. Until then keep -3pp haircut per CLAUDE.md principle #6.</t>
+          <t>Passive wait. Re-check on 2026-05-24; verify the equity curve flips from BACKTEST badge to REAL badge once n_resolved &gt;= 5.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>WAIT-WF-EQUITY-REAL</t>
+          <t>PARITY-10-CHARTS-GRID</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -4328,22 +4328,22 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Walk-Forward</t>
+          <t>UI / Layout / Platform Parity</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Walk-forward equity curve switches to REAL track</t>
+          <t>10-chart multi-pane grid</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Currently the equity curve renders backtest-derived returns. Switches to REAL track once 5+ resolved AI Edge picks are available — first batch resolves ~2026-05-23, so REAL curve activates ~2026-05-24.</t>
+          <t>Display up to 10 ticker charts side-by-side in a configurable grid (2x5, 3x4, etc.) for at-a-glance correlation/leadership reads — what TrendSpider and Trade Ideas users default to.</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>Passive wait. Re-check on 2026-05-24; verify the equity curve flips from BACKTEST badge to REAL badge once n_resolved &gt;= 5.</t>
+          <t>New 'Grid' workspace in kairos that renders N lightweight-chart canvases; ticker list drag-droppable; persists ticker set per layout.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>PARITY-10-CHARTS-GRID</t>
+          <t>PARITY-CUSTOM-LAYOUTS</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -4379,17 +4379,17 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>10-chart multi-pane grid</t>
+          <t>Customizable Layouts (save/load workspace presets)</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Display up to 10 ticker charts side-by-side in a configurable grid (2x5, 3x4, etc.) for at-a-glance correlation/leadership reads — what TrendSpider and Trade Ideas users default to.</t>
+          <t>User drags/resizes panels in the kairos workspace and saves the arrangement as a named preset (Day-Trade view / Swing view / Research view) and switches between them.</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>New 'Grid' workspace in kairos that renders N lightweight-chart canvases; ticker list drag-droppable; persists ticker set per layout.</t>
+          <t>Persist layout JSON in cache/user_layouts.json (per-user once auth lands); sidebar dropdown to switch; default presets shipped (Swing / Position / Research).</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -4404,13 +4404,13 @@
       <c r="M80" s="3" t="inlineStr"/>
       <c r="N80" s="8" t="inlineStr"/>
     </row>
-    <row r="81" ht="60" customHeight="1">
+    <row r="81" ht="75" customHeight="1">
       <c r="A81" s="2" t="n">
         <v>80</v>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>PARITY-CUSTOM-LAYOUTS</t>
+          <t>STRUCT-TARGETS-PHASE2</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -4420,35 +4420,51 @@
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>UI / Layout / Platform Parity</t>
+          <t>Strategy / Targets</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Customizable Layouts (save/load workspace presets)</t>
+          <t>Structural targets Phase 2 — engine uses them as T1/T2</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>User drags/resizes panels in the kairos workspace and saves the arrangement as a named preset (Day-Trade view / Swing view / Research view) and switches between them.</t>
+          <t>Phase 1 (shipped 2026-05-10): structural target sources (fractal, fib, EW Wave-3) display on Plan tab as informational. Phase 2: actually use these as T1/T2 instead of ATR-multiple targets. Needs per-source x regime evidence (&gt;=30 trades each).</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Persist layout JSON in cache/user_layouts.json (per-user once auth lands); sidebar dropdown to switch; default presets shipped (Swing / Position / Research).</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr"/>
-      <c r="I81" s="5" t="inlineStr"/>
-      <c r="J81" s="5" t="inlineStr"/>
-      <c r="K81" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>Add config flag target_source = atr_multiple | structural. When structural, T1 = nearest_above with R:R&gt;=3 from {fractal_high, fib_127, EW_T1}. Fall back to ATR if R:R floor not met. Backtest side-by-side with current ATR-multiple.</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>1 day + backtest</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>High win potential, medium risk</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>Awaiting evidence. Phase 1 currently just populates display field; need 3-4 weeks of trade data with target_sources captured before Phase 2 is decidable.</t>
+        </is>
+      </c>
+      <c r="K81" s="11" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="3" t="inlineStr"/>
-      <c r="N81" s="8" t="inlineStr"/>
+      <c r="N81" s="8" t="inlineStr">
+        <is>
+          <t>Run backtest with target_source=structural and target_source=atr_multiple on same window. Compare PF/WR/avg_win.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="2" t="n">
@@ -4456,69 +4472,77 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>STRUCT-TARGETS-PHASE2</t>
-        </is>
-      </c>
-      <c r="C82" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Targets</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Structural targets Phase 2 — engine uses them as T1/T2</t>
+          <t>Single canonical trade plan object — every tab reads from one source</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (shipped 2026-05-10): structural target sources (fractal, fib, EW Wave-3) display on Plan tab as informational. Phase 2: actually use these as T1/T2 instead of ATR-multiple targets. Needs per-source x regime evidence (&gt;=30 trades each).</t>
+          <t>Different dashboard tabs (Plan, Overview, Technicals, Models) computed their own derived values from raw signal data — drift risk, inconsistent UI numbers.</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>Add config flag target_source = atr_multiple | structural. When structural, T1 = nearest_above with R:R&gt;=3 from {fractal_high, fib_127, EW_T1}. Fall back to ATR if R:R floor not met. Backtest side-by-side with current ATR-multiple.</t>
+          <t>New canonical_trade_plan.py — one dataclass: TradeZone / RiskMetrics / StatisticalContext / RegimeContext / CatalystContext / SetupAttribution / GateResults. swing_trade.py attaches it per signal. Live Wilson-CI lookup from signal_log per setup×regime. Mechanism hypothesis per setup family.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>1 day + backtest</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>High win potential, medium risk</t>
+          <t>Win: tabs converge on one truth; future tabs bind to dataclass fields.</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>Awaiting evidence. Phase 1 currently just populates display field; need 3-4 weeks of trade data with target_sources captured before Phase 2 is decidable.</t>
-        </is>
-      </c>
-      <c r="K82" s="11" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr"/>
-      <c r="M82" s="3" t="inlineStr"/>
+          <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
+        </is>
+      </c>
+      <c r="K82" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>2c9b9f339</t>
+        </is>
+      </c>
       <c r="N82" s="8" t="inlineStr">
         <is>
-          <t>Run backtest with target_source=structural and target_source=atr_multiple on same window. Compare PF/WR/avg_win.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="75" customHeight="1">
+          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="90" customHeight="1">
       <c r="A83" s="2" t="n">
         <v>82</v>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>B3-WEEKLY-FIX</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4528,37 +4552,29 @@
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>Backtest / Bug Fix</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Single canonical trade plan object — every tab reads from one source</t>
+          <t>Backtest must build weekly_df from daily for weekly_bull computation</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Different dashboard tabs (Plan, Overview, Technicals, Models) computed their own derived values from raw signal data — drift risk, inconsistent UI numbers.</t>
+          <t>Backtest harness was passing only the daily df to the engine, but weekly_bull (a hard gate in trend-continuation setups) requires resampled weekly bars. Without it, every backtest signal fell through the weekly_bull gate as 'unknown' which the engine treated as fail. Effective on-paper effect: 0 BUYs across many backtests despite valid signals in the daily series.</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>New canonical_trade_plan.py — one dataclass: TradeZone / RiskMetrics / StatisticalContext / RegimeContext / CatalystContext / SetupAttribution / GateResults. swing_trade.py attaches it per signal. Live Wilson-CI lookup from signal_log per setup×regime. Mechanism hypothesis per setup family.</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I83" s="5" t="inlineStr">
-        <is>
-          <t>Win: tabs converge on one truth; future tabs bind to dataclass fields.</t>
-        </is>
-      </c>
+          <t>Build weekly_df via df.resample('W').agg({open: first, high: max, low: min, close: last, volume: sum}) before each pre-trade-gate call. Pass alongside daily.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="5" t="inlineStr"/>
       <c r="J83" s="5" t="inlineStr">
         <is>
-          <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
+          <t>P0 because this silently invalidated every Trend-Continuation backtest signal in the 750d simulations Saturday. Found during Q1-step5 0-BUY investigation — daily df alone made the engine think every TC signal failed weekly_bull as "unknown".</t>
         </is>
       </c>
       <c r="K83" s="12" t="inlineStr">
@@ -4568,27 +4584,27 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t>2c9b9f339</t>
+          <t>985cd182b</t>
         </is>
       </c>
       <c r="N83" s="8" t="inlineStr">
         <is>
-          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="90" customHeight="1">
+          <t>1. python3 backtest.py --window 250d --min-score 65 → confirm BUYs &gt; 0. 2. Compare cache/portfolio_backtest_250d_min65_h5_20260510_*.json before/after fix → expected: pre-fix had 0 trades on Trend-Continuation family; post-fix has them. 3. grep -E "weekly_df|weekly_bull" backtest.py to verify the resample call is in the inner loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="75" customHeight="1">
       <c r="A84" s="2" t="n">
         <v>83</v>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>B3-WEEKLY-FIX</t>
+          <t>VARIANT-F-BT</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4598,31 +4614,27 @@
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Backtest / Bug Fix</t>
+          <t>Backtest Parity</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>Backtest must build weekly_df from daily for weekly_bull computation</t>
+          <t>Variant F regime-conditional multipliers not wired into backtest path</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>Backtest harness was passing only the daily df to the engine, but weekly_bull (a hard gate in trend-continuation setups) requires resampled weekly bars. Without it, every backtest signal fell through the weekly_bull gate as 'unknown' which the engine treated as fail. Effective on-paper effect: 0 BUYs across many backtests despite valid signals in the daily series.</t>
+          <t>backtest.py:418 uses tracker.get_setup_weight_multiplier (reading picks_history) but never consults config.setup_score_multiplier_by_regime. So Variant F's TC×bull=0.0 kill never applied in backtest — explains why 105 TC bull trades persisted in 250d backtest despite live kill in config.</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>Build weekly_df via df.resample('W').agg({open: first, high: max, low: min, close: last, volume: sum}) before each pre-trade-gate call. Pass alongside daily.</t>
+          <t>Add Variant F lookup at backtest.py:442 mirroring analysis.py:8867 logic. Same demotion gate (n&gt;=30 + wr_lb&lt;0.30). Comment cross-reference live path.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="5" t="inlineStr"/>
-      <c r="J84" s="5" t="inlineStr">
-        <is>
-          <t>P0 because this silently invalidated every Trend-Continuation backtest signal in the 750d simulations Saturday. Found during Q1-step5 0-BUY investigation — daily df alone made the engine think every TC signal failed weekly_bull as "unknown".</t>
-        </is>
-      </c>
+      <c r="J84" s="5" t="inlineStr"/>
       <c r="K84" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4635,22 +4647,18 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>985cd182b</t>
-        </is>
-      </c>
-      <c r="N84" s="8" t="inlineStr">
-        <is>
-          <t>1. python3 backtest.py --window 250d --min-score 65 → confirm BUYs &gt; 0. 2. Compare cache/portfolio_backtest_250d_min65_h5_20260510_*.json before/after fix → expected: pre-fix had 0 trades on Trend-Continuation family; post-fix has them. 3. grep -E "weekly_df|weekly_bull" backtest.py to verify the resample call is in the inner loop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="75" customHeight="1">
+          <t>0cdb13340</t>
+        </is>
+      </c>
+      <c r="N84" s="8" t="inlineStr"/>
+    </row>
+    <row r="85" ht="45" customHeight="1">
       <c r="A85" s="2" t="n">
         <v>84</v>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>VARIANT-F-BT</t>
+          <t>P0-WEEKLY</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -4660,27 +4668,39 @@
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Backtest Parity</t>
+          <t>Backtest infra</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Variant F regime-conditional multipliers not wired into backtest path</t>
+          <t>Backtest must build weekly_df from daily (0-BUYs root cause)</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>backtest.py:418 uses tracker.get_setup_weight_multiplier (reading picks_history) but never consults config.setup_score_multiplier_by_regime. So Variant F's TC×bull=0.0 kill never applied in backtest — explains why 105 TC bull trades persisted in 250d backtest despite live kill in config.</t>
+          <t>GATE-1 produced 0 BUYs because backtest _score_as_of did not pass weekly_df. _weekly_ema_alignment(None) returned bullish=False; setup_gates demoted every BUY.</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Add Variant F lookup at backtest.py:442 mirroring analysis.py:8867 logic. Same demotion gate (n&gt;=30 + wr_lb&lt;0.30). Comment cross-reference live path.</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr"/>
-      <c r="I85" s="5" t="inlineStr"/>
-      <c r="J85" s="5" t="inlineStr"/>
+          <t>Resample daily OHLCV to W-FRI inside _score_as_of. Pass weekly_df to score_technicals. Leakage-free.</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>CRITICAL — system was unable to backtest</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>Validated: --smoke produced 5 BUYs in 5d, PF 7.74.</t>
+        </is>
+      </c>
       <c r="K85" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4693,18 +4713,22 @@
       </c>
       <c r="M85" s="3" t="inlineStr">
         <is>
-          <t>0cdb13340</t>
-        </is>
-      </c>
-      <c r="N85" s="8" t="inlineStr"/>
-    </row>
-    <row r="86" ht="45" customHeight="1">
+          <t>985cd182b</t>
+        </is>
+      </c>
+      <c r="N85" s="8" t="inlineStr">
+        <is>
+          <t>python3 backtest.py --smoke - cache/portfolio_backtest.json total_trades &gt; 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="75" customHeight="1">
       <c r="A86" s="2" t="n">
         <v>85</v>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>P0-WEEKLY</t>
+          <t>ROLLING-SHARPE-FIX</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -4714,39 +4738,27 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Backtest infra</t>
+          <t>Decision Engine / Bug</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>Backtest must build weekly_df from daily (0-BUYs root cause)</t>
+          <t>Rolling-Sharpe brake firing on contaminated data</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>GATE-1 produced 0 BUYs because backtest _score_as_of did not pass weekly_df. _weekly_ema_alignment(None) returned bullish=False; setup_gates demoted every BUY.</t>
+          <t>Two bugs: (a) WATCH-conviction signals being written with verdict='BUY' inflated loss count; (b) same physical trade re-emitted as fresh daily signal counted 3× in rolling-20 window. Net: false brake activation pausing ALL new BUYs system-wide. Real Sharpe -0.42; system reported -1.732</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Resample daily OHLCV to W-FRI inside _score_as_of. Pass weekly_df to score_technicals. Leakage-free.</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
-        <is>
-          <t>20 min</t>
-        </is>
-      </c>
-      <c r="I86" s="5" t="inlineStr">
-        <is>
-          <t>CRITICAL — system was unable to backtest</t>
-        </is>
-      </c>
-      <c r="J86" s="5" t="inlineStr">
-        <is>
-          <t>Validated: --smoke produced 5 BUYs in 5d, PF 7.74.</t>
-        </is>
-      </c>
+          <t>Upstream fix: swing_trade.py line 3110 _resolve_verdict() detects WATCH conviction and overrides bucket label. Read-time fix: decision_engine.compute_rolling_sharpe_kill_state dedupes by (ticker,entry,pnl,exit_reason). Historical cleanup: scripts/dedupe_signal_log.py removed 133 mislabels + 90 dupes (backed up)</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="5" t="inlineStr"/>
+      <c r="J86" s="5" t="inlineStr"/>
       <c r="K86" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4754,27 +4766,23 @@
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>985cd182b</t>
-        </is>
-      </c>
-      <c r="N86" s="8" t="inlineStr">
-        <is>
-          <t>python3 backtest.py --smoke - cache/portfolio_backtest.json total_trades &gt; 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="75" customHeight="1">
+          <t>27fd646b1</t>
+        </is>
+      </c>
+      <c r="N86" s="8" t="inlineStr"/>
+    </row>
+    <row r="87" ht="90" customHeight="1">
       <c r="A87" s="2" t="n">
         <v>86</v>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>ROLLING-SHARPE-FIX</t>
+          <t>OPERATING-MINDSET</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4784,27 +4792,39 @@
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine / Bug</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>Rolling-Sharpe brake firing on contaminated data</t>
+          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Two bugs: (a) WATCH-conviction signals being written with verdict='BUY' inflated loss count; (b) same physical trade re-emitted as fresh daily signal counted 3× in rolling-20 window. Net: false brake activation pausing ALL new BUYs system-wide. Real Sharpe -0.42; system reported -1.732</t>
+          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>Upstream fix: swing_trade.py line 3110 _resolve_verdict() detects WATCH conviction and overrides bucket label. Read-time fix: decision_engine.compute_rolling_sharpe_kill_state dedupes by (ticker,entry,pnl,exit_reason). Historical cleanup: scripts/dedupe_signal_log.py removed 133 mislabels + 90 dupes (backed up)</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr"/>
-      <c r="I87" s="5" t="inlineStr"/>
-      <c r="J87" s="5" t="inlineStr"/>
+          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>Win: codified discipline survives session/agent boundaries.</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
+        </is>
+      </c>
       <c r="K87" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4812,23 +4832,27 @@
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N87" s="8" t="inlineStr"/>
-    </row>
-    <row r="88" ht="90" customHeight="1">
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N87" s="8" t="inlineStr">
+        <is>
+          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="60" customHeight="1">
       <c r="A88" s="2" t="n">
         <v>87</v>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>OPERATING-MINDSET</t>
+          <t>EXEC-TRADABLE-ENUM</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4838,39 +4862,27 @@
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Execution · Auto-Trade</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
+          <t>Stock executor skipped all active names (enum bug)</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
+          <t>alpaca-py AssetStatus enum stringified to 'AssetStatus.ACTIVE'; check 'assetstatus.active' != 'active' wrongly skipped EVERY tradable stock since ~2026-05-28 → stock auto-trade silently dead, options-only</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I88" s="5" t="inlineStr">
-        <is>
-          <t>Win: codified discipline survives session/agent boundaries.</t>
-        </is>
-      </c>
-      <c r="J88" s="5" t="inlineStr">
-        <is>
-          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
-        </is>
-      </c>
+          <t>executor.py: read enum .value ('active') before lowercasing</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="5" t="inlineStr"/>
+      <c r="J88" s="5" t="inlineStr"/>
       <c r="K88" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4878,27 +4890,23 @@
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="N88" s="8" t="inlineStr">
-        <is>
-          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="60" customHeight="1">
+          <t>c7098178a</t>
+        </is>
+      </c>
+      <c r="N88" s="8" t="inlineStr"/>
+    </row>
+    <row r="89" ht="105" customHeight="1">
       <c r="A89" s="2" t="n">
         <v>88</v>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>EXEC-TRADABLE-ENUM</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4908,27 +4916,39 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Execution · Auto-Trade</t>
+          <t>ML / Data Logging</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Stock executor skipped all active names (enum bug)</t>
+          <t>Entry-time feature logger in swing_trade.py</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>alpaca-py AssetStatus enum stringified to 'AssetStatus.ACTIVE'; check 'assetstatus.active' != 'active' wrongly skipped EVERY tradable stock since ~2026-05-28 → stock auto-trade silently dead, options-only</t>
+          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>executor.py: read enum .value ('active') before lowercasing</t>
-        </is>
-      </c>
-      <c r="H89" s="2" t="inlineStr"/>
-      <c r="I89" s="5" t="inlineStr"/>
-      <c r="J89" s="5" t="inlineStr"/>
+          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
+        </is>
+      </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
+        </is>
+      </c>
       <c r="K89" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4936,15 +4956,19 @@
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr">
         <is>
-          <t>c7098178a</t>
-        </is>
-      </c>
-      <c r="N89" s="8" t="inlineStr"/>
+          <t>0574c60d4</t>
+        </is>
+      </c>
+      <c r="N89" s="8" t="inlineStr">
+        <is>
+          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="105" customHeight="1">
       <c r="A90" s="2" t="n">
@@ -4952,7 +4976,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>ML-FEATURE-MISMATCH</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4962,39 +4986,27 @@
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>ML / Data Logging</t>
+          <t>ML · Inference</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Entry-time feature logger in swing_trade.py</t>
+          <t>Live predict_one degenerate — 29-feat model vs 17-feat extractor</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
+          <t>Models retrained 2026-06-09 on 29 features but ml.feature_extractor.FEATURE_COLS still emits 17, so live predict_one feeds a mismatched vector and returns ~0 p_up for EVERY ticker (AI Edge 0% bug, all names). Batch ml-predict path extracts 29 correctly. /api/ml now prefers the batch cache + rejects degenerate live; ROOT FIX still needed: align FEATURE_COLS to 29 (or guard retrain to the live feature set). Also cache 4d stale.</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I90" s="5" t="inlineStr">
-        <is>
-          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
-        </is>
-      </c>
-      <c r="J90" s="5" t="inlineStr">
-        <is>
-          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
-        </is>
-      </c>
+          <t>server /api/ml cache-first + degenerate guard (done); align ml/feature_extractor.FEATURE_COLS to model n_features_in_ (pending)</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="5" t="inlineStr"/>
+      <c r="J90" s="5" t="inlineStr"/>
       <c r="K90" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -5002,19 +5014,15 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr">
         <is>
-          <t>0574c60d4</t>
-        </is>
-      </c>
-      <c r="N90" s="8" t="inlineStr">
-        <is>
-          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
-        </is>
-      </c>
+          <t>33877186c</t>
+        </is>
+      </c>
+      <c r="N90" s="8" t="inlineStr"/>
     </row>
     <row r="91" ht="45" customHeight="1">
       <c r="A91" s="2" t="n">
@@ -15715,7 +15723,7 @@
         </is>
       </c>
       <c r="B2" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="18" t="n">
         <v>20</v>
@@ -15724,7 +15732,7 @@
         <v>58</v>
       </c>
       <c r="E2" s="18" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -15753,7 +15761,7 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>77</v>
@@ -15762,7 +15770,7 @@
         <v>68</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
FIX: scan-column ranks every surface by score DESC (align with signal scanner)
The MAP surface sorted by |%change| (top movers) and BULLISH/ELITE didn't
re-sort at all, so the 01–N rank didn't match the score column (the scanner's
sort key). Now all four surfaces (MAP/BULLISH/WATCH/ELITE) sort by score
descending via a shared null-safe comparator (_byScoreDesc — null/non-finite
scores sink to the bottom). MAP still draws from the top-mover universe but
ranks it by score. Rebuilt BullVeda.html.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-06-09.xlsx
+++ b/cache/open_items_2026-06-09.xlsx
@@ -706,13 +706,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="105" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>STRUCT-TARGETS-M25-CUTOVER</t>
+          <t>ML-FEATURE-MISMATCH</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -722,22 +722,22 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Targets</t>
+          <t>ML · Inference</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Structural targets · M2.5 — cutover gate (flip use_structural_targets=true)</t>
+          <t>Live predict_one degenerate — 29-feat model vs 17-feat extractor</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Pending. After M2.1-2.4 settle in production (one week of nightly precompute + dashboard observation with flag=false), flip use_structural_targets=true in config/config.json so build_data.py overlays structural fields into data.json. Frontend consumers (Plan tab, candidate ladder, target behavior) start picking up t1_structural/t2_structural in parallel with legacy t1/t2.</t>
+          <t>Models retrained 2026-06-09 on 29 features but ml.feature_extractor.FEATURE_COLS still emits 17, so live predict_one feeds a mismatched vector and returns ~0 p_up for EVERY ticker (AI Edge 0% bug, all names). Batch ml-predict path extracts 29 correctly. /api/ml now prefers the batch cache + rejects degenerate live; ROOT FIX still needed: align FEATURE_COLS to 29 (or guard retrain to the live feature set). Also cache 4d stale.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Cutover requires: (1) one week of clean nightly precompute (no &gt;10 percent failure rate per scripts/precompute_targets.py exit code), (2) one clean te_regression run with errors &lt;= 1, (3) v2 dashboard frontend updated to read t1_structural fields when present (still falls back to t1 legacy when not). Until all three pass, leave flag=false.</t>
+          <t>server /api/ml cache-first + degenerate guard (done); align ml/feature_extractor.FEATURE_COLS to model n_features_in_ (pending)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -752,38 +752,38 @@
       <c r="M2" s="3" t="inlineStr"/>
       <c r="N2" s="8" t="inlineStr"/>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>SCALE-2</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>STRUCT-TARGETS-M25-CUTOVER</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Auth · 500-user</t>
+          <t>Strategy / Targets</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Enforce per-user Supabase login (not shared basic-auth)</t>
+          <t>Structural targets · M2.5 — cutover gate (flip use_structural_targets=true)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Per-user UserPrefs isolation (NAV/plans/watchlist) only holds when users authenticate via Supabase; if they share the single basic-auth (gari/Swing2026), UserPrefs falls back to per-browser localStorage = no true per-user separation</t>
+          <t>Pending. After M2.1-2.4 settle in production (one week of nightly precompute + dashboard observation with flag=false), flip use_structural_targets=true in config/config.json so build_data.py overlays structural fields into data.json. Frontend consumers (Plan tab, candidate ladder, target behavior) start picking up t1_structural/t2_structural in parallel with legacy t1/t2.</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Require Supabase login for multi-user; verify UserPrefs keys per auth id end-to-end (user-prefs.jsx setUser binds sb.auth.getUser)</t>
+          <t>Cutover requires: (1) one week of clean nightly precompute (no &gt;10 percent failure rate per scripts/precompute_targets.py exit code), (2) one clean te_regression run with errors &lt;= 1, (3) v2 dashboard frontend updated to read t1_structural fields when present (still falls back to t1 legacy when not). Until all three pass, leave flag=false.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -798,13 +798,13 @@
       <c r="M3" s="3" t="inlineStr"/>
       <c r="N3" s="8" t="inlineStr"/>
     </row>
-    <row r="4" ht="75" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>BUG-WEEKEND-PHANTOM-PICKS</t>
+          <t>SCALE-2</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -814,22 +814,22 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Bugs / Audit Ledger</t>
+          <t>Auth · 500-user</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Weekend phantom picks in audit ledger</t>
+          <t>Enforce per-user Supabase login (not shared basic-auth)</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Audit ledger shows phantom picks on May 10 (Sun), May 16 (Sat), May 17 (Sun) — markets closed. Likely a scan-date assignment bug (writing today's date to a Friday pick that re-scans on Sat/Sun, or weekend cron runs that should skip).</t>
+          <t>Per-user UserPrefs isolation (NAV/plans/watchlist) only holds when users authenticate via Supabase; if they share the single basic-auth (gari/Swing2026), UserPrefs falls back to per-browser localStorage = no true per-user separation</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Trace which writer emits these entries: check run_daily_scan.sh weekday gate, swing_trade.py scan-date logic, and infra/prototype/build_audit_ledger.py date assignment. Weekend launchd should be gated; if it runs intentionally for paper-resolve, mark those rows as REPLAY not PICK.</t>
+          <t>Require Supabase login for multi-user; verify UserPrefs keys per auth id end-to-end (user-prefs.jsx setUser binds sb.auth.getUser)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -844,13 +844,13 @@
       <c r="M4" s="3" t="inlineStr"/>
       <c r="N4" s="8" t="inlineStr"/>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="75" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>DATA-BROKEN-IPO-CALENDAR</t>
+          <t>BUG-WEEKEND-PHANTOM-PICKS</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -860,22 +860,22 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Data / Calendars (broken)</t>
+          <t>Bugs / Audit Ledger</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>ipo_calendar — NASDAQ API times out</t>
+          <t>Weekend phantom picks in audit ledger</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>NASDAQ public IPO API times out from this host (~30s no response). Calendar slot is wired but produces 0 rows.</t>
+          <t>Audit ledger shows phantom picks on May 10 (Sun), May 16 (Sat), May 17 (Sun) — markets closed. Likely a scan-date assignment bug (writing today's date to a Friday pick that re-scans on Sat/Sun, or weekend cron runs that should skip).</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Investigate timeout first (UA headers / proxy / rate-limited IP) before alt-source. Candidate alternates: SEC S-1 filings via EDGAR full-text-search, IPO Monitor RSS, Yahoo Finance IPO page.</t>
+          <t>Trace which writer emits these entries: check run_daily_scan.sh weekday gate, swing_trade.py scan-date logic, and infra/prototype/build_audit_ledger.py date assignment. Weekend launchd should be gated; if it runs intentionally for paper-resolve, mark those rows as REPLAY not PICK.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>DATA-BROKEN-CONGRESSIONAL-TRADES</t>
+          <t>DATA-BROKEN-IPO-CALENDAR</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -906,22 +906,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Data / Catalysts (broken)</t>
+          <t>Data / Calendars (broken)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>congressional_trades — sources dead</t>
+          <t>ipo_calendar — NASDAQ API times out</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Senate Stock Watcher GitHub + S3 mirror both return dead/empty responses. The catalysts slot is wired but the scraper produces 0 rows.</t>
+          <t>NASDAQ public IPO API times out from this host (~30s no response). Calendar slot is wired but produces 0 rows.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Replace dead source with direct efts.sec.gov integration (Form 4 XBRL parsing); add House Clerk site fallback for House STOCK Act filings. Scope: 1-2d dev + XBRL schema work. Free-data only per CLAUDE.md.</t>
+          <t>Investigate timeout first (UA headers / proxy / rate-limited IP) before alt-source. Candidate alternates: SEC S-1 filings via EDGAR full-text-search, IPO Monitor RSS, Yahoo Finance IPO page.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -942,7 +942,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>PARITY-REALTIME-DATA</t>
+          <t>DATA-BROKEN-CONGRESSIONAL-TRADES</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -952,22 +952,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Data / Infrastructure / Platform Parity</t>
+          <t>Data / Catalysts (broken)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Real-Time Data (streaming quotes)</t>
+          <t>congressional_trades — sources dead</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Replace the 5-minute batch refresh with sub-second streaming quotes during market hours so charts + price ladder + Trade Plan PnL update in real time.</t>
+          <t>Senate Stock Watcher GitHub + S3 mirror both return dead/empty responses. The catalysts slot is wired but the scraper produces 0 rows.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Use the Schwab websocket feed (already in the paid stack — no new license per CLAUDE.md) into a local pub/sub buffer; kairos sub-tabs subscribe via SSE/WebSocket from server.py; cache TTL pinned at 1s during RTH.</t>
+          <t>Replace dead source with direct efts.sec.gov integration (Form 4 XBRL parsing); add House Clerk site fallback for House STOCK Act filings. Scope: 1-2d dev + XBRL schema work. Free-data only per CLAUDE.md.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -988,7 +988,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-1</t>
+          <t>PARITY-REALTIME-DATA</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -998,22 +998,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Data Infra / Bar-Store</t>
+          <t>Data / Infrastructure / Platform Parity</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>SQLite daily_bars schema + read/write</t>
+          <t>Real-Time Data (streaming quotes)</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>No local OHLCV history store exists; scans re-fetch per-ticker daily bars from EODHD (~10K calls/day, ~68% of 2026-06-08 usage; tripped 95K quota guard). See docs/scope_bar_store.md.</t>
+          <t>Replace the 5-minute batch refresh with sub-second streaming quotes during market hours so charts + price ladder + Trade Plan PnL update in real time.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Add daily_bars(ticker,date,o,h,l,c,v,adjusted_close,source,ingested_at) to data/swingtrade.db (PK ticker+date, idx). Idempotent upsert writer + DB reader + tests. SQLite stays primary; no new deps.</t>
+          <t>Use the Schwab websocket feed (already in the paid stack — no new license per CLAUDE.md) into a local pub/sub buffer; kairos sub-tabs subscribe via SSE/WebSocket from server.py; cache TTL pinned at 1s during RTH.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-2</t>
+          <t>BARSTORE-1</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1049,17 +1049,17 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>One-time 20yr backfill</t>
+          <t>SQLite daily_bars schema + read/write</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>One eod(ticker,from_date=2005) returns full history = 1 call/ticker; backfilling the universe is ~6-8K calls ONCE vs ~10K/day recurring.</t>
+          <t>No local OHLCV history store exists; scans re-fetch per-ticker daily bars from EODHD (~10K calls/day, ~68% of 2026-06-08 usage; tripped 95K quota guard). See docs/scope_bar_store.md.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>eodhd_client.backfill_history() pages the universe 1-call/ticker, paced under EODHD_SHARED_LIMITER (950/min), overnight launchd only, resumable. NO new license (uses existing EODHD).</t>
+          <t>Add daily_bars(ticker,date,o,h,l,c,v,adjusted_close,source,ingested_at) to data/swingtrade.db (PK ticker+date, idx). Idempotent upsert writer + DB reader + tests. SQLite stays primary; no new deps.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-3</t>
+          <t>BARSTORE-2</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1095,17 +1095,17 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>DB-first failover in fetch_ohlcv_with_failover</t>
+          <t>One-time 20yr backfill</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Once history is local, scans/backtests must read DB-first and hit EODHD only for the current incomplete day + gaps.</t>
+          <t>One eod(ticker,from_date=2005) returns full history = 1 call/ticker; backfilling the universe is ~6-8K calls ONCE vs ~10K/day recurring.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Repoint data_fetcher.fetch_ohlcv_with_failover to read daily_bars first; EODHD fallback for today/gaps. Parity-check 100 tickers vs current cache/eodhd within float tol.</t>
+          <t>eodhd_client.backfill_history() pages the universe 1-call/ticker, paced under EODHD_SHARED_LIMITER (950/min), overnight launchd only, resumable. NO new license (uses existing EODHD).</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1120,13 +1120,13 @@
       <c r="M10" s="3" t="inlineStr"/>
       <c r="N10" s="8" t="inlineStr"/>
     </row>
-    <row r="11" ht="75" customHeight="1">
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>MODE-4</t>
+          <t>BARSTORE-3</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1136,22 +1136,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine</t>
+          <t>Data Infra / Bar-Store</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Walk-forward validation of Phase-3 per-mode pillar weights</t>
+          <t>DB-first failover in fetch_ohlcv_with_failover</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>MODE-3 shipped intuition-based pillar weights without backtest evidence (principle 7 override). Need walk-forward validation that the per-mode weights don't degrade vs the single-set baseline.</t>
+          <t>Once history is local, scans/backtests must read DB-first and hit EODHD only for the current incomplete day + gaps.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>scripts/validate_per_mode_weights.py: runs baseline backtest + 3 mode-weighted backtests (252d, min_score=50), compares WR/PF/maxDD/Sharpe per mode. Revert criterion: any mode ≤1.0× PF or ≤-5pp WR vs baseline → flip per_mode_pillar_reweight._enabled to false. See docs/per_mode_decisions_roadmap.md Phase 3.</t>
+          <t>Repoint data_fetcher.fetch_ohlcv_with_failover to read daily_bars first; EODHD fallback for today/gaps. Parity-check 100 tickers vs current cache/eodhd within float tol.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1166,13 +1166,13 @@
       <c r="M11" s="3" t="inlineStr"/>
       <c r="N11" s="8" t="inlineStr"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="75" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SCALE-1</t>
+          <t>MODE-4</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1182,22 +1182,22 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Deployment · 500-user</t>
+          <t>Decision Engine</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Multi-worker server + concurrency load test</t>
+          <t>Walk-forward validation of Phase-3 per-mode pillar weights</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Single uvicorn worker (uvicorn.run, no workers=); CPU-bound paths (65MB ML-file parse, scoring) block the event loop; untested at 500 concurrent on one Cloudflare tunnel</t>
+          <t>MODE-3 shipped intuition-based pillar weights without backtest evidence (principle 7 override). Need walk-forward validation that the per-mode weights don't degrade vs the single-set baseline.</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>gunicorn/uvicorn --workers N (or app server), profile + offload blocking calls, run a 500-concurrent load test before certifying</t>
+          <t>scripts/validate_per_mode_weights.py: runs baseline backtest + 3 mode-weighted backtests (252d, min_score=50), compares WR/PF/maxDD/Sharpe per mode. Revert criterion: any mode ≤1.0× PF or ≤-5pp WR vs baseline → flip per_mode_pillar_reweight._enabled to false. See docs/per_mode_decisions_roadmap.md Phase 3.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1212,13 +1212,13 @@
       <c r="M12" s="3" t="inlineStr"/>
       <c r="N12" s="8" t="inlineStr"/>
     </row>
-    <row r="13" ht="75" customHeight="1">
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>PARITY-PAPER-TRADING-RT</t>
+          <t>SCALE-1</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1228,22 +1228,22 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Execution / Paper / Platform Parity</t>
+          <t>Deployment · 500-user</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Real-Time Paper Trading</t>
+          <t>Multi-worker server + concurrency load test</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Execute simulated trades against live market prices via the Alpaca paper account; track fills, slippage and PnL in real time so paper validation mirrors what live trading would look like.</t>
+          <t>Single uvicorn worker (uvicorn.run, no workers=); CPU-bound paths (65MB ML-file parse, scoring) block the event loop; untested at 500 concurrent on one Cloudflare tunnel</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Extend executor.py to route signals through the Alpaca paper REST + websocket API; webhook fills back into cache/portfolio.json; expose a 'Paper Trade' toggle on the Trade Plan card. Partially built (executor.py --submit), needs always-on wrapper.</t>
+          <t>gunicorn/uvicorn --workers N (or app server), profile + offload blocking calls, run a 500-concurrent load test before certifying</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -1258,13 +1258,13 @@
       <c r="M13" s="3" t="inlineStr"/>
       <c r="N13" s="8" t="inlineStr"/>
     </row>
-    <row r="14" ht="45" customHeight="1">
+    <row r="14" ht="75" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>REGIME-CONDITIONAL-MODELS</t>
+          <t>PARITY-PAPER-TRADING-RT</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -1274,22 +1274,22 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>ML / Accuracy</t>
+          <t>Execution / Paper / Platform Parity</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional ML models (principle 5)</t>
+          <t>Real-Time Paper Trading</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>train separate direction models per regime instead of one spanning all; #1 accuracy lever</t>
+          <t>Execute simulated trades against live market prices via the Alpaca paper account; track fills, slippage and PnL in real time so paper validation mirrors what live trading would look like.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>ml/train.py regime split</t>
+          <t>Extend executor.py to route signals through the Alpaca paper REST + websocket API; webhook fills back into cache/portfolio.json; expose a 'Paper Trade' toggle on the Trade Plan card. Partially built (executor.py --submit), needs always-on wrapper.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>OPS-1</t>
+          <t>REGIME-CONDITIONAL-MODELS</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1320,39 +1320,27 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>ML / Accuracy</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Snapshot cleanup (scripts/cleanup_after_2026_05_16.sh)</t>
+          <t>Regime-conditional ML models (principle 5)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Pre-Saturday session migration created intermediate snapshot files safe to remove after a week.</t>
+          <t>train separate direction models per regime instead of one spanning all; #1 accuracy lever</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Run scripts/cleanup_after_2026_05_16.sh after 2026-05-16 cutoff.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>2 min</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Win: cleaner repo.</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Calendar reminder for 2026-05-16.</t>
-        </is>
-      </c>
+          <t>ml/train.py regime split</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1360,19 +1348,15 @@
       </c>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+      <c r="N15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>SCHWAB-REAUTH-PENDING</t>
+          <t>OPS-1</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1382,27 +1366,39 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Ops / Schwab (operational)</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Schwab re-auth to unlock option Greeks</t>
+          <t>Snapshot cleanup (scripts/cleanup_after_2026_05_16.sh)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>refresh token expired (invalid_grant, 7-day). Run python3 schwab_auth.py oauth -&gt; real option premiums/Greeks flow into the Options calc (currently honest BS-model fallback).</t>
+          <t>Pre-Saturday session migration created intermediate snapshot files safe to remove after a week.</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>user action: schwab_auth.py oauth</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="5" t="inlineStr"/>
+          <t>Run scripts/cleanup_after_2026_05_16.sh after 2026-05-16 cutoff.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2 min</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Win: cleaner repo.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Calendar reminder for 2026-05-16.</t>
+        </is>
+      </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1410,7 +1406,11 @@
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="3" t="inlineStr"/>
-      <c r="N16" s="8" t="inlineStr"/>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>QUANT-5</t>
+          <t>SCHWAB-REAUTH-PENDING</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1428,39 +1428,27 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Quant</t>
+          <t>Ops / Schwab (operational)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Mover predictor v3 — NLP earnings tone + options flow features</t>
+          <t>Schwab re-auth to unlock option Greeks</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>v1 had leakage. v2 fixed leakage but AUC stuck at 0.546 — pure technical features at entry don't predict mover success.</t>
+          <t>refresh token expired (invalid_grant, 7-day). Run python3 schwab_auth.py oauth -&gt; real option premiums/Greeks flow into the Options calc (currently honest BS-model fallback).</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Build v3 with NEW feature classes (don't retrain): NLP earnings-call tone embeddings, options-flow IV skew + UOA put/call delta, catalyst-conditional models (subset by tag). A6 logger captures most inputs going forward.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>days</t>
-        </is>
-      </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>Caveat: exploratory research, not config-tuning.</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Don't retrain v1/v2 — both definitive AUC 0.546 negative.</t>
-        </is>
-      </c>
+          <t>user action: schwab_auth.py oauth</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1468,19 +1456,15 @@
       </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="165" customHeight="1">
+      <c r="N17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>TV-RATING-CROSS-CHECK</t>
+          <t>QUANT-5</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -1490,37 +1474,37 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Signals / Cross-Check</t>
+          <t>Quant</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Validate (or zero out) the ±3 TV-rating tech-score bonus</t>
+          <t>Mover predictor v3 — NLP earnings tone + options flow features</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>DISCOVERY 2026-05-11: TV-rating ±3 score bonus has been live in analysis.py:8627 for some time, modifying every BUY signal's technical pillar score. NO _validations entry, NO Wilson-CI, NO walk-forward justification for the ±3 magnitude. Worse: tv_rating was never captured on the 689 closed trades in picks_history or 1,301 signal_log entries — retroactive validation is impossible. Violates Principle 1 (n&lt;30 refusal) + Principle 7 (no knob-tweaking without evidence).</t>
+          <t>v1 had leakage. v2 fixed leakage but AUC stuck at 0.546 — pure technical features at entry don't predict mover success.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (SHIPPED 2026-05-11): (a) tv_bonus zeroed in analysis.py:8627 — score no longer mutated; (b) tv_recommendation + tv_rec_value + buy/sell/neutral counts now logged per signal in signal_tracker.log_signals() so prospective evidence accumulates; (c) tv_rating still surfaced in tech['details'] as INFORMATIONAL only — no score impact. Phase 2 (PENDING n&gt;=30, est. 6-12 weeks): run Wilson-LB(BUY|TV STRONG_BUY) vs Wilson-LB(BUY) over the prospectively-logged signals. If the agreement-conditional Wilson-LB beats unconditional by a meaningful margin (&gt;=3pp), re-enable with a magnitude justified by the regression. If not, kill the cross-check permanently (Principle 4 falsification — do not retune, do not lower the threshold).</t>
+          <t>Build v3 with NEW feature classes (don't retrain): NLP earnings-call tone embeddings, options-flow IV skew + UOA put/call delta, catalyst-conditional models (subset by tag). A6 logger captures most inputs going forward.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Phase 1: hours (done). Phase 2: hours of analysis + calendar wait for n&gt;=30.</t>
+          <t>days</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Mechanism (Principle 2): TV rating is an independent server-side aggregation of ~26 indicators. Two independent technical aggregations may improve precision over our 5-pillar score alone. Falsification (Principle 4): if agreement-conditional Wilson-LB &lt;= unconditional after n&gt;=30, the cross-check has no edge — kill, don't retune. Risk of CURRENT state (Phase 1): we have been over-weighting TV-STRONG_BUY signals by +3 tech-pts with zero evidence; this could have systematically biased BUY selection. Capping at 0 removes that bias going forward but does not undo past trade selection bias.</t>
+          <t>Caveat: exploratory research, not config-tuning.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Default apply_to_score=false locked. Validation requires logged tv_rating on &gt;=30 CLOSED BUY trades (currently 0). Earliest Phase-2 validation window: ~6-12 weeks of scans from 2026-05-11. Pairs with the v2 dashboard TV sub-tab (infra/prototype/subtabs/tv/) which is iframe-only today. Do NOT add per-mode / per-regime elaboration until Phase 2 evidence justifies even the basic bonus.</t>
+          <t>Don't retrain v1/v2 — both definitive AUC 0.546 negative.</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
@@ -1532,17 +1516,17 @@
       <c r="M18" s="3" t="inlineStr"/>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>Phase 1 smoke: run python3 swing_trade.py and confirm (1) tech['details']['tv_rating'] still appears in deep-dive output labeled 'informational — bonus disabled pending validation'; (2) signal_log.json entries for new scans contain tv_recommendation + tv_rec_value + buy/sell/neutral_count populated. Phase 2 trigger: when `python3 -c 'import json; print(sum(1 for r in json.load(open("data/signal_log.json")) if r.get("tv_recommendation") and r.get("result")))'` &gt;= 30, run the agreement-conditional Wilson-LB analysis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="90" customHeight="1">
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="165" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>TEST-MAE-MFE</t>
+          <t>TV-RATING-CROSS-CHECK</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1552,27 +1536,39 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Testing / Validation (Tier 1)</t>
+          <t>Signals / Cross-Check</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>MAE / MFE Analyzer — tune stops + targets from data</t>
+          <t>Validate (or zero out) the ±3 TV-rating tech-score bonus</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Maximum Adverse Excursion vs Maximum Favorable Excursion analyzer. signal_log.json already tracks mae_pct + mfe_pct for closed trades. Output: 'Stops triggered at -5% on winners that later hit +20% → stops too tight' or 'Trades exited at +6% target left avg +12% on table → targets too conservative'. Directly improves trade-plan math.</t>
+          <t>DISCOVERY 2026-05-11: TV-rating ±3 score bonus has been live in analysis.py:8627 for some time, modifying every BUY signal's technical pillar score. NO _validations entry, NO Wilson-CI, NO walk-forward justification for the ±3 magnitude. Worse: tv_rating was never captured on the 689 closed trades in picks_history or 1,301 signal_log entries — retroactive validation is impossible. Violates Principle 1 (n&lt;30 refusal) + Principle 7 (no knob-tweaking without evidence).</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Read signal_log.json closed entries; scatter-plot mae vs realized PnL + mfe vs realized PnL; quantile bins (10/25/50/75/90); render as a new Testing tab card. Effort ~30min — data already there.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr"/>
+          <t>Phase 1 (SHIPPED 2026-05-11): (a) tv_bonus zeroed in analysis.py:8627 — score no longer mutated; (b) tv_recommendation + tv_rec_value + buy/sell/neutral counts now logged per signal in signal_tracker.log_signals() so prospective evidence accumulates; (c) tv_rating still surfaced in tech['details'] as INFORMATIONAL only — no score impact. Phase 2 (PENDING n&gt;=30, est. 6-12 weeks): run Wilson-LB(BUY|TV STRONG_BUY) vs Wilson-LB(BUY) over the prospectively-logged signals. If the agreement-conditional Wilson-LB beats unconditional by a meaningful margin (&gt;=3pp), re-enable with a magnitude justified by the regression. If not, kill the cross-check permanently (Principle 4 falsification — do not retune, do not lower the threshold).</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1: hours (done). Phase 2: hours of analysis + calendar wait for n&gt;=30.</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Mechanism (Principle 2): TV rating is an independent server-side aggregation of ~26 indicators. Two independent technical aggregations may improve precision over our 5-pillar score alone. Falsification (Principle 4): if agreement-conditional Wilson-LB &lt;= unconditional after n&gt;=30, the cross-check has no edge — kill, don't retune. Risk of CURRENT state (Phase 1): we have been over-weighting TV-STRONG_BUY signals by +3 tech-pts with zero evidence; this could have systematically biased BUY selection. Capping at 0 removes that bias going forward but does not undo past trade selection bias.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Default apply_to_score=false locked. Validation requires logged tv_rating on &gt;=30 CLOSED BUY trades (currently 0). Earliest Phase-2 validation window: ~6-12 weeks of scans from 2026-05-11. Pairs with the v2 dashboard TV sub-tab (infra/prototype/subtabs/tv/) which is iframe-only today. Do NOT add per-mode / per-regime elaboration until Phase 2 evidence justifies even the basic bonus.</t>
+        </is>
+      </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1580,7 +1576,11 @@
       </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="8" t="inlineStr"/>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>Phase 1 smoke: run python3 swing_trade.py and confirm (1) tech['details']['tv_rating'] still appears in deep-dive output labeled 'informational — bonus disabled pending validation'; (2) signal_log.json entries for new scans contain tv_recommendation + tv_rec_value + buy/sell/neutral_count populated. Phase 2 trigger: when `python3 -c 'import json; print(sum(1 for r in json.load(open("data/signal_log.json")) if r.get("tv_recommendation") and r.get("result")))'` &gt;= 30, run the agreement-conditional Wilson-LB analysis.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>TEST-MC-BOOTSTRAP</t>
+          <t>TEST-MAE-MFE</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -1603,17 +1603,17 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Monte Carlo Bootstrap — confidence intervals on Sharpe/PF/WR</t>
+          <t>MAE / MFE Analyzer — tune stops + targets from data</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Randomly resample closed trades 10,000x to build distributions over each metric. Wilson LB only covers WR; this covers Sharpe, Sortino, PF, max-DD, hit-rate, payoff ratio. Output: 'Sharpe 1.42, 95% CI [0.88, 1.94]' — you would know whether 1.42 is robust or noise. Standard hedge-fund metric, supports principle #1 (statistical rigor).</t>
+          <t>Maximum Adverse Excursion vs Maximum Favorable Excursion analyzer. signal_log.json already tracks mae_pct + mfe_pct for closed trades. Output: 'Stops triggered at -5% on winners that later hit +20% → stops too tight' or 'Trades exited at +6% target left avg +12% on table → targets too conservative'. Directly improves trade-plan math.</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Numpy bootstrap on signal_log trade PnL array, k=10000 resamples; compute distributions over each metric; render percentile bands. Effort 1-2hr.</t>
+          <t>Read signal_log.json closed entries; scatter-plot mae vs realized PnL + mfe vs realized PnL; quantile bins (10/25/50/75/90); render as a new Testing tab card. Effort ~30min — data already there.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>TEST-PERMUTATION</t>
+          <t>TEST-MC-BOOTSTRAP</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Permutation Test — is the edge REAL or coin flip?</t>
+          <t>Monte Carlo Bootstrap — confidence intervals on Sharpe/PF/WR</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Randomly shuffle BUY/SELL/AVOID labels on historical signals 1000x, recompute strategy returns. If real returns are not significantly better than scrambled returns, there is no edge. Direct test of principle #4 (adversarial mindset / falsification). Output: 'Real strategy: +18.7%. Random labels (1000 sims): +0.2% +/- 4.1%. p-value: 0.0001'.</t>
+          <t>Randomly resample closed trades 10,000x to build distributions over each metric. Wilson LB only covers WR; this covers Sharpe, Sortino, PF, max-DD, hit-rate, payoff ratio. Output: 'Sharpe 1.42, 95% CI [0.88, 1.94]' — you would know whether 1.42 is robust or noise. Standard hedge-fund metric, supports principle #1 (statistical rigor).</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Shuffle decision-column of signal_log 1000x; recompute portfolio return per shuffle; rank real return vs null distribution; report p-value. Effort ~1hr.</t>
+          <t>Numpy bootstrap on signal_log trade PnL array, k=10000 resamples; compute distributions over each metric; render percentile bands. Effort 1-2hr.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>TEST-REGIME-COND</t>
+          <t>TEST-PERMUTATION</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -1695,17 +1695,17 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Regime-Conditional Performance — where does it work?</t>
+          <t>Permutation Test — is the edge REAL or coin flip?</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Partition closed trades by regime (risk_on_trending / choppy / risk_off / panic) and compute WR / PF / Sharpe per regime. Per principle #5 (regime conditioning over averages). Example output: 'Trend Continuation WR: 41% overall · 62% in risk_on_trending · 18% in choppy'. Tells you which sleeves to size up/down per regime.</t>
+          <t>Randomly shuffle BUY/SELL/AVOID labels on historical signals 1000x, recompute strategy returns. If real returns are not significantly better than scrambled returns, there is no edge. Direct test of principle #4 (adversarial mindset / falsification). Output: 'Real strategy: +18.7%. Random labels (1000 sims): +0.2% +/- 4.1%. p-value: 0.0001'.</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Group signal_log entries by regime_at_signal (already logged); compute Wilson LB on WR + bootstrapped PF/Sharpe per regime; output a (setup x regime) heatmap. Effort ~1hr.</t>
+          <t>Shuffle decision-column of signal_log 1000x; recompute portfolio return per shuffle; rank real return vs null distribution; report p-value. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1720,38 +1720,38 @@
       <c r="M22" s="3" t="inlineStr"/>
       <c r="N22" s="8" t="inlineStr"/>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>PARITY-BACKTEST-UI</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>TEST-REGIME-COND</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Backtesting / Platform Parity</t>
+          <t>Testing / Validation (Tier 1)</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>In-app Backtesting UI</t>
+          <t>Regime-Conditional Performance — where does it work?</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Expose backtest.py + walk_forward_v2.py inside the kairos UI — a user picks a strategy/date range/universe and runs it without dropping to the terminal.</t>
+          <t>Partition closed trades by regime (risk_on_trending / choppy / risk_off / panic) and compute WR / PF / Sharpe per regime. Per principle #5 (regime conditioning over averages). Example output: 'Trend Continuation WR: 41% overall · 62% in risk_on_trending · 18% in choppy'. Tells you which sleeves to size up/down per regime.</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Add a 'Backtest' workspace in the kairos sidebar; wire a form to a /v2/backtest endpoint that shells out to backtest.py and streams stdout via SSE; render Sharpe / PF / Wilson-LB / equity curve when the run completes.</t>
+          <t>Group signal_log entries by regime_at_signal (already logged); compute Wilson LB on WR + bootstrapped PF/Sharpe per regime; output a (setup x regime) heatmap. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>BUG-MISSING-D1S</t>
+          <t>PARITY-BACKTEST-UI</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1782,22 +1782,22 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Bugs / Audit Ledger</t>
+          <t>Backtesting / Platform Parity</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>4 missing D1s for May 15 (out of 87)</t>
+          <t>In-app Backtesting UI</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>4 of 87 May-15 picks have null D1 (next-day close). Probably thin EODHD coverage on small-caps — acceptable noise band but worth confirming.</t>
+          <t>Expose backtest.py + walk_forward_v2.py inside the kairos UI — a user picks a strategy/date range/universe and runs it without dropping to the terminal.</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Identify the 4 tickers; check EODHD eod() response for each on 2026-05-16; if EODHD returned null, document as known-limitation; if EODHD returned a value, fix the ingest. Effort ~20min.</t>
+          <t>Add a 'Backtest' workspace in the kairos sidebar; wire a form to a /v2/backtest endpoint that shells out to backtest.py and streams stdout via SSE; render Sharpe / PF / Wilson-LB / equity curve when the run completes.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>PARITY-CHANNEL-BAR</t>
+          <t>BUG-MISSING-D1S</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1828,22 +1828,22 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Chart Indicators / Platform Parity</t>
+          <t>Bugs / Audit Ledger</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Channel Bar overlay</t>
+          <t>4 missing D1s for May 15 (out of 87)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Donchian / Keltner / Bollinger envelope overlay on the chart — top + bottom band with mid-line.</t>
+          <t>4 of 87 May-15 picks have null D1 (next-day close). Probably thin EODHD coverage on small-caps — acceptable noise band but worth confirming.</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Compute channels via pandas-ta in feature_extractor.py (or live in chart.js using bar data); render as semi-transparent band; toggle in the Chart sub-tab control bar.</t>
+          <t>Identify the 4 tickers; check EODHD eod() response for each on 2026-05-16; if EODHD returned null, document as known-limitation; if EODHD returned a value, fix the ingest. Effort ~20min.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>PARITY-RBI-GBI-WINDOW</t>
+          <t>PARITY-CHANNEL-BAR</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
@@ -1879,17 +1879,17 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>RBI/GBI Window (regime bias bands)</t>
+          <t>Channel Bar overlay</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Color-coded vertical bands on the chart timeline showing risk-on (green/GBI) vs risk-off (red/RBI) regime windows so the user can see at-a-glance whether prior price action happened in a hostile or friendly regime.</t>
+          <t>Donchian / Keltner / Bollinger envelope overlay on the chart — top + bottom band with mid-line.</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Read cache/regime_history.json and draw vertical color bands at each regime transition on the chart canvas; tooltip explains the regime classification (4-regime model: risk_on_trending / risk_on_choppy / risk_off_trending / panic).</t>
+          <t>Compute channels via pandas-ta in feature_extractor.py (or live in chart.js using bar data); render as semi-transparent band; toggle in the Chart sub-tab control bar.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1904,13 +1904,13 @@
       <c r="M26" s="3" t="inlineStr"/>
       <c r="N26" s="8" t="inlineStr"/>
     </row>
-    <row r="27" ht="45" customHeight="1">
+    <row r="27" ht="60" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-HOT-SECTORS-DEAD</t>
+          <t>PARITY-RBI-GBI-WINDOW</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -1920,22 +1920,22 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup</t>
+          <t>Chart Indicators / Platform Parity</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>panelHotSectors() dead-code in kairos.html</t>
+          <t>RBI/GBI Window (regime bias bands)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Hot Sectors panel was removed from the Signal Scanner grid but the panelHotSectors() function is still defined in kairos.html — dead code.</t>
+          <t>Color-coded vertical bands on the chart timeline showing risk-on (green/GBI) vs risk-off (red/RBI) regime windows so the user can see at-a-glance whether prior price action happened in a hostile or friendly regime.</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>grep for panelHotSectors callers; delete function + any unused helpers; verify no console errors. Effort ~2min.</t>
+          <t>Read cache/regime_history.json and draw vertical color bands at each regime transition on the chart canvas; tooltip explains the regime classification (4-regime model: risk_on_trending / risk_on_choppy / risk_off_trending / panic).</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-4</t>
+          <t>CLEAN-HOT-SECTORS-DEAD</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1966,39 +1966,27 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Code Cleanup</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>scripts/migrate_role_capabilities.py — cleanup after 2026-05-16</t>
+          <t>panelHotSectors() dead-code in kairos.html</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>One-shot CapStudio backfill. Already run. Tied to OPS-1 cleanup window.</t>
+          <t>Hot Sectors panel was removed from the Signal Scanner grid but the panelHotSectors() function is still defined in kairos.html — dead code.</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Delete during OPS-1 cleanup pass after 2026-05-16.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>1 min</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>Win: -X lines.</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>Couples with OPS-1.</t>
-        </is>
-      </c>
+          <t>grep for panelHotSectors callers; delete function + any unused helpers; verify no console errors. Effort ~2min.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -2006,19 +1994,15 @@
       </c>
       <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr"/>
-      <c r="N28" s="8" t="inlineStr">
-        <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1">
+      <c r="N28" s="8" t="inlineStr"/>
+    </row>
+    <row r="29" ht="45" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-EARNINGS-CAL-PIT</t>
+          <t>CLEAN-4</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -2028,27 +2012,39 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Data / Calendars (future)</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>earnings_calendar_pit — point-in-time integrity</t>
+          <t>scripts/migrate_role_capabilities.py — cleanup after 2026-05-16</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Earnings calendar with point-in-time integrity (what was expected when). Needed for clean PEAD backtest replay; today's calendar uses the most-recent snapshot only, which leaks future revisions into prior dates.</t>
+          <t>One-shot CapStudio backfill. Already run. Tied to OPS-1 cleanup window.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Snapshot the EODHD earnings calendar daily into a versioned earnings_calendar_history table; join on (ticker, report_date, snapshot_date) for PIT correctness in PEAD backtests.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="5" t="inlineStr"/>
+          <t>Delete during OPS-1 cleanup pass after 2026-05-16.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>1 min</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Win: -X lines.</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Couples with OPS-1.</t>
+        </is>
+      </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -2056,15 +2052,19 @@
       </c>
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr"/>
-      <c r="N29" s="8" t="inlineStr"/>
-    </row>
-    <row r="30" ht="45" customHeight="1">
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-ECONOMIC-CAL</t>
+          <t>DATA-FUTURE-EARNINGS-CAL-PIT</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -2079,17 +2079,17 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>economic_calendar — CPI/PCE/NFP/FOMC dates</t>
+          <t>earnings_calendar_pit — point-in-time integrity</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Macro event calendar with consensus expectations. No source wired today; the pre-FOMC sleeve uses hard-coded FOMC dates and there is no CPI/PCE/NFP awareness.</t>
+          <t>Earnings calendar with point-in-time integrity (what was expected when). Needed for clean PEAD backtest replay; today's calendar uses the most-recent snapshot only, which leaks future revisions into prior dates.</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Investing.com calendar scrape OR Trading Economics free tier; daily refresh; write to economic_calendar; feed pre-FOMC sleeve + risk_off blackout windows.</t>
+          <t>Snapshot the EODHD earnings calendar daily into a versioned earnings_calendar_history table; join on (ticker, report_date, snapshot_date) for PIT correctness in PEAD backtests.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-FDA-CAL</t>
+          <t>DATA-FUTURE-ECONOMIC-CAL</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -2125,17 +2125,17 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>fda_calendar — PDUFA / AdCom dates</t>
+          <t>economic_calendar — CPI/PCE/NFP/FOMC dates</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>FDA decision calendar (PDUFA dates, Advisory Committee meetings) for biotech catalyst tracking.</t>
+          <t>Macro event calendar with consensus expectations. No source wired today; the pre-FOMC sleeve uses hard-coded FOMC dates and there is no CPI/PCE/NFP awareness.</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>FDA public calendar scrape + BiopharmCatalyst free RSS; write to fda_calendar; surface as catalyst tier in any biotech sleeve.</t>
+          <t>Investing.com calendar scrape OR Trading Economics free tier; daily refresh; write to economic_calendar; feed pre-FOMC sleeve + risk_off blackout windows.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-SPLITS-CALENDAR</t>
+          <t>DATA-FUTURE-FDA-CAL</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -2166,22 +2166,22 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Data / Corporate Actions (empty by sample)</t>
+          <t>Data / Calendars (future)</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>splits_calendar — 0 splits in current universe sample</t>
+          <t>fda_calendar — PDUFA / AdCom dates</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>corporate_actions table populates from EODHD but the current universe sample (449 tickers) had 0 splits in the recent window. Calendar reads empty.</t>
+          <t>FDA decision calendar (PDUFA dates, Advisory Committee meetings) for biotech catalyst tracking.</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Expand corporate-actions polling universe to S&amp;P 500 + Russell 1000 (universe list already available); 1-line change in the populator script.</t>
+          <t>FDA public calendar scrape + BiopharmCatalyst free RSS; write to fda_calendar; surface as catalyst tier in any biotech sleeve.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-MODEL-CALIBRATION</t>
+          <t>DATA-EMPTY-SPLITS-CALENDAR</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -2212,22 +2212,22 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Data / ML (empty by design)</t>
+          <t>Data / Corporate Actions (empty by sample)</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>model_calibration — waiting on realization</t>
+          <t>splits_calendar — 0 splits in current universe sample</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Calibration metrics table has no rows because the 5-20 day prediction horizons have not elapsed yet (today's predictions realize over 1-4 weeks).</t>
+          <t>corporate_actions table populates from EODHD but the current universe sample (449 tickers) had 0 splits in the recent window. Calendar reads empty.</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>No code action; populates passively as time passes. Re-check after 2026-06-15 (30d post-shipping).</t>
+          <t>Expand corporate-actions polling universe to S&amp;P 500 + Russell 1000 (universe list already available); 1-line change in the populator script.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-VAR-BREACHES</t>
+          <t>DATA-EMPTY-MODEL-CALIBRATION</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2258,22 +2258,22 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Data / Risk (empty by design)</t>
+          <t>Data / ML (empty by design)</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>var_breaches — waiting on snapshots + drawdown</t>
+          <t>model_calibration — waiting on realization</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>VaR breach log empty because (1) daily portfolio_risk snapshots are still ramping up and (2) no real drawdown day has happened to trigger a breach.</t>
+          <t>Calibration metrics table has no rows because the 5-20 day prediction horizons have not elapsed yet (today's predictions realize over 1-4 weeks).</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>No code action; populates passively. Re-check after first portfolio drawdown &gt;2% or after 60 daily snapshots.</t>
+          <t>No code action; populates passively as time passes. Re-check after 2026-06-15 (30d post-shipping).</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -2288,13 +2288,13 @@
       <c r="M34" s="3" t="inlineStr"/>
       <c r="N34" s="8" t="inlineStr"/>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="45" customHeight="1">
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-INSIDER-EDGAR</t>
+          <t>DATA-EMPTY-VAR-BREACHES</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -2304,22 +2304,22 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Data / SEC EDGAR (future)</t>
+          <t>Data / Risk (empty by design)</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>insider_transactions via Form 4 XBRL</t>
+          <t>var_breaches — waiting on snapshots + drawdown</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker insider buy/sell stream sourced direct from SEC Form 4 filings. Today sourced indirectly via Finviz Elite bulk; direct EDGAR is point-in-time accurate and free.</t>
+          <t>VaR breach log empty because (1) daily portfolio_risk snapshots are still ramping up and (2) no real drawdown day has happened to trigger a breach.</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Build Form 4 XBRL parser; daily ingest from efts.sec.gov; write to insider_transactions table; reconcile against Finviz bulk for cross-check.</t>
+          <t>No code action; populates passively. Re-check after first portfolio drawdown &gt;2% or after 60 daily snapshots.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -2334,13 +2334,13 @@
       <c r="M35" s="3" t="inlineStr"/>
       <c r="N35" s="8" t="inlineStr"/>
     </row>
-    <row r="36" ht="45" customHeight="1">
+    <row r="36" ht="60" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-INSTITUTIONAL-EDGAR</t>
+          <t>DATA-FUTURE-INSIDER-EDGAR</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>institutional_holdings via 13F XBRL</t>
+          <t>insider_transactions via Form 4 XBRL</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker institutional ownership tracking (Form 13F, quarterly). Useful for the Smart Money pillar; today only Finviz inst_own_pct snapshot.</t>
+          <t>Per-ticker insider buy/sell stream sourced direct from SEC Form 4 filings. Today sourced indirectly via Finviz Elite bulk; direct EDGAR is point-in-time accurate and free.</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>13F XBRL parser; quarterly ingest from EDGAR; write to institutional_holdings table with the 45-day reporting lag accounted for in any backtest joins.</t>
+          <t>Build Form 4 XBRL parser; daily ingest from efts.sec.gov; write to insider_transactions table; reconcile against Finviz bulk for cross-check.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-CONGRESSIONAL-EDGAR</t>
+          <t>DATA-FUTURE-INSTITUTIONAL-EDGAR</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -2396,22 +2396,22 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Data / SEC EDGAR (future, alt for broken)</t>
+          <t>Data / SEC EDGAR (future)</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>congressional_trades via EDGAR / House Clerk (alt source)</t>
+          <t>institutional_holdings via 13F XBRL</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Alternate sourcing for congressional trades after Senate Stock Watcher death (see DATA-BROKEN-CONGRESSIONAL-TRADES). Direct from House Clerk + Senate eFD.</t>
+          <t>Per-ticker institutional ownership tracking (Form 13F, quarterly). Useful for the Smart Money pillar; today only Finviz inst_own_pct snapshot.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Scrape House STOCK Act PTR PDFs (House Clerk site); Senate eFD JSON; merge into normalized congressional_trades table.</t>
+          <t>13F XBRL parser; quarterly ingest from EDGAR; write to institutional_holdings table with the 45-day reporting lag accounted for in any backtest joins.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -2432,7 +2432,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>SUPABASE-SYNC-VERIFY</t>
+          <t>DATA-FUTURE-CONGRESSIONAL-EDGAR</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -2442,22 +2442,22 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Data / Supabase</t>
+          <t>Data / SEC EDGAR (future, alt for broken)</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Verify supabase_analysis_sync actually writes</t>
+          <t>congressional_trades via EDGAR / House Clerk (alt source)</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>confirm sync_scan writes (psycopg2 raw SQL not .table API); not silent no-op</t>
+          <t>Alternate sourcing for congressional trades after Senate Stock Watcher death (see DATA-BROKEN-CONGRESSIONAL-TRADES). Direct from House Clerk + Senate eFD.</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>supabase_analysis_sync.py</t>
+          <t>Scrape House STOCK Act PTR PDFs (House Clerk site); Senate eFD JSON; merge into normalized congressional_trades table.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -2472,13 +2472,13 @@
       <c r="M38" s="3" t="inlineStr"/>
       <c r="N38" s="8" t="inlineStr"/>
     </row>
-    <row r="39" ht="60" customHeight="1">
+    <row r="39" ht="45" customHeight="1">
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>DATA-EMPTY-PROD-ENGINE-DEFERRED</t>
+          <t>SUPABASE-SYNC-VERIFY</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -2488,22 +2488,22 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Data / Telemetry (deferred for safety)</t>
+          <t>Data / Supabase</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>8 empty slots — production-engine touches deferred</t>
+          <t>Verify supabase_analysis_sync actually writes</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>8 telemetry/data slots remain empty because populating them requires editing backtest.py / executor.py / signal_filter.py / analysis.py. Deliberately deferred to avoid risk to the live scan + exec paths.</t>
+          <t>confirm sync_scan writes (psycopg2 raw SQL not .table API); not silent no-op</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Enumerate the 8 specifically and grade each one for in-place vs side-car instrumentation. Side-car (write to telemetry DB without changing decision flow) is preferred over hot-path edits.</t>
+          <t>supabase_analysis_sync.py</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -2518,13 +2518,13 @@
       <c r="M39" s="3" t="inlineStr"/>
       <c r="N39" s="8" t="inlineStr"/>
     </row>
-    <row r="40" ht="45" customHeight="1">
+    <row r="40" ht="60" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-4</t>
+          <t>DATA-EMPTY-PROD-ENGINE-DEFERRED</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
@@ -2534,22 +2534,22 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Data Infra / Bar-Store</t>
+          <t>Data / Telemetry (deferred for safety)</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Daily incremental via bulk_eod</t>
+          <t>8 empty slots — production-engine touches deferred</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>After backfill, only the latest bar is needed daily; bulk_eod returns the whole exchange in 1 call.</t>
+          <t>8 telemetry/data slots remain empty because populating them requires editing backtest.py / executor.py / signal_filter.py / analysis.py. Deliberately deferred to avoid risk to the live scan + exec paths.</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Daily launchd job: 1 bulk_eod(exchange) appends last-day bar for all tickers into daily_bars. Target &lt;=2 EODHD calls/day total for OHLCV.</t>
+          <t>Enumerate the 8 specifically and grade each one for in-place vs side-car instrumentation. Side-car (write to telemetry DB without changing decision flow) is preferred over hot-path edits.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-5</t>
+          <t>BARSTORE-4</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
@@ -2585,17 +2585,17 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Corporate-action re-adjustment</t>
+          <t>Daily incremental via bulk_eod</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Stored history must stay split/div-adjusted; a new split re-bases all prior bars. This is where data-integrity bugs hide.</t>
+          <t>After backfill, only the latest bar is needed daily; bulk_eod returns the whole exchange in 1 call.</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Store raw + adjusted_close; small daily job re-adjusts history on split/div events (EODHD div/splits endpoints). Validate no adjustment drift.</t>
+          <t>Daily launchd job: 1 bulk_eod(exchange) appends last-day bar for all tickers into daily_bars. Target &lt;=2 EODHD calls/day total for OHLCV.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -2610,13 +2610,13 @@
       <c r="M41" s="3" t="inlineStr"/>
       <c r="N41" s="8" t="inlineStr"/>
     </row>
-    <row r="42" ht="60" customHeight="1">
+    <row r="42" ht="45" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>BARSTORE-6</t>
+          <t>BARSTORE-5</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -2631,17 +2631,17 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Delisted backfill -&gt; survivorship fix</t>
+          <t>Corporate-action re-adjustment</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Honest backtests need delisted tickers' history + point-in-time membership (membership snapshots already DONE via AIPRED-SURVIVORSHIP). Unblocks audit #1.</t>
+          <t>Stored history must stay split/div-adjusted; a new split re-bases all prior bars. This is where data-integrity bugs hide.</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Backfill delisted-ticker history into daily_bars; point walk_forward_v2 at DB over 20yr. Enables survivorship-bias-free backtests + free validation of staged accuracy tweaks.</t>
+          <t>Store raw + adjusted_close; small daily job re-adjusts history on split/div events (EODHD div/splits endpoints). Validate no adjustment drift.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>EODHD-WIRES-VALIDATE</t>
+          <t>BARSTORE-6</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
@@ -2672,22 +2672,22 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Data Wiring (validate)</t>
+          <t>Data Infra / Bar-Store</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Validate EODHD-side wires on quota reset</t>
+          <t>Delisted backfill -&gt; survivorship fix</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>DCF net-debt/FCF + per-name beta + Book Risk crowding are code-complete + fallback-safe but untested against live EODHD (quota was exhausted). Confirm real values flow after reset.</t>
+          <t>Honest backtests need delisted tickers' history + point-in-time membership (membership snapshots already DONE via AIPRED-SURVIVORSHIP). Unblocks audit #1.</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html /api/fundamentals consumers</t>
+          <t>Backfill delisted-ticker history into daily_bars; point walk_forward_v2 at DB over 20yr. Enables survivorship-bias-free backtests + free validation of staged accuracy tweaks.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2702,13 +2702,13 @@
       <c r="M43" s="3" t="inlineStr"/>
       <c r="N43" s="8" t="inlineStr"/>
     </row>
-    <row r="44" ht="75" customHeight="1">
+    <row r="44" ht="60" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>OVERVIEW-VERDICT-RECON</t>
+          <t>EODHD-WIRES-VALIDATE</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
@@ -2718,22 +2718,22 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine</t>
+          <t>Data Wiring (validate)</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Reconcile compute_final_verdict (stage) vs decisions_by_mode</t>
+          <t>Validate EODHD-side wires on quota reset</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Two engines emit different swing score+verdict for the same name (FTNT: stage=BUY/67 vs decisions_by_mode.swing=WATCH/57). decisions_by_mode omits the catalyst-sleeve EXTENDED-entry relaxation that compute_final_verdict applies, so they disagree.</t>
+          <t>DCF net-debt/FCF + per-name beta + Book Risk crowding are code-complete + fallback-safe but untested against live EODHD (quota was exhausted). Confirm real values flow after reset.</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Have decisions_by_mode consume the same relaxation OR emit a diverges-from-composite flag; decide direction after the entry-quality EXTENDED/MISSED A/B validation lands. Display already fixed (overview.js binds stage).</t>
+          <t>Stocksmith.html /api/fundamentals consumers</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-TRAFFIC-LIGHT-INPUTS</t>
+          <t>OVERVIEW-VERDICT-RECON</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -2764,22 +2764,22 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Detail Lens / Traffic Lights</t>
+          <t>Decision Engine</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Per-ticker risk/fundamentals inputs for lens dots</t>
+          <t>Reconcile compute_final_verdict (stage) vs decisions_by_mode</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Wire t.f_score · t.altman_z · t.roic · t.wacc · t.sharpe_1y · t.dd_recovery_months · t.peer_rank · t.is_held into build_data.py. _qdComputeLensStatus has cascading fallbacks (PEG → fund_score → F-score; beta → kelly → Sharpe), so dots upgrade automatically as fields land.</t>
+          <t>Two engines emit different swing score+verdict for the same name (FTNT: stage=BUY/67 vs decisions_by_mode.swing=WATCH/57). decisions_by_mode omits the catalyst-sleeve EXTENDED-entry relaxation that compute_final_verdict applies, so they disagree.</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Compute in analysis.py / portfolio.py: Piotroski F (existing data), Altman Z (existing data), ROIC vs WACC, 1y Sharpe from price history, peer_rank from cohort, is_held from portfolio_state.json.</t>
+          <t>Have decisions_by_mode consume the same relaxation OR emit a diverges-from-composite flag; decide direction after the entry-quality EXTENDED/MISSED A/B validation lands. Display already fixed (overview.js binds stage).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
@@ -2794,13 +2794,13 @@
       <c r="M45" s="3" t="inlineStr"/>
       <c r="N45" s="8" t="inlineStr"/>
     </row>
-    <row r="46" ht="60" customHeight="1">
+    <row r="46" ht="75" customHeight="1">
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-COHORT-SYMPATHY</t>
+          <t>KAIROS-TRAFFIC-LIGHT-INPUTS</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
@@ -2810,22 +2810,22 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Earnings Lens / Cohort</t>
+          <t>Detail Lens / Traffic Lights</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Peer cohort sympathy correlations</t>
+          <t>Per-ticker risk/fundamentals inputs for lens dots</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Wire t.cohort_peers[].er_sympathy_corr + er_sympathy_move_1d + t.sympathy_history in build_data.py. Today: renderEarnings_Sympathy shows scaffold rows from t.cohort_peers if populated, else placeholder.</t>
+          <t>Wire t.f_score · t.altman_z · t.roic · t.wacc · t.sharpe_1y · t.dd_recovery_months · t.peer_rank · t.is_held into build_data.py. _qdComputeLensStatus has cascading fallbacks (PEG → fund_score → F-score; beta → kelly → Sharpe), so dots upgrade automatically as fields land.</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Compute 8-quarter rolling correlation of 1d post-print move between this name and each cohort peer's ER date. Persist to data.json under t.cohort_peers + t.sympathy_history.</t>
+          <t>Compute in analysis.py / portfolio.py: Piotroski F (existing data), Altman Z (existing data), ROIC vs WACC, 1y Sharpe from price history, peer_rank from cohort, is_held from portfolio_state.json.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -2840,13 +2840,13 @@
       <c r="M46" s="3" t="inlineStr"/>
       <c r="N46" s="8" t="inlineStr"/>
     </row>
-    <row r="47" ht="75" customHeight="1">
+    <row r="47" ht="60" customHeight="1">
       <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>PARITY-IN-APP-TRADING</t>
+          <t>KAIROS-COHORT-SYMPATHY</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -2856,22 +2856,22 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Execution / Live / Platform Parity</t>
+          <t>Earnings Lens / Cohort</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>In-app Trading (broker-integrated live execution)</t>
+          <t>Peer cohort sympathy correlations</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>One-click BUY/SELL from the dashboard to a live Schwab/Alpaca brokerage account.</t>
+          <t>Wire t.cohort_peers[].er_sympathy_corr + er_sympathy_move_1d + t.sympathy_history in build_data.py. Today: renderEarnings_Sympathy shows scaffold rows from t.cohort_peers if populated, else placeholder.</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>OAuth-link the Schwab API (already paid stack); surface an 'Execute' button on the Trade Plan card; explicit AUTHORIZE LIVE TRADING gate per CLAUDE.md security protocol; route every order through the existing risk checks (max-loss-pct, drawdown haircut, regime gate).</t>
+          <t>Compute 8-quarter rolling correlation of 1d post-print move between this name and each cohort peer's ER date. Persist to data.json under t.cohort_peers + t.sympathy_history.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-LIVE-D1</t>
+          <t>PARITY-IN-APP-TRADING</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -2902,22 +2902,22 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Kairos / Audit Ledger</t>
+          <t>Execution / Live / Platform Parity</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Live D1 estimate from Schwab quote during RTH</t>
+          <t>In-app Trading (broker-integrated live execution)</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Replace placeholder D1 (yesterday's close-to-close) with a live Schwab-quote-based intraday estimate during market hours so the audit ledger D1 column is non-stale. Discussed and deferred as semantically muddy (D1 = next-day close, intraday quote is a forecast not a fill).</t>
+          <t>One-click BUY/SELL from the dashboard to a live Schwab/Alpaca brokerage account.</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Add a SCHWAB_LIVE_D1=1 env flag; when ON and during RTH, compute D1_est = (live_quote - signal_entry) / signal_entry and annotate the cell with an 'est' chip. Effort ~1hr.</t>
+          <t>OAuth-link the Schwab API (already paid stack); surface an 'Execute' button on the Trade Plan card; explicit AUTHORIZE LIVE TRADING gate per CLAUDE.md security protocol; route every order through the existing risk checks (max-loss-pct, drawdown haircut, regime gate).</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -2932,13 +2932,13 @@
       <c r="M48" s="3" t="inlineStr"/>
       <c r="N48" s="8" t="inlineStr"/>
     </row>
-    <row r="49" ht="45" customHeight="1">
+    <row r="49" ht="75" customHeight="1">
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-SCANNER-BEARS</t>
+          <t>KAIROS-LIVE-D1</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -2948,22 +2948,22 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Kairos / Signal Scanner</t>
+          <t>Kairos / Audit Ledger</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Top 5 Bears panel</t>
+          <t>Live D1 estimate from Schwab quote during RTH</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Add a 'Top 5 Bears' panel to the Signal Scanner alongside Fresh / Momentum / Earnings / Volume — was proposed but not selected in the initial build.</t>
+          <t>Replace placeholder D1 (yesterday's close-to-close) with a live Schwab-quote-based intraday estimate during market hours so the audit ledger D1 column is non-stale. Discussed and deferred as semantically muddy (D1 = next-day close, intraday quote is a forecast not a fill).</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Mirror existing 4 panels' structure; sort universe by composite bear-score desc; cap at 5; render in the Scanner grid. Effort ~10min.</t>
+          <t>Add a SCHWAB_LIVE_D1=1 env flag; when ON and during RTH, compute D1_est = (live_quote - signal_entry) / signal_entry and annotate the cell with an 'est' chip. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -2978,13 +2978,13 @@
       <c r="M49" s="3" t="inlineStr"/>
       <c r="N49" s="8" t="inlineStr"/>
     </row>
-    <row r="50" ht="60" customHeight="1">
+    <row r="50" ht="45" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-SCANNER-FLIPS</t>
+          <t>KAIROS-SCANNER-BEARS</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
@@ -2999,17 +2999,17 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Today's Flips panel</t>
+          <t>Top 5 Bears panel</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Add a 'Today's Flips' panel to the Signal Scanner — tickers whose verdict flipped vs yesterday (e.g., BUY -&gt; WATCH, WATCH -&gt; BUY, AVOID -&gt; WATCH). Proposed in the 'what else' menu, not selected.</t>
+          <t>Add a 'Top 5 Bears' panel to the Signal Scanner alongside Fresh / Momentum / Earnings / Volume — was proposed but not selected in the initial build.</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Diff today's bundle.verdict against yesterday.verdict per ticker; surface the 5-10 most material flips. Effort ~30min.</t>
+          <t>Mirror existing 4 panels' structure; sort universe by composite bear-score desc; cap at 5; render in the Scanner grid. Effort ~10min.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>ML-RETRAIN-FINBERT-FEATURE</t>
+          <t>KAIROS-SCANNER-FLIPS</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -3040,22 +3040,22 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>ML / Features (future)</t>
+          <t>Kairos / Signal Scanner</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Add FinBERT as a GBM training feature (leak-free)</t>
+          <t>Today's Flips panel</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>needs historical sentiment series — accumulate forward via cache/ml/sentiment_log.jsonl (asof-stamped); add as feature #18 + retrain once ~3-6mo of leak-free history exists</t>
+          <t>Add a 'Today's Flips' panel to the Signal Scanner — tickers whose verdict flipped vs yesterday (e.g., BUY -&gt; WATCH, WATCH -&gt; BUY, AVOID -&gt; WATCH). Proposed in the 'what else' menu, not selected.</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>ml/feature_extractor + historical backfill</t>
+          <t>Diff today's bundle.verdict against yesterday.verdict per ticker; surface the 5-10 most material flips. Effort ~30min.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>ML-AUTOREFRESH-VALIDATE</t>
+          <t>ML-RETRAIN-FINBERT-FEATURE</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -3086,22 +3086,22 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>ML / Pipeline (validate)</t>
+          <t>ML / Features (future)</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Validate ML auto-refresh post-scan + cached-bar reuse</t>
+          <t>Add FinBERT as a GBM training feature (leak-free)</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>ml_edge.run_after_scan=true runs ml.run_ml_edge over the fresh bundle; feature_extractor prefers data_archive (no re-fetch). Confirm end-to-end on next clean scan.</t>
+          <t>needs historical sentiment series — accumulate forward via cache/ml/sentiment_log.jsonl (asof-stamped); add as feature #18 + retrain once ~3-6mo of leak-free history exists</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>swing_trade ML hook + ml/feature_extractor</t>
+          <t>ml/feature_extractor + historical backfill</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-MACRO-EVENTS</t>
+          <t>ML-AUTOREFRESH-VALIDATE</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Macro Lens / Calendar</t>
+          <t>ML / Pipeline (validate)</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>14-day high-impact event window flag</t>
+          <t>Validate ML auto-refresh post-scan + cached-bar reuse</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Wire t.next_macro_event_days = days to next FOMC/CPI/NFP/jobs. _qdComputeLensStatus reads this and downgrades macro lens to amber when event &lt;= 14d even in risk_on_trending regime.</t>
+          <t>ml_edge.run_after_scan=true runs ml.run_ml_edge over the fresh bundle; feature_extractor prefers data_archive (no re-fetch). Confirm end-to-end on next clean scan.</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Add macro_calendar fetch in data_fetcher.py (FRED/Trading Economics free tier or EODHD calendar). Persist to t.next_macro_event_days.</t>
+          <t>swing_trade ML hook + ml/feature_extractor</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -3162,13 +3162,13 @@
       <c r="M53" s="3" t="inlineStr"/>
       <c r="N53" s="8" t="inlineStr"/>
     </row>
-    <row r="54" ht="45" customHeight="1">
+    <row r="54" ht="60" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>CACHE-RECLAIM</t>
+          <t>KAIROS-MACRO-EVENTS</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -3178,22 +3178,22 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Ops / Hygiene</t>
+          <t>Macro Lens / Calendar</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Reclaim ~6GB cache (stray bak + edgar TTL)</t>
+          <t>14-day high-impact event window flag</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>delete 300MB last_bundle.json.bak.precap_promote + add edgar companyfacts prune/TTL (6.1GB)</t>
+          <t>Wire t.next_macro_event_days = days to next FOMC/CPI/NFP/jobs. _qdComputeLensStatus reads this and downgrades macro lens to amber when event &lt;= 14d even in risk_on_trending regime.</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>cache cleanup + edgar_client TTL</t>
+          <t>Add macro_calendar fetch in data_fetcher.py (FRED/Trading Economics free tier or EODHD calendar). Persist to t.next_macro_event_days.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>JOBS-MOMENTUM-SNAPSHOT</t>
+          <t>CACHE-RECLAIM</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -3224,22 +3224,22 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Hygiene</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot job: load or disable</t>
+          <t>Reclaim ~6GB cache (stray bak + edgar TTL)</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>valid plist in repo but not currently loaded; decide launchctl bootstrap vs move to disabled/.</t>
+          <t>delete 300MB last_bundle.json.bak.precap_promote + add edgar companyfacts prune/TTL (6.1GB)</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd/com.swingtrade.momentum-snapshot.plist</t>
+          <t>cache cleanup + edgar_client TTL</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -3254,13 +3254,13 @@
       <c r="M55" s="3" t="inlineStr"/>
       <c r="N55" s="8" t="inlineStr"/>
     </row>
-    <row r="56" ht="60" customHeight="1">
+    <row r="56" ht="45" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>DATA-FUTURE-OPS-TELEMETRY-6</t>
+          <t>JOBS-MOMENTUM-SNAPSHOT</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -3270,22 +3270,22 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Ops / Telemetry (future)</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>6 ops telemetry slots — app-side instrumentation</t>
+          <t>Decide momentum-snapshot job: load or disable</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>6 ops telemetry slots remain unbuilt because they require app-side instrumentation: server middleware, git hooks, scan-time emitters, executor probes, sub-tab render timings, fetch-latency probes.</t>
+          <t>valid plist in repo but not currently loaded; decide launchctl bootstrap vs move to disabled/.</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Build a shared emitter (lib/telemetry.py) writing to a telemetry SQLite; instrument incrementally — server middleware first, then scan emitters; surface in System Status sub-tab.</t>
+          <t>infra/launchd/com.swingtrade.momentum-snapshot.plist</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>SCALE-4</t>
+          <t>DATA-FUTURE-OPS-TELEMETRY-6</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -3316,22 +3316,22 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Ops · 500-user</t>
+          <t>Ops / Telemetry (future)</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Scan reliability so Home is not sparse</t>
+          <t>6 ops telemetry slots — app-side instrumentation</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>When the daily scan is empty (EODHD quota outage), Home shows honest-empty sections + stale-badged regime; users landing mid-outage see little actionable content</t>
+          <t>6 ops telemetry slots remain unbuilt because they require app-side instrumentation: server middleware, git hooks, scan-time emitters, executor probes, sub-tab render timings, fetch-latency probes.</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Ensure morning scan runs reliably + quota headroom; keep STALE badge UX; consider serving last-good bundle with clear age</t>
+          <t>Build a shared emitter (lib/telemetry.py) writing to a telemetry SQLite; instrument incrementally — server middleware first, then scan emitters; surface in System Status sub-tab.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -3346,13 +3346,13 @@
       <c r="M57" s="3" t="inlineStr"/>
       <c r="N57" s="8" t="inlineStr"/>
     </row>
-    <row r="58" ht="75" customHeight="1">
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>OV-INVEST-STRUCT</t>
+          <t>SCALE-4</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -3362,22 +3362,22 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Overview / Target Engine</t>
+          <t>Ops · 500-user</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Real structural invest targets (kill analyst-PT stub)</t>
+          <t>Scan reliability so Home is not sparse</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Invest-mode targets fall back to analyst 12mo PT (invest_stub) for low-vol names (e.g. AAPL) when no structural level qualifies in the invest R-band off the wider stop -&gt; near T1, poor R:R. Per-mode stop scaling fix (2026-06-08) made invest coherent for higher-vol names (NVDA stub=False) but low-vol names still stub.</t>
+          <t>When the daily scan is empty (EODHD quota outage), Home shows honest-empty sections + stale-badged regime; users landing mid-outage see little actionable content</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Wire multi-year structural levels (monthly/yearly swing highs, weekly Fib ext) into the invest candidate set so the invest R-band is populated without the analyst-PT fallback; raise invest max_reach_atr to match a 1-5yr horizon.</t>
+          <t>Ensure morning scan runs reliably + quota headroom; keep STALE badge UX; consider serving last-good bundle with clear age</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -3392,13 +3392,13 @@
       <c r="M58" s="3" t="inlineStr"/>
       <c r="N58" s="8" t="inlineStr"/>
     </row>
-    <row r="59" ht="60" customHeight="1">
+    <row r="59" ht="75" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>SCALE-3</t>
+          <t>OV-INVEST-STRUCT</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -3408,22 +3408,22 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Portfolio · 500-user</t>
+          <t>Overview / Target Engine</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Per-user portfolio vs shared automated book</t>
+          <t>Real structural invest targets (kill analyst-PT stub)</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Home AUTOMATED BOOK is the single shared Alpaca-paper auto-trade account; every viewer sees identical positions; no per-user book (NAV is per-user, positions are not)</t>
+          <t>Invest-mode targets fall back to analyst 12mo PT (invest_stub) for low-vol names (e.g. AAPL) when no structural level qualifies in the invest R-band off the wider stop -&gt; near T1, poor R:R. Per-mode stop scaling fix (2026-06-08) made invest coherent for higher-vol names (NVDA stub=False) but low-vol names still stub.</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Decide: keep as shared model/track-record book by design, OR add a per-user position store keyed to UserPrefs auth id</t>
+          <t>Wire multi-year structural levels (monthly/yearly swing highs, weekly Fib ext) into the invest candidate set so the invest R-band is populated without the analyst-PT fallback; raise invest max_reach_atr to match a 1-5yr horizon.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -3438,13 +3438,13 @@
       <c r="M59" s="3" t="inlineStr"/>
       <c r="N59" s="8" t="inlineStr"/>
     </row>
-    <row r="60" ht="90" customHeight="1">
+    <row r="60" ht="60" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>QUANT-HMM-FF-LGBM-ROADMAP</t>
+          <t>SCALE-3</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -3454,22 +3454,22 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Quant / Modeling Roadmap</t>
+          <t>Portfolio · 500-user</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>HMM regime / Fama-French / LightGBM swap (status unclear)</t>
+          <t>Per-user portfolio vs shared automated book</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Roadmap items pasted as a status table — clarification pending whether user wants execution or just context tracking. Three potential upgrades: (a) HMM-based regime classifier replacing the rule-based 4-regime model, (b) Fama-French factor exposure analysis on closed trades, (c) LightGBM swap-in for HistGradientBoosting in ml/train_historical.py. Each 1-3 days.</t>
+          <t>Home AUTOMATED BOOK is the single shared Alpaca-paper auto-trade account; every viewer sees identical positions; no per-user book (NAV is per-user, positions are not)</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>Confirm intent before executing. If go: HMM first (decouples regime classifier from heuristics, principle #18), then Fama-French attribution (per-strategy factor exposure), then LightGBM swap (likely-marginal accuracy gain vs current HistGB). Each upgrade gated by Wilson-LB validation vs current baseline.</t>
+          <t>Decide: keep as shared model/track-record book by design, OR add a per-user position store keyed to UserPrefs auth id</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -3484,13 +3484,13 @@
       <c r="M60" s="3" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr"/>
     </row>
-    <row r="61" ht="60" customHeight="1">
+    <row r="61" ht="90" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>PARITY-SMART-RISK-LEVELS</t>
+          <t>QUANT-HMM-FF-LGBM-ROADMAP</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
@@ -3500,22 +3500,22 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Risk / Targets / Platform Parity</t>
+          <t>Quant / Modeling Roadmap</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Smart Risk Levels (auto stop + T1/T2)</t>
+          <t>HMM regime / Fama-French / LightGBM swap (status unclear)</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Auto-place stop / T1 / T2 dots on the chart with confluence reasoning (HVN, AVWAP, fractal, ATR, Fib). Already computed by the structural target engine but not surfaced on the new Chart sub-tab.</t>
+          <t>Roadmap items pasted as a status table — clarification pending whether user wants execution or just context tracking. Three potential upgrades: (a) HMM-based regime classifier replacing the rule-based 4-regime model, (b) Fama-French factor exposure analysis on closed trades, (c) LightGBM swap-in for HistGradientBoosting in ml/train_historical.py. Each 1-3 days.</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Read cache/target_engine/{TICKER}_{MODE}.json and overlay the levels on the chart canvas with hover tooltips citing the confluence factors; gated by use_structural_targets flag (M2.5 cutover).</t>
+          <t>Confirm intent before executing. If go: HMM first (decouples regime classifier from heuristics, principle #18), then Fama-French attribution (per-strategy factor exposure), then LightGBM swap (likely-marginal accuracy gain vs current HistGB). Each upgrade gated by Wilson-LB validation vs current baseline.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>KAIROS-L2-BOOK</t>
+          <t>PARITY-SMART-RISK-LEVELS</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
@@ -3546,22 +3546,22 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Risk Lens / Execution</t>
+          <t>Risk / Targets / Platform Parity</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>L2 bid/ask depth at price levels</t>
+          <t>Smart Risk Levels (auto stop + T1/T2)</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Wire t.l2_book from Schwab streaming API → render in renderRisk_LiquidityLadder. Today: ADV-derived size tiers shown as scaffold. Schwab streaming requires WebSocket session — see schwab_client.py.</t>
+          <t>Auto-place stop / T1 / T2 dots on the chart with confluence reasoning (HVN, AVWAP, fractal, ATR, Fib). Already computed by the structural target engine but not surfaced on the new Chart sub-tab.</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Subscribe to Schwab Level-II quote stream; persist top-of-book snapshot into t.l2_book = {bid:[{px,size}], ask:[{px,size}]}. Frontend already reads these fields if present.</t>
+          <t>Read cache/target_engine/{TICKER}_{MODE}.json and overlay the levels on the chart canvas with hover tooltips citing the confluence factors; gated by use_structural_targets flag (M2.5 cutover).</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -3582,7 +3582,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>PARITY-AI-SIGNALS-V1</t>
+          <t>KAIROS-L2-BOOK</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
@@ -3592,22 +3592,22 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Signals / Platform Parity</t>
+          <t>Risk Lens / Execution</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>1st-Gen AI Signals</t>
+          <t>L2 bid/ask depth at price levels</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Surface a baseline AI BUY/SELL signal stream on the chart as quick-glance arrows/dots — the competitor-platform feature (TrendSpider, Trade Ideas) users expect to see at a glance, separate from the full ML Edge sub-tab.</t>
+          <t>Wire t.l2_book from Schwab streaming API → render in renderRisk_LiquidityLadder. Today: ADV-derived size tiers shown as scaffold. Schwab streaming requires WebSocket session — see schwab_client.py.</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Reuse ML Edge dir-head + cone outputs but render as 1-bar arrows/markers on the new Chart sub-tab; isolate from the 10-section Technicals view; respect cache/ml_edge_predictions.json freshness.</t>
+          <t>Subscribe to Schwab Level-II quote stream; persist top-of-book snapshot into t.l2_book = {bid:[{px,size}], ask:[{px,size}]}. Frontend already reads these fields if present.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -3622,13 +3622,13 @@
       <c r="M63" s="3" t="inlineStr"/>
       <c r="N63" s="8" t="inlineStr"/>
     </row>
-    <row r="64" ht="45" customHeight="1">
+    <row r="64" ht="60" customHeight="1">
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>TEST-AB-PAPER</t>
+          <t>PARITY-AI-SIGNALS-V1</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
@@ -3638,22 +3638,22 @@
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Testing / Validation (Tier 2)</t>
+          <t>Signals / Platform Parity</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>A/B Paper Split — live comparison</t>
+          <t>1st-Gen AI Signals</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Run config A on half the paper portfolio and config B on the other half; real-time comparison of WR / PF / equity divergence over 30-60d window.</t>
+          <t>Surface a baseline AI BUY/SELL signal stream on the chart as quick-glance arrows/dots — the competitor-platform feature (TrendSpider, Trade Ideas) users expect to see at a glance, separate from the full ML Edge sub-tab.</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>Extend executor.py to accept --variant flag; persist per-variant portfolio state; cross-section panel in System Status sub-tab. Effort 3-4hr.</t>
+          <t>Reuse ML Edge dir-head + cone outputs but render as 1-bar arrows/markers on the new Chart sub-tab; isolate from the 10-section Technicals view; respect cache/ml_edge_predictions.json freshness.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -3668,13 +3668,13 @@
       <c r="M64" s="3" t="inlineStr"/>
       <c r="N64" s="8" t="inlineStr"/>
     </row>
-    <row r="65" ht="60" customHeight="1">
+    <row r="65" ht="45" customHeight="1">
       <c r="A65" s="2" t="n">
         <v>64</v>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>TEST-BENCHMARK-SPY</t>
+          <t>TEST-AB-PAPER</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
@@ -3689,17 +3689,17 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>Benchmark vs SPY — alpha / beta / IR</t>
+          <t>A/B Paper Split — live comparison</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Compute strategy alpha, beta, information ratio vs SPY benchmark. Standard performance attribution; turns 'we made +X%' into 'we made +Y% over SPY at lower drawdown'.</t>
+          <t>Run config A on half the paper portfolio and config B on the other half; real-time comparison of WR / PF / equity divergence over 30-60d window.</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Daily portfolio_value series joined to SPY adjusted-close; regress daily returns -&gt; SPY returns for beta + alpha; IR = (mean excess return) / (std excess return); render in System Status. Effort ~1hr.</t>
+          <t>Extend executor.py to accept --variant flag; persist per-variant portfolio state; cross-section panel in System Status sub-tab. Effort 3-4hr.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr"/>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>TEST-DD-DIST</t>
+          <t>TEST-BENCHMARK-SPY</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
@@ -3735,17 +3735,17 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Drawdown Distribution Simulator</t>
+          <t>Benchmark vs SPY — alpha / beta / IR</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Bootstrap 1000 portfolio paths from closed-trade distribution; measure tail-drawdown probability at p95/p99; supports principle #9 (drawdown asymmetry — losing 50% requires +100% to recover).</t>
+          <t>Compute strategy alpha, beta, information ratio vs SPY benchmark. Standard performance attribution; turns 'we made +X%' into 'we made +Y% over SPY at lower drawdown'.</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>Resample trade sequence with replacement; build equity curves; compute max-DD per path; histogram + tail percentiles; feed into position-sizing math. Effort 2-3hr.</t>
+          <t>Daily portfolio_value series joined to SPY adjusted-close; regress daily returns -&gt; SPY returns for beta + alpha; IR = (mean excess return) / (std excess return); render in System Status. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>TEST-SENSITIVITY</t>
+          <t>TEST-DD-DIST</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
@@ -3781,17 +3781,17 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Sensitivity / Robustness Test</t>
+          <t>Drawdown Distribution Simulator</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Perturb each config parameter +/-20% (score floors, stop ATR mult, R:R floor, regime thresholds) and check whether the strategy still passes the gate. Finds overfit knobs that only work at one exact value.</t>
+          <t>Bootstrap 1000 portfolio paths from closed-trade distribution; measure tail-drawdown probability at p95/p99; supports principle #9 (drawdown asymmetry — losing 50% requires +100% to recover).</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Grid-walk key config thresholds; re-run backtest at each point; build sensitivity heatmap (param vs PF); flag any knob whose +/-20% perturbation collapses PF &gt;50%. Effort ~2hr.</t>
+          <t>Resample trade sequence with replacement; build equity curves; compute max-DD per path; histogram + tail percentiles; feed into position-sizing math. Effort 2-3hr.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>TEST-SLIPPAGE-STRESS</t>
+          <t>TEST-SENSITIVITY</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
@@ -3827,17 +3827,17 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Slippage Stress Test</t>
+          <t>Sensitivity / Robustness Test</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Double the slippage assumption (ATR/ADV-scaled model from audit #5) and recompute backtest stats. Validates fragile execution dependence per principle #19 (slippage realism).</t>
+          <t>Perturb each config parameter +/-20% (score floors, stop ATR mult, R:R floor, regime thresholds) and check whether the strategy still passes the gate. Finds overfit knobs that only work at one exact value.</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>Re-run backtest with SLIPPAGE_MULT=2.0; compare WR/PF/Sharpe deltas; if a strategy collapses at 2x slippage it is execution-fragile and should be down-sized. Effort ~1hr.</t>
+          <t>Grid-walk key config thresholds; re-run backtest at each point; build sensitivity heatmap (param vs PF); flag any knob whose +/-20% perturbation collapses PF &gt;50%. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>TEST-CORRELATED-FAILURE</t>
+          <t>TEST-SLIPPAGE-STRESS</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
@@ -3868,22 +3868,22 @@
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Testing / Validation (Tier 3)</t>
+          <t>Testing / Validation (Tier 2)</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>Correlated-Failure — what if EODHD goes down 24h?</t>
+          <t>Slippage Stress Test</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Simulate the impact of the sole data provider (EODHD) being unavailable for 24-48h during market hours. What happens to (a) the scan, (b) live exec, (c) the dashboard?</t>
+          <t>Double the slippage assumption (ATR/ADV-scaled model from audit #5) and recompute backtest stats. Validates fragile execution dependence per principle #19 (slippage realism).</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>Inject EODHD error responses in a paper environment; observe failure modes (fallback to last-known cache vs hard error vs degraded scan); document recovery RTO; tighten any silent-fail paths discovered. Effort 2-3hr.</t>
+          <t>Re-run backtest with SLIPPAGE_MULT=2.0; compare WR/PF/Sharpe deltas; if a strategy collapses at 2x slippage it is execution-fragile and should be down-sized. Effort ~1hr.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -3898,13 +3898,13 @@
       <c r="M69" s="3" t="inlineStr"/>
       <c r="N69" s="8" t="inlineStr"/>
     </row>
-    <row r="70" ht="45" customHeight="1">
+    <row r="70" ht="60" customHeight="1">
       <c r="A70" s="2" t="n">
         <v>69</v>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>TEST-CRASH-REPLAY</t>
+          <t>TEST-CORRELATED-FAILURE</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -3919,17 +3919,17 @@
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Crash Replay — 2008/2020/2022 stress</t>
+          <t>Correlated-Failure — what if EODHD goes down 24h?</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Apply current portfolio composition to historical crash days (2008 GFC, 2020 COVID, 2022 rate-shock); measure realized drawdown + recovery time per scenario.</t>
+          <t>Simulate the impact of the sole data provider (EODHD) being unavailable for 24-48h during market hours. What happens to (a) the scan, (b) live exec, (c) the dashboard?</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>Snapshot today's positions; price-replay against historical daily OHLC from those windows; report per-crisis max-DD and time-to-recovery. Effort 2-3hr.</t>
+          <t>Inject EODHD error responses in a paper environment; observe failure modes (fallback to last-known cache vs hard error vs degraded scan); document recovery RTO; tighten any silent-fail paths discovered. Effort 2-3hr.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -3944,13 +3944,13 @@
       <c r="M70" s="3" t="inlineStr"/>
       <c r="N70" s="8" t="inlineStr"/>
     </row>
-    <row r="71" ht="60" customHeight="1">
+    <row r="71" ht="45" customHeight="1">
       <c r="A71" s="2" t="n">
         <v>70</v>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>TEST-KELLY-SIM</t>
+          <t>TEST-CRASH-REPLAY</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
@@ -3965,17 +3965,17 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Half-Kelly vs Full-Kelly sizing simulation</t>
+          <t>Crash Replay — 2008/2020/2022 stress</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Visualize portfolio growth under Half-Kelly (current default) vs Full-Kelly vs Quarter-Kelly sizing rules; quantifies the volatility-vs-CAGR tradeoff that principle #9 codifies.</t>
+          <t>Apply current portfolio composition to historical crash days (2008 GFC, 2020 COVID, 2022 rate-shock); measure realized drawdown + recovery time per scenario.</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>Bootstrap N portfolio paths under each Kelly fraction; chart median equity curve + percentile fans; surface terminal-wealth distribution. Effort ~2hr.</t>
+          <t>Snapshot today's positions; price-replay against historical daily OHLC from those windows; report per-crisis max-DD and time-to-recovery. Effort 2-3hr.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>TEST-SLIPPAGE-ATTR</t>
+          <t>TEST-KELLY-SIM</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
@@ -4011,17 +4011,17 @@
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Slippage Attribution — signal PnL vs realized PnL gap</t>
+          <t>Half-Kelly vs Full-Kelly sizing simulation</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>For each closed trade, compute the gap between the model's predicted entry/exit and the actual fill price. Aggregate by setup/ticker/regime to find where slippage eats edge.</t>
+          <t>Visualize portfolio growth under Half-Kelly (current default) vs Full-Kelly vs Quarter-Kelly sizing rules; quantifies the volatility-vs-CAGR tradeoff that principle #9 codifies.</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>Read signal_log entries (which has the signal price) and join to paper_fills.json (which has the realized price); compute slippage_bp per trade; group + percentile. Effort ~2hr.</t>
+          <t>Bootstrap N portfolio paths under each Kelly fraction; chart median equity curve + percentile fans; surface terminal-wealth distribution. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>TEST-TAX-AWARE</t>
+          <t>TEST-SLIPPAGE-ATTR</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
@@ -4057,17 +4057,17 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Tax-Aware Backtest — short-term cap-gains haircut</t>
+          <t>Slippage Attribution — signal PnL vs realized PnL gap</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Apply short-term capital-gains tax (35-40% on gains held &lt;1yr) to backtest PnL. Real after-tax return for a US retail account is materially lower than gross.</t>
+          <t>For each closed trade, compute the gap between the model's predicted entry/exit and the actual fill price. Aggregate by setup/ticker/regime to find where slippage eats edge.</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>Add post_tax_pnl column to backtest output; apply 35% haircut to short-term gains (&gt;0 PnL, held &lt;365d) and 15% to long-term; report Sharpe / total-return pre vs post tax. Effort ~2hr.</t>
+          <t>Read signal_log entries (which has the signal price) and join to paper_fills.json (which has the realized price); compute slippage_bp per trade; group + percentile. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>WAIT-CALIB-DRIFT-SPARK</t>
+          <t>TEST-TAX-AWARE</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
@@ -4098,22 +4098,22 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Calibration</t>
+          <t>Testing / Validation (Tier 3)</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>Calibration drift sparkline populates</t>
+          <t>Tax-Aware Backtest — short-term cap-gains haircut</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>The calibration-drift sparkline in the ML Edge sub-tab needs multiple training cycles to populate (weeks). Each morning scan retrains and appends a calibration row; the sparkline reads from that history table.</t>
+          <t>Apply short-term capital-gains tax (35-40% on gains held &lt;1yr) to backtest PnL. Real after-tax return for a US retail account is materially lower than gross.</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Passive wait. Re-check after 4-6 weekly retrain cycles. If still empty, verify ml.train_historical writes to cache/ml/calibration_history.jsonl on each run.</t>
+          <t>Add post_tax_pnl column to backtest output; apply 35% haircut to short-term gains (&gt;0 PnL, held &lt;365d) and 15% to long-term; report Sharpe / total-return pre vs post tax. Effort ~2hr.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -4128,13 +4128,13 @@
       <c r="M74" s="3" t="inlineStr"/>
       <c r="N74" s="8" t="inlineStr"/>
     </row>
-    <row r="75" ht="45" customHeight="1">
+    <row r="75" ht="60" customHeight="1">
       <c r="A75" s="2" t="n">
         <v>74</v>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>WAIT-DRIFT-SNAPSHOTS</t>
+          <t>WAIT-CALIB-DRIFT-SPARK</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
@@ -4144,22 +4144,22 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Drift Tracking</t>
+          <t>Time-Dependent / Calibration</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Diff vs yesterday + 30-day drift populate</t>
+          <t>Calibration drift sparkline populates</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>The 'diff vs yesterday' + 30-day drift columns need 2+ daily snapshots stored. Starts populating tomorrow's scan.</t>
+          <t>The calibration-drift sparkline in the ML Edge sub-tab needs multiple training cycles to populate (weeks). Each morning scan retrains and appends a calibration row; the sparkline reads from that history table.</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>Passive wait; first populated values appear in the next morning's scan output. Verify the snapshot persister wrote a row today.</t>
+          <t>Passive wait. Re-check after 4-6 weekly retrain cycles. If still empty, verify ml.train_historical writes to cache/ml/calibration_history.jsonl on each run.</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>WAIT-ML-PICKS-RESOLVE</t>
+          <t>WAIT-DRIFT-SNAPSHOTS</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -4190,22 +4190,22 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Picks History</t>
+          <t>Time-Dependent / Drift Tracking</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Picks-history outcome resolution (resolve_ml_picks.py)</t>
+          <t>Diff vs yesterday + 30-day drift populate</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>resolve_ml_picks.py needs 5 trading days from each pick to resolve outcomes. First AI Edge batch (picks from ~2026-05-18) resolves around 2026-05-23.</t>
+          <t>The 'diff vs yesterday' + 30-day drift columns need 2+ daily snapshots stored. Starts populating tomorrow's scan.</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>Passive wait. Re-check on 2026-05-23; verify resolve_ml_picks.py runs in run_daily_scan.sh and populates picks_history.json outcome columns.</t>
+          <t>Passive wait; first populated values appear in the next morning's scan output. Verify the snapshot persister wrote a row today.</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -4220,13 +4220,13 @@
       <c r="M76" s="3" t="inlineStr"/>
       <c r="N76" s="8" t="inlineStr"/>
     </row>
-    <row r="77" ht="60" customHeight="1">
+    <row r="77" ht="45" customHeight="1">
       <c r="A77" s="2" t="n">
         <v>76</v>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>WAIT-SURVIVORSHIP-DECAY</t>
+          <t>WAIT-ML-PICKS-RESOLVE</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
@@ -4236,22 +4236,22 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Survivorship Haircut</t>
+          <t>Time-Dependent / Picks History</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Survivorship haircut shrinking 3pp -&gt; 0.5pp</t>
+          <t>Picks-history outcome resolution (resolve_ml_picks.py)</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>The -3pp WR survivorship haircut should shrink as monthly S&amp;P 500 / R1000 membership snapshots accumulate (Wikipedia revision history). Once 24+ months of snapshots are stored, the haircut can fade toward 0.5pp.</t>
+          <t>resolve_ml_picks.py needs 5 trading days from each pick to resolve outcomes. First AI Edge batch (picks from ~2026-05-18) resolves around 2026-05-23.</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>Passive wait — currently only current-membership data. Re-evaluate annually. Until then keep -3pp haircut per CLAUDE.md principle #6.</t>
+          <t>Passive wait. Re-check on 2026-05-23; verify resolve_ml_picks.py runs in run_daily_scan.sh and populates picks_history.json outcome columns.</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>WAIT-WF-EQUITY-REAL</t>
+          <t>WAIT-SURVIVORSHIP-DECAY</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
@@ -4282,22 +4282,22 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Time-Dependent / Walk-Forward</t>
+          <t>Time-Dependent / Survivorship Haircut</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Walk-forward equity curve switches to REAL track</t>
+          <t>Survivorship haircut shrinking 3pp -&gt; 0.5pp</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Currently the equity curve renders backtest-derived returns. Switches to REAL track once 5+ resolved AI Edge picks are available — first batch resolves ~2026-05-23, so REAL curve activates ~2026-05-24.</t>
+          <t>The -3pp WR survivorship haircut should shrink as monthly S&amp;P 500 / R1000 membership snapshots accumulate (Wikipedia revision history). Once 24+ months of snapshots are stored, the haircut can fade toward 0.5pp.</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>Passive wait. Re-check on 2026-05-24; verify the equity curve flips from BACKTEST badge to REAL badge once n_resolved &gt;= 5.</t>
+          <t>Passive wait — currently only current-membership data. Re-evaluate annually. Until then keep -3pp haircut per CLAUDE.md principle #6.</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>PARITY-10-CHARTS-GRID</t>
+          <t>WAIT-WF-EQUITY-REAL</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
@@ -4328,22 +4328,22 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>UI / Layout / Platform Parity</t>
+          <t>Time-Dependent / Walk-Forward</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>10-chart multi-pane grid</t>
+          <t>Walk-forward equity curve switches to REAL track</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Display up to 10 ticker charts side-by-side in a configurable grid (2x5, 3x4, etc.) for at-a-glance correlation/leadership reads — what TrendSpider and Trade Ideas users default to.</t>
+          <t>Currently the equity curve renders backtest-derived returns. Switches to REAL track once 5+ resolved AI Edge picks are available — first batch resolves ~2026-05-23, so REAL curve activates ~2026-05-24.</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>New 'Grid' workspace in kairos that renders N lightweight-chart canvases; ticker list drag-droppable; persists ticker set per layout.</t>
+          <t>Passive wait. Re-check on 2026-05-24; verify the equity curve flips from BACKTEST badge to REAL badge once n_resolved &gt;= 5.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>PARITY-CUSTOM-LAYOUTS</t>
+          <t>PARITY-10-CHARTS-GRID</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
@@ -4379,17 +4379,17 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Customizable Layouts (save/load workspace presets)</t>
+          <t>10-chart multi-pane grid</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>User drags/resizes panels in the kairos workspace and saves the arrangement as a named preset (Day-Trade view / Swing view / Research view) and switches between them.</t>
+          <t>Display up to 10 ticker charts side-by-side in a configurable grid (2x5, 3x4, etc.) for at-a-glance correlation/leadership reads — what TrendSpider and Trade Ideas users default to.</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>Persist layout JSON in cache/user_layouts.json (per-user once auth lands); sidebar dropdown to switch; default presets shipped (Swing / Position / Research).</t>
+          <t>New 'Grid' workspace in kairos that renders N lightweight-chart canvases; ticker list drag-droppable; persists ticker set per layout.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -4404,13 +4404,13 @@
       <c r="M80" s="3" t="inlineStr"/>
       <c r="N80" s="8" t="inlineStr"/>
     </row>
-    <row r="81" ht="75" customHeight="1">
+    <row r="81" ht="60" customHeight="1">
       <c r="A81" s="2" t="n">
         <v>80</v>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>STRUCT-TARGETS-PHASE2</t>
+          <t>PARITY-CUSTOM-LAYOUTS</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
@@ -4420,51 +4420,35 @@
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Targets</t>
+          <t>UI / Layout / Platform Parity</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Structural targets Phase 2 — engine uses them as T1/T2</t>
+          <t>Customizable Layouts (save/load workspace presets)</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (shipped 2026-05-10): structural target sources (fractal, fib, EW Wave-3) display on Plan tab as informational. Phase 2: actually use these as T1/T2 instead of ATR-multiple targets. Needs per-source x regime evidence (&gt;=30 trades each).</t>
+          <t>User drags/resizes panels in the kairos workspace and saves the arrangement as a named preset (Day-Trade view / Swing view / Research view) and switches between them.</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Add config flag target_source = atr_multiple | structural. When structural, T1 = nearest_above with R:R&gt;=3 from {fractal_high, fib_127, EW_T1}. Fall back to ATR if R:R floor not met. Backtest side-by-side with current ATR-multiple.</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
-        <is>
-          <t>1 day + backtest</t>
-        </is>
-      </c>
-      <c r="I81" s="5" t="inlineStr">
-        <is>
-          <t>High win potential, medium risk</t>
-        </is>
-      </c>
-      <c r="J81" s="5" t="inlineStr">
-        <is>
-          <t>Awaiting evidence. Phase 1 currently just populates display field; need 3-4 weeks of trade data with target_sources captured before Phase 2 is decidable.</t>
-        </is>
-      </c>
-      <c r="K81" s="11" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
+          <t>Persist layout JSON in cache/user_layouts.json (per-user once auth lands); sidebar dropdown to switch; default presets shipped (Swing / Position / Research).</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="5" t="inlineStr"/>
+      <c r="J81" s="5" t="inlineStr"/>
+      <c r="K81" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr"/>
       <c r="M81" s="3" t="inlineStr"/>
-      <c r="N81" s="8" t="inlineStr">
-        <is>
-          <t>Run backtest with target_source=structural and target_source=atr_multiple on same window. Compare PF/WR/avg_win.</t>
-        </is>
-      </c>
+      <c r="N81" s="8" t="inlineStr"/>
     </row>
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="2" t="n">
@@ -4472,77 +4456,69 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>K6</t>
-        </is>
-      </c>
-      <c r="C82" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>STRUCT-TARGETS-PHASE2</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>Strategy / Targets</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Single canonical trade plan object — every tab reads from one source</t>
+          <t>Structural targets Phase 2 — engine uses them as T1/T2</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Different dashboard tabs (Plan, Overview, Technicals, Models) computed their own derived values from raw signal data — drift risk, inconsistent UI numbers.</t>
+          <t>Phase 1 (shipped 2026-05-10): structural target sources (fractal, fib, EW Wave-3) display on Plan tab as informational. Phase 2: actually use these as T1/T2 instead of ATR-multiple targets. Needs per-source x regime evidence (&gt;=30 trades each).</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>New canonical_trade_plan.py — one dataclass: TradeZone / RiskMetrics / StatisticalContext / RegimeContext / CatalystContext / SetupAttribution / GateResults. swing_trade.py attaches it per signal. Live Wilson-CI lookup from signal_log per setup×regime. Mechanism hypothesis per setup family.</t>
+          <t>Add config flag target_source = atr_multiple | structural. When structural, T1 = nearest_above with R:R&gt;=3 from {fractal_high, fib_127, EW_T1}. Fall back to ATR if R:R floor not met. Backtest side-by-side with current ATR-multiple.</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>1 day + backtest</t>
         </is>
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Win: tabs converge on one truth; future tabs bind to dataclass fields.</t>
+          <t>High win potential, medium risk</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
         <is>
-          <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
-        </is>
-      </c>
-      <c r="K82" s="12" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M82" s="3" t="inlineStr">
-        <is>
-          <t>2c9b9f339</t>
-        </is>
-      </c>
+          <t>Awaiting evidence. Phase 1 currently just populates display field; need 3-4 weeks of trade data with target_sources captured before Phase 2 is decidable.</t>
+        </is>
+      </c>
+      <c r="K82" s="11" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="3" t="inlineStr"/>
       <c r="N82" s="8" t="inlineStr">
         <is>
-          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="90" customHeight="1">
+          <t>Run backtest with target_source=structural and target_source=atr_multiple on same window. Compare PF/WR/avg_win.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="75" customHeight="1">
       <c r="A83" s="2" t="n">
         <v>82</v>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>B3-WEEKLY-FIX</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4552,29 +4528,37 @@
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Backtest / Bug Fix</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Backtest must build weekly_df from daily for weekly_bull computation</t>
+          <t>Single canonical trade plan object — every tab reads from one source</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Backtest harness was passing only the daily df to the engine, but weekly_bull (a hard gate in trend-continuation setups) requires resampled weekly bars. Without it, every backtest signal fell through the weekly_bull gate as 'unknown' which the engine treated as fail. Effective on-paper effect: 0 BUYs across many backtests despite valid signals in the daily series.</t>
+          <t>Different dashboard tabs (Plan, Overview, Technicals, Models) computed their own derived values from raw signal data — drift risk, inconsistent UI numbers.</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>Build weekly_df via df.resample('W').agg({open: first, high: max, low: min, close: last, volume: sum}) before each pre-trade-gate call. Pass alongside daily.</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr"/>
-      <c r="I83" s="5" t="inlineStr"/>
+          <t>New canonical_trade_plan.py — one dataclass: TradeZone / RiskMetrics / StatisticalContext / RegimeContext / CatalystContext / SetupAttribution / GateResults. swing_trade.py attaches it per signal. Live Wilson-CI lookup from signal_log per setup×regime. Mechanism hypothesis per setup family.</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>Win: tabs converge on one truth; future tabs bind to dataclass fields.</t>
+        </is>
+      </c>
       <c r="J83" s="5" t="inlineStr">
         <is>
-          <t>P0 because this silently invalidated every Trend-Continuation backtest signal in the 750d simulations Saturday. Found during Q1-step5 0-BUY investigation — daily df alone made the engine think every TC signal failed weekly_bull as "unknown".</t>
+          <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
         </is>
       </c>
       <c r="K83" s="12" t="inlineStr">
@@ -4584,27 +4568,27 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t>985cd182b</t>
+          <t>2c9b9f339</t>
         </is>
       </c>
       <c r="N83" s="8" t="inlineStr">
         <is>
-          <t>1. python3 backtest.py --window 250d --min-score 65 → confirm BUYs &gt; 0. 2. Compare cache/portfolio_backtest_250d_min65_h5_20260510_*.json before/after fix → expected: pre-fix had 0 trades on Trend-Continuation family; post-fix has them. 3. grep -E "weekly_df|weekly_bull" backtest.py to verify the resample call is in the inner loop.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="75" customHeight="1">
+          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="90" customHeight="1">
       <c r="A84" s="2" t="n">
         <v>83</v>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>VARIANT-F-BT</t>
+          <t>B3-WEEKLY-FIX</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4614,27 +4598,31 @@
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Backtest Parity</t>
+          <t>Backtest / Bug Fix</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>Variant F regime-conditional multipliers not wired into backtest path</t>
+          <t>Backtest must build weekly_df from daily for weekly_bull computation</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>backtest.py:418 uses tracker.get_setup_weight_multiplier (reading picks_history) but never consults config.setup_score_multiplier_by_regime. So Variant F's TC×bull=0.0 kill never applied in backtest — explains why 105 TC bull trades persisted in 250d backtest despite live kill in config.</t>
+          <t>Backtest harness was passing only the daily df to the engine, but weekly_bull (a hard gate in trend-continuation setups) requires resampled weekly bars. Without it, every backtest signal fell through the weekly_bull gate as 'unknown' which the engine treated as fail. Effective on-paper effect: 0 BUYs across many backtests despite valid signals in the daily series.</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>Add Variant F lookup at backtest.py:442 mirroring analysis.py:8867 logic. Same demotion gate (n&gt;=30 + wr_lb&lt;0.30). Comment cross-reference live path.</t>
+          <t>Build weekly_df via df.resample('W').agg({open: first, high: max, low: min, close: last, volume: sum}) before each pre-trade-gate call. Pass alongside daily.</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="5" t="inlineStr"/>
-      <c r="J84" s="5" t="inlineStr"/>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>P0 because this silently invalidated every Trend-Continuation backtest signal in the 750d simulations Saturday. Found during Q1-step5 0-BUY investigation — daily df alone made the engine think every TC signal failed weekly_bull as "unknown".</t>
+        </is>
+      </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4647,18 +4635,22 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>0cdb13340</t>
-        </is>
-      </c>
-      <c r="N84" s="8" t="inlineStr"/>
-    </row>
-    <row r="85" ht="45" customHeight="1">
+          <t>985cd182b</t>
+        </is>
+      </c>
+      <c r="N84" s="8" t="inlineStr">
+        <is>
+          <t>1. python3 backtest.py --window 250d --min-score 65 → confirm BUYs &gt; 0. 2. Compare cache/portfolio_backtest_250d_min65_h5_20260510_*.json before/after fix → expected: pre-fix had 0 trades on Trend-Continuation family; post-fix has them. 3. grep -E "weekly_df|weekly_bull" backtest.py to verify the resample call is in the inner loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="75" customHeight="1">
       <c r="A85" s="2" t="n">
         <v>84</v>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>P0-WEEKLY</t>
+          <t>VARIANT-F-BT</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -4668,39 +4660,27 @@
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Backtest infra</t>
+          <t>Backtest Parity</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Backtest must build weekly_df from daily (0-BUYs root cause)</t>
+          <t>Variant F regime-conditional multipliers not wired into backtest path</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>GATE-1 produced 0 BUYs because backtest _score_as_of did not pass weekly_df. _weekly_ema_alignment(None) returned bullish=False; setup_gates demoted every BUY.</t>
+          <t>backtest.py:418 uses tracker.get_setup_weight_multiplier (reading picks_history) but never consults config.setup_score_multiplier_by_regime. So Variant F's TC×bull=0.0 kill never applied in backtest — explains why 105 TC bull trades persisted in 250d backtest despite live kill in config.</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Resample daily OHLCV to W-FRI inside _score_as_of. Pass weekly_df to score_technicals. Leakage-free.</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>20 min</t>
-        </is>
-      </c>
-      <c r="I85" s="5" t="inlineStr">
-        <is>
-          <t>CRITICAL — system was unable to backtest</t>
-        </is>
-      </c>
-      <c r="J85" s="5" t="inlineStr">
-        <is>
-          <t>Validated: --smoke produced 5 BUYs in 5d, PF 7.74.</t>
-        </is>
-      </c>
+          <t>Add Variant F lookup at backtest.py:442 mirroring analysis.py:8867 logic. Same demotion gate (n&gt;=30 + wr_lb&lt;0.30). Comment cross-reference live path.</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="5" t="inlineStr"/>
+      <c r="J85" s="5" t="inlineStr"/>
       <c r="K85" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4713,22 +4693,18 @@
       </c>
       <c r="M85" s="3" t="inlineStr">
         <is>
-          <t>985cd182b</t>
-        </is>
-      </c>
-      <c r="N85" s="8" t="inlineStr">
-        <is>
-          <t>python3 backtest.py --smoke - cache/portfolio_backtest.json total_trades &gt; 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="75" customHeight="1">
+          <t>0cdb13340</t>
+        </is>
+      </c>
+      <c r="N85" s="8" t="inlineStr"/>
+    </row>
+    <row r="86" ht="45" customHeight="1">
       <c r="A86" s="2" t="n">
         <v>85</v>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>ROLLING-SHARPE-FIX</t>
+          <t>P0-WEEKLY</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -4738,27 +4714,39 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Decision Engine / Bug</t>
+          <t>Backtest infra</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>Rolling-Sharpe brake firing on contaminated data</t>
+          <t>Backtest must build weekly_df from daily (0-BUYs root cause)</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>Two bugs: (a) WATCH-conviction signals being written with verdict='BUY' inflated loss count; (b) same physical trade re-emitted as fresh daily signal counted 3× in rolling-20 window. Net: false brake activation pausing ALL new BUYs system-wide. Real Sharpe -0.42; system reported -1.732</t>
+          <t>GATE-1 produced 0 BUYs because backtest _score_as_of did not pass weekly_df. _weekly_ema_alignment(None) returned bullish=False; setup_gates demoted every BUY.</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Upstream fix: swing_trade.py line 3110 _resolve_verdict() detects WATCH conviction and overrides bucket label. Read-time fix: decision_engine.compute_rolling_sharpe_kill_state dedupes by (ticker,entry,pnl,exit_reason). Historical cleanup: scripts/dedupe_signal_log.py removed 133 mislabels + 90 dupes (backed up)</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr"/>
-      <c r="I86" s="5" t="inlineStr"/>
-      <c r="J86" s="5" t="inlineStr"/>
+          <t>Resample daily OHLCV to W-FRI inside _score_as_of. Pass weekly_df to score_technicals. Leakage-free.</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>20 min</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>CRITICAL — system was unable to backtest</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>Validated: --smoke produced 5 BUYs in 5d, PF 7.74.</t>
+        </is>
+      </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4766,23 +4754,27 @@
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N86" s="8" t="inlineStr"/>
-    </row>
-    <row r="87" ht="90" customHeight="1">
+          <t>985cd182b</t>
+        </is>
+      </c>
+      <c r="N86" s="8" t="inlineStr">
+        <is>
+          <t>python3 backtest.py --smoke - cache/portfolio_backtest.json total_trades &gt; 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="75" customHeight="1">
       <c r="A87" s="2" t="n">
         <v>86</v>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>OPERATING-MINDSET</t>
+          <t>ROLLING-SHARPE-FIX</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4792,39 +4784,27 @@
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Decision Engine / Bug</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
+          <t>Rolling-Sharpe brake firing on contaminated data</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
+          <t>Two bugs: (a) WATCH-conviction signals being written with verdict='BUY' inflated loss count; (b) same physical trade re-emitted as fresh daily signal counted 3× in rolling-20 window. Net: false brake activation pausing ALL new BUYs system-wide. Real Sharpe -0.42; system reported -1.732</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I87" s="5" t="inlineStr">
-        <is>
-          <t>Win: codified discipline survives session/agent boundaries.</t>
-        </is>
-      </c>
-      <c r="J87" s="5" t="inlineStr">
-        <is>
-          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
-        </is>
-      </c>
+          <t>Upstream fix: swing_trade.py line 3110 _resolve_verdict() detects WATCH conviction and overrides bucket label. Read-time fix: decision_engine.compute_rolling_sharpe_kill_state dedupes by (ticker,entry,pnl,exit_reason). Historical cleanup: scripts/dedupe_signal_log.py removed 133 mislabels + 90 dupes (backed up)</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="5" t="inlineStr"/>
+      <c r="J87" s="5" t="inlineStr"/>
       <c r="K87" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4832,27 +4812,23 @@
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="N87" s="8" t="inlineStr">
-        <is>
-          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="60" customHeight="1">
+          <t>27fd646b1</t>
+        </is>
+      </c>
+      <c r="N87" s="8" t="inlineStr"/>
+    </row>
+    <row r="88" ht="90" customHeight="1">
       <c r="A88" s="2" t="n">
         <v>87</v>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>EXEC-TRADABLE-ENUM</t>
+          <t>OPERATING-MINDSET</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4862,27 +4838,39 @@
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Execution · Auto-Trade</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>Stock executor skipped all active names (enum bug)</t>
+          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>alpaca-py AssetStatus enum stringified to 'AssetStatus.ACTIVE'; check 'assetstatus.active' != 'active' wrongly skipped EVERY tradable stock since ~2026-05-28 → stock auto-trade silently dead, options-only</t>
+          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>executor.py: read enum .value ('active') before lowercasing</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr"/>
-      <c r="I88" s="5" t="inlineStr"/>
-      <c r="J88" s="5" t="inlineStr"/>
+          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Win: codified discipline survives session/agent boundaries.</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
+        </is>
+      </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4890,23 +4878,27 @@
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr">
         <is>
-          <t>c7098178a</t>
-        </is>
-      </c>
-      <c r="N88" s="8" t="inlineStr"/>
-    </row>
-    <row r="89" ht="105" customHeight="1">
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N88" s="8" t="inlineStr">
+        <is>
+          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="60" customHeight="1">
       <c r="A89" s="2" t="n">
         <v>88</v>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>EXEC-TRADABLE-ENUM</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4916,39 +4908,27 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>ML / Data Logging</t>
+          <t>Execution · Auto-Trade</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>Entry-time feature logger in swing_trade.py</t>
+          <t>Stock executor skipped all active names (enum bug)</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
+          <t>alpaca-py AssetStatus enum stringified to 'AssetStatus.ACTIVE'; check 'assetstatus.active' != 'active' wrongly skipped EVERY tradable stock since ~2026-05-28 → stock auto-trade silently dead, options-only</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
-        </is>
-      </c>
-      <c r="H89" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I89" s="5" t="inlineStr">
-        <is>
-          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
-        </is>
-      </c>
-      <c r="J89" s="5" t="inlineStr">
-        <is>
-          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
-        </is>
-      </c>
+          <t>executor.py: read enum .value ('active') before lowercasing</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="5" t="inlineStr"/>
+      <c r="J89" s="5" t="inlineStr"/>
       <c r="K89" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4956,19 +4936,15 @@
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="M89" s="3" t="inlineStr">
         <is>
-          <t>0574c60d4</t>
-        </is>
-      </c>
-      <c r="N89" s="8" t="inlineStr">
-        <is>
-          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
-        </is>
-      </c>
+          <t>c7098178a</t>
+        </is>
+      </c>
+      <c r="N89" s="8" t="inlineStr"/>
     </row>
     <row r="90" ht="105" customHeight="1">
       <c r="A90" s="2" t="n">
@@ -4976,7 +4952,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>ML-FEATURE-MISMATCH</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4986,27 +4962,39 @@
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>ML · Inference</t>
+          <t>ML / Data Logging</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>Live predict_one degenerate — 29-feat model vs 17-feat extractor</t>
+          <t>Entry-time feature logger in swing_trade.py</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Models retrained 2026-06-09 on 29 features but ml.feature_extractor.FEATURE_COLS still emits 17, so live predict_one feeds a mismatched vector and returns ~0 p_up for EVERY ticker (AI Edge 0% bug, all names). Batch ml-predict path extracts 29 correctly. /api/ml now prefers the batch cache + rejects degenerate live; ROOT FIX still needed: align FEATURE_COLS to 29 (or guard retrain to the live feature set). Also cache 4d stale.</t>
+          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>server /api/ml cache-first + degenerate guard (done); align ml/feature_extractor.FEATURE_COLS to model n_features_in_ (pending)</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr"/>
-      <c r="I90" s="5" t="inlineStr"/>
-      <c r="J90" s="5" t="inlineStr"/>
+          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
+        </is>
+      </c>
       <c r="K90" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -5014,15 +5002,19 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M90" s="3" t="inlineStr">
         <is>
-          <t>33877186c</t>
-        </is>
-      </c>
-      <c r="N90" s="8" t="inlineStr"/>
+          <t>0574c60d4</t>
+        </is>
+      </c>
+      <c r="N90" s="8" t="inlineStr">
+        <is>
+          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="45" customHeight="1">
       <c r="A91" s="2" t="n">
@@ -15723,7 +15715,7 @@
         </is>
       </c>
       <c r="B2" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="18" t="n">
         <v>20</v>
@@ -15732,7 +15724,7 @@
         <v>58</v>
       </c>
       <c r="E2" s="18" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
@@ -15761,7 +15753,7 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>77</v>
@@ -15770,7 +15762,7 @@
         <v>68</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5">

</xml_diff>